<commit_message>
WasteAndCircularity: Work on anaerobic digestion method
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -2,7 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
@@ -20,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="103">
   <si>
     <t>parameter</t>
   </si>
@@ -148,9 +153,6 @@
     <t>Assumed same as retail</t>
   </si>
   <si>
-    <t>Vall</t>
-  </si>
-  <si>
     <t>Avfall Sverige. (2009). Substrathandbok för biogasproduktion. RAPPORT U2009:14. BILAGA 1 – SUBSTRATLISTA</t>
   </si>
   <si>
@@ -208,9 +210,6 @@
     <t>HBK Biogasredovisning, ver 4.2. https://www.energigas.se/publikationer/hallbarhetskriterier-for-biodrivmedel-och-biobranslen/excel-verktyg-for-hbk-redovisning-och-berakning-av-vaxthusgasutslapp-for-biogas-och-biogasol/</t>
   </si>
   <si>
-    <t>non-waste, crop</t>
-  </si>
-  <si>
     <t>crop feedstock</t>
   </si>
   <si>
@@ -223,21 +222,127 @@
     <t>Share of B0 yielded as biogas</t>
   </si>
   <si>
-    <t>Nilsson et al??</t>
-  </si>
-  <si>
     <t>see FeedMgmt</t>
   </si>
   <si>
     <t>Note: This report states that N, P and K contents are given as "kg/ton DM" but should be "kg/ton wet weight" according to pers. comm. with Lindfors</t>
+  </si>
+  <si>
+    <t>digestate_B0</t>
+  </si>
+  <si>
+    <t>digestate_TAN_share</t>
+  </si>
+  <si>
+    <t>% of total N</t>
+  </si>
+  <si>
+    <t>Nilsson, J., Ernfors, M., Prade, T., &amp; Hansson, P. A. (2024). Cover crop cultivation strategies in a Scandinavian context for climate change mitigation and biogas production–Insights from a life cycle perspective. Science of The Total Environment, 170629.</t>
+  </si>
+  <si>
+    <t>Nilsson et al (2024)</t>
+  </si>
+  <si>
+    <t>vol. %</t>
+  </si>
+  <si>
+    <t>GENERAL</t>
+  </si>
+  <si>
+    <t>CH4_density</t>
+  </si>
+  <si>
+    <t>kg/Nm3</t>
+  </si>
+  <si>
+    <t>CO2_density</t>
+  </si>
+  <si>
+    <t>CH4_energy</t>
+  </si>
+  <si>
+    <t>MJ/kg</t>
+  </si>
+  <si>
+    <t>digestate_MCF</t>
+  </si>
+  <si>
+    <t>% of B0</t>
+  </si>
+  <si>
+    <t>Same for "Nötflytgödsel" and "Svinflytgödsel"</t>
+  </si>
+  <si>
+    <t>"Vall"</t>
+  </si>
+  <si>
+    <t>f_element</t>
+  </si>
+  <si>
+    <t>f_compound</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>digestate_loss_storage</t>
+  </si>
+  <si>
+    <t>NH3-N</t>
+  </si>
+  <si>
+    <t>NOx-N</t>
+  </si>
+  <si>
+    <t>N2O-N</t>
+  </si>
+  <si>
+    <t>N2</t>
+  </si>
+  <si>
+    <t>% of TAN</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>% of P</t>
+  </si>
+  <si>
+    <t>% of K</t>
+  </si>
+  <si>
+    <t>biogas_upgrading_electricity_use</t>
+  </si>
+  <si>
+    <t>kWh/Nm3 raw biogas</t>
+  </si>
+  <si>
+    <t>biogas_upgrading_CH4_slip</t>
+  </si>
+  <si>
+    <t>biogas_upgrading_share</t>
+  </si>
+  <si>
+    <t>Share of biogas upgraded</t>
+  </si>
+  <si>
+    <t>Biogas stat. Tabell 6</t>
+  </si>
+  <si>
+    <t>% of CH4 to upgrading</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
   </numFmts>
   <fonts count="7" x14ac:knownFonts="1">
     <font>
@@ -318,7 +423,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -331,6 +436,8 @@
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,7 +718,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K75"/>
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:M98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -619,13 +727,14 @@
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.7109375" customWidth="1"/>
-    <col min="8" max="8" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="32.42578125" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" customWidth="1"/>
+    <col min="6" max="7" width="21.28515625" customWidth="1"/>
+    <col min="8" max="8" width="25.7109375" customWidth="1"/>
+    <col min="10" max="10" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="32.42578125" customWidth="1"/>
+    <col min="12" max="12" width="20.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -636,28 +745,34 @@
         <v>5</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -670,281 +785,283 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F5" s="3" t="s">
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="3">
+      <c r="I5" s="3">
         <v>0</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>8</v>
       </c>
       <c r="E7" t="s">
         <v>14</v>
       </c>
-      <c r="F7" t="s">
+      <c r="H7" t="s">
         <v>7</v>
       </c>
-      <c r="G7">
+      <c r="I7">
         <v>40</v>
       </c>
-      <c r="H7" t="s">
+      <c r="J7" t="s">
         <v>12</v>
       </c>
-      <c r="I7" t="s">
+      <c r="K7" t="s">
         <v>20</v>
       </c>
-      <c r="J7" t="s">
+      <c r="L7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
         <v>8</v>
       </c>
       <c r="E8" t="s">
         <v>15</v>
       </c>
-      <c r="F8" t="s">
+      <c r="H8" t="s">
         <v>7</v>
       </c>
-      <c r="G8">
+      <c r="I8">
         <v>5</v>
       </c>
-      <c r="H8" t="s">
+      <c r="J8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
         <v>8</v>
       </c>
       <c r="E9" t="s">
         <v>16</v>
       </c>
-      <c r="F9" t="s">
+      <c r="H9" t="s">
         <v>7</v>
       </c>
-      <c r="G9">
+      <c r="I9">
         <v>50</v>
       </c>
-      <c r="H9" t="s">
+      <c r="J9" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
         <v>8</v>
       </c>
       <c r="E10" t="s">
         <v>17</v>
       </c>
-      <c r="F10" t="s">
+      <c r="H10" t="s">
         <v>7</v>
       </c>
-      <c r="G10">
+      <c r="I10">
         <v>5</v>
       </c>
-      <c r="H10" t="s">
+      <c r="J10" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
         <v>9</v>
       </c>
       <c r="E12" t="s">
         <v>14</v>
       </c>
-      <c r="F12" t="s">
+      <c r="H12" t="s">
         <v>7</v>
       </c>
-      <c r="G12">
+      <c r="I12">
         <v>40</v>
       </c>
-      <c r="H12" t="s">
+      <c r="J12" t="s">
         <v>12</v>
       </c>
-      <c r="I12" t="s">
+      <c r="K12" t="s">
         <v>20</v>
       </c>
-      <c r="J12" t="s">
+      <c r="L12" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
         <v>9</v>
       </c>
       <c r="E13" t="s">
         <v>15</v>
       </c>
-      <c r="F13" t="s">
+      <c r="H13" t="s">
         <v>7</v>
       </c>
-      <c r="G13">
+      <c r="I13">
         <v>5</v>
       </c>
-      <c r="H13" t="s">
+      <c r="J13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
         <v>9</v>
       </c>
       <c r="E14" t="s">
         <v>16</v>
       </c>
-      <c r="F14" t="s">
+      <c r="H14" t="s">
         <v>7</v>
       </c>
-      <c r="G14">
+      <c r="I14">
         <v>50</v>
       </c>
-      <c r="H14" t="s">
+      <c r="J14" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
         <v>9</v>
       </c>
       <c r="E15" t="s">
         <v>17</v>
       </c>
-      <c r="F15" t="s">
+      <c r="H15" t="s">
         <v>7</v>
       </c>
-      <c r="G15">
+      <c r="I15">
         <v>5</v>
       </c>
-      <c r="H15" t="s">
+      <c r="J15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
         <v>10</v>
       </c>
       <c r="E17" t="s">
         <v>14</v>
       </c>
-      <c r="F17" t="s">
+      <c r="H17" t="s">
         <v>7</v>
       </c>
-      <c r="G17">
+      <c r="I17">
         <v>40</v>
       </c>
-      <c r="H17" t="s">
+      <c r="J17" t="s">
         <v>12</v>
       </c>
-      <c r="I17" t="s">
+      <c r="K17" t="s">
         <v>20</v>
       </c>
-      <c r="J17" t="s">
+      <c r="L17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
         <v>10</v>
       </c>
       <c r="E18" t="s">
         <v>15</v>
       </c>
-      <c r="F18" t="s">
+      <c r="H18" t="s">
         <v>7</v>
       </c>
-      <c r="G18">
+      <c r="I18">
         <v>5</v>
       </c>
-      <c r="H18" t="s">
+      <c r="J18" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
         <v>10</v>
       </c>
       <c r="E19" t="s">
         <v>16</v>
       </c>
-      <c r="F19" t="s">
+      <c r="H19" t="s">
         <v>7</v>
       </c>
-      <c r="G19">
+      <c r="I19">
         <v>50</v>
       </c>
-      <c r="H19" t="s">
+      <c r="J19" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>10</v>
       </c>
       <c r="E20" t="s">
         <v>17</v>
       </c>
-      <c r="F20" t="s">
+      <c r="H20" t="s">
         <v>7</v>
       </c>
-      <c r="G20">
+      <c r="I20">
         <v>5</v>
       </c>
-      <c r="H20" t="s">
+      <c r="J20" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
         <v>11</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E22" t="s">
         <v>14</v>
       </c>
-      <c r="F22" t="s">
+      <c r="H22" t="s">
         <v>7</v>
       </c>
-      <c r="G22">
+      <c r="I22">
         <v>100</v>
       </c>
-      <c r="H22" t="s">
+      <c r="J22" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E24" t="s">
         <v>14</v>
       </c>
-      <c r="F24" t="s">
+      <c r="H24" t="s">
         <v>7</v>
       </c>
-      <c r="G24">
+      <c r="I24">
         <v>100</v>
       </c>
-      <c r="H24" t="s">
+      <c r="J24" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>22</v>
       </c>
@@ -957,29 +1074,31 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K26" s="5"/>
+      <c r="L26" s="5"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E28" t="s">
         <v>14</v>
       </c>
-      <c r="F28" t="s">
+      <c r="H28" t="s">
         <v>7</v>
       </c>
-      <c r="G28">
+      <c r="I28">
         <v>100</v>
       </c>
-      <c r="H28" t="s">
+      <c r="J28" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
@@ -992,492 +1111,499 @@
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
       <c r="J30" s="2"/>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F32" s="3" t="s">
+      <c r="K30" s="2"/>
+      <c r="L30" s="2"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H32" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="G32" s="3">
+      <c r="I32" s="3">
         <v>0.5</v>
       </c>
-      <c r="H32" s="3" t="s">
+      <c r="J32" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="I32" s="3" t="s">
+      <c r="K32" s="3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="4"/>
       <c r="B34" s="4"/>
       <c r="C34" t="s">
         <v>8</v>
       </c>
-      <c r="F34" t="s">
+      <c r="H34" t="s">
         <v>31</v>
       </c>
-      <c r="G34">
+      <c r="I34">
         <v>0.33</v>
       </c>
-      <c r="H34" t="s">
+      <c r="J34" t="s">
         <v>32</v>
       </c>
-      <c r="I34" t="s">
+      <c r="K34" t="s">
         <v>40</v>
       </c>
-      <c r="J34" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L34" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" t="s">
         <v>8</v>
       </c>
-      <c r="F35" t="s">
+      <c r="H35" t="s">
         <v>24</v>
       </c>
-      <c r="G35">
+      <c r="I35">
         <v>0.85</v>
       </c>
-      <c r="H35" t="s">
+      <c r="J35" t="s">
         <v>33</v>
       </c>
-      <c r="J35" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L35" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C36" t="s">
         <v>8</v>
       </c>
-      <c r="F36" t="s">
-        <v>50</v>
-      </c>
-      <c r="G36">
+      <c r="H36" t="s">
+        <v>49</v>
+      </c>
+      <c r="I36">
         <v>0.46100000000000002</v>
       </c>
-      <c r="H36" t="s">
-        <v>44</v>
-      </c>
       <c r="J36" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="L36" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" t="s">
         <v>8</v>
       </c>
-      <c r="F37" t="s">
+      <c r="H37" t="s">
         <v>25</v>
       </c>
-      <c r="G37" s="8">
+      <c r="I37" s="8">
         <f>8.3/1000/0.33</f>
         <v>2.515151515151515E-2</v>
       </c>
-      <c r="H37" t="s">
+      <c r="J37" t="s">
         <v>34</v>
       </c>
-      <c r="J37" t="s">
-        <v>64</v>
-      </c>
-      <c r="K37" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L37" t="s">
+        <v>62</v>
+      </c>
+      <c r="M37" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" t="s">
         <v>8</v>
       </c>
-      <c r="F38" t="s">
+      <c r="H38" t="s">
         <v>26</v>
       </c>
-      <c r="G38" s="8">
+      <c r="I38" s="8">
         <f>1/1000/0.33</f>
         <v>3.0303030303030303E-3</v>
       </c>
-      <c r="H38" t="s">
+      <c r="J38" t="s">
         <v>35</v>
       </c>
-      <c r="J38" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L38" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" t="s">
         <v>8</v>
       </c>
-      <c r="F39" t="s">
+      <c r="H39" t="s">
         <v>27</v>
       </c>
-      <c r="G39" s="8">
+      <c r="I39" s="8">
         <f>2.6/1000/0.33</f>
         <v>7.8787878787878775E-3</v>
       </c>
-      <c r="H39" t="s">
+      <c r="J39" t="s">
         <v>36</v>
       </c>
-      <c r="J39" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L39" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" t="s">
         <v>9</v>
       </c>
-      <c r="F41" t="s">
+      <c r="H41" t="s">
         <v>31</v>
       </c>
-      <c r="G41">
+      <c r="I41">
         <v>0.15</v>
       </c>
-      <c r="H41" t="s">
+      <c r="J41" t="s">
         <v>32</v>
       </c>
-      <c r="J41" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L41" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" t="s">
         <v>9</v>
       </c>
-      <c r="F42" t="s">
+      <c r="H42" t="s">
         <v>24</v>
       </c>
-      <c r="G42" s="10">
+      <c r="I42" s="10">
         <v>0.9</v>
       </c>
-      <c r="H42" t="s">
+      <c r="J42" t="s">
         <v>33</v>
       </c>
-      <c r="I42" s="7"/>
-      <c r="J42" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K42" s="7"/>
+      <c r="L42" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C43" t="s">
         <v>9</v>
       </c>
-      <c r="F43" t="s">
-        <v>50</v>
-      </c>
-      <c r="G43" s="8">
+      <c r="H43" t="s">
+        <v>49</v>
+      </c>
+      <c r="I43" s="8">
         <v>0.55000000000000004</v>
       </c>
-      <c r="H43" t="s">
-        <v>44</v>
-      </c>
       <c r="J43" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="L43" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" t="s">
         <v>9</v>
       </c>
-      <c r="F44" t="s">
+      <c r="H44" t="s">
         <v>25</v>
       </c>
-      <c r="G44" s="8">
+      <c r="I44" s="8">
         <f>3.8/1000/0.15</f>
         <v>2.5333333333333333E-2</v>
       </c>
-      <c r="H44" t="s">
+      <c r="J44" t="s">
         <v>34</v>
       </c>
-      <c r="J44" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L44" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" t="s">
         <v>9</v>
       </c>
-      <c r="F45" t="s">
+      <c r="H45" t="s">
         <v>26</v>
       </c>
-      <c r="G45" s="8">
+      <c r="I45" s="8">
         <f>0.5/1000/0.15</f>
         <v>3.3333333333333335E-3</v>
       </c>
-      <c r="H45" t="s">
+      <c r="J45" t="s">
         <v>35</v>
       </c>
-      <c r="J45" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L45" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" t="s">
         <v>9</v>
       </c>
-      <c r="F46" t="s">
+      <c r="H46" t="s">
         <v>27</v>
       </c>
-      <c r="G46" s="8">
+      <c r="I46" s="8">
         <f>1.2/1000/0.15</f>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="H46" t="s">
+      <c r="J46" t="s">
         <v>36</v>
       </c>
-      <c r="J46" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="L46" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" t="s">
         <v>10</v>
       </c>
-      <c r="F48" t="s">
+      <c r="H48" t="s">
         <v>31</v>
       </c>
-      <c r="G48" s="6">
-        <f>G41</f>
+      <c r="I48" s="6">
+        <f t="shared" ref="I48:I53" si="0">I41</f>
         <v>0.15</v>
       </c>
-      <c r="H48" t="s">
+      <c r="J48" t="s">
         <v>32</v>
       </c>
-      <c r="I48" s="7" t="s">
+      <c r="K48" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" t="s">
         <v>10</v>
       </c>
-      <c r="F49" t="s">
+      <c r="H49" t="s">
         <v>24</v>
       </c>
-      <c r="G49" s="6">
-        <f>G42</f>
+      <c r="I49" s="6">
+        <f t="shared" si="0"/>
         <v>0.9</v>
       </c>
-      <c r="H49" t="s">
+      <c r="J49" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" t="s">
         <v>10</v>
       </c>
-      <c r="F50" t="s">
-        <v>50</v>
-      </c>
-      <c r="G50" s="9">
-        <f>G43</f>
+      <c r="H50" t="s">
+        <v>49</v>
+      </c>
+      <c r="I50" s="9">
+        <f t="shared" si="0"/>
         <v>0.55000000000000004</v>
       </c>
-      <c r="H50" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="J50" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
       <c r="C51" t="s">
         <v>10</v>
       </c>
-      <c r="F51" t="s">
+      <c r="H51" t="s">
         <v>25</v>
       </c>
-      <c r="G51" s="9">
-        <f>G44</f>
+      <c r="I51" s="9">
+        <f t="shared" si="0"/>
         <v>2.5333333333333333E-2</v>
       </c>
-      <c r="H51" t="s">
+      <c r="J51" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" t="s">
         <v>10</v>
       </c>
-      <c r="F52" t="s">
+      <c r="H52" t="s">
         <v>26</v>
       </c>
-      <c r="G52" s="9">
-        <f>G45</f>
+      <c r="I52" s="9">
+        <f t="shared" si="0"/>
         <v>3.3333333333333335E-3</v>
       </c>
-      <c r="H52" t="s">
+      <c r="J52" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" t="s">
         <v>10</v>
       </c>
-      <c r="F53" t="s">
+      <c r="H53" t="s">
         <v>27</v>
       </c>
-      <c r="G53" s="9">
-        <f>G46</f>
+      <c r="I53" s="9">
+        <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="H53" t="s">
+      <c r="J53" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B55" s="4"/>
       <c r="C55" t="s">
-        <v>63</v>
-      </c>
-      <c r="F55" t="s">
+        <v>61</v>
+      </c>
+      <c r="H55" t="s">
         <v>31</v>
       </c>
-      <c r="G55">
+      <c r="I55">
         <v>1</v>
       </c>
-      <c r="H55" t="s">
+      <c r="J55" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" t="s">
-        <v>63</v>
-      </c>
-      <c r="F56" t="s">
+        <v>61</v>
+      </c>
+      <c r="H56" t="s">
         <v>24</v>
       </c>
-      <c r="G56">
+      <c r="I56">
         <v>0.88</v>
       </c>
-      <c r="H56" t="s">
+      <c r="J56" t="s">
         <v>33</v>
       </c>
-      <c r="J56" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L56" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" t="s">
-        <v>63</v>
-      </c>
-      <c r="F57" t="s">
-        <v>50</v>
-      </c>
-      <c r="G57" s="8">
+        <v>61</v>
+      </c>
+      <c r="H57" t="s">
+        <v>49</v>
+      </c>
+      <c r="I57" s="8">
         <v>0.3</v>
       </c>
-      <c r="H57" t="s">
-        <v>44</v>
-      </c>
       <c r="J57" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+      <c r="L57" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" t="s">
-        <v>63</v>
-      </c>
-      <c r="F58" t="s">
+        <v>61</v>
+      </c>
+      <c r="H58" t="s">
         <v>25</v>
       </c>
-      <c r="G58" s="4">
+      <c r="I58" s="4">
         <f>2.1/100</f>
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="H58" t="s">
+      <c r="J58" t="s">
         <v>34</v>
       </c>
-      <c r="J58" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L58" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A59" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B59" s="4"/>
       <c r="C59" t="s">
-        <v>63</v>
-      </c>
-      <c r="F59" t="s">
+        <v>61</v>
+      </c>
+      <c r="H59" t="s">
         <v>26</v>
       </c>
-      <c r="G59" s="11">
+      <c r="I59" s="11">
         <f>0.27/100</f>
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="H59" t="s">
+      <c r="J59" t="s">
         <v>35</v>
       </c>
-      <c r="J59" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L59" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B60" s="4"/>
       <c r="C60" t="s">
-        <v>63</v>
-      </c>
-      <c r="F60" t="s">
+        <v>61</v>
+      </c>
+      <c r="H60" t="s">
         <v>27</v>
       </c>
-      <c r="G60" s="11">
+      <c r="I60" s="11">
         <f>2.34/100</f>
         <v>2.3399999999999997E-2</v>
       </c>
-      <c r="H60" t="s">
+      <c r="J60" t="s">
         <v>36</v>
       </c>
-      <c r="J60" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="L60" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A61" s="4"/>
+      <c r="B61" s="4"/>
+      <c r="I61" s="11"/>
+    </row>
+    <row r="62" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -1488,177 +1614,486 @@
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F64" t="s">
-        <v>45</v>
-      </c>
-      <c r="G64" s="4">
+      <c r="K62" s="2"/>
+      <c r="L62" s="2"/>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A63" s="4"/>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4"/>
+      <c r="D63" s="4"/>
+      <c r="E63" s="4"/>
+      <c r="F63" s="4"/>
+      <c r="G63" s="4"/>
+      <c r="H63" s="4"/>
+      <c r="I63" s="4"/>
+      <c r="J63" s="4"/>
+      <c r="K63" s="4"/>
+      <c r="L63" s="4"/>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A64" s="4"/>
+      <c r="B64" s="4"/>
+      <c r="H64" t="s">
+        <v>74</v>
+      </c>
+      <c r="I64" s="11">
+        <v>0.71750000000000003</v>
+      </c>
+      <c r="J64" t="s">
+        <v>75</v>
+      </c>
+      <c r="L64" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A65" s="4"/>
+      <c r="B65" s="4"/>
+      <c r="H65" t="s">
+        <v>76</v>
+      </c>
+      <c r="I65" s="11">
+        <v>1.9496</v>
+      </c>
+      <c r="J65" t="s">
+        <v>75</v>
+      </c>
+      <c r="L65" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A66" s="4"/>
+      <c r="B66" s="4"/>
+      <c r="H66" t="s">
+        <v>77</v>
+      </c>
+      <c r="I66" s="13">
+        <v>50</v>
+      </c>
+      <c r="J66" t="s">
+        <v>78</v>
+      </c>
+      <c r="L66" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B68" s="2"/>
+      <c r="C68" s="2"/>
+      <c r="D68" s="2"/>
+      <c r="E68" s="2"/>
+      <c r="F68" s="2"/>
+      <c r="G68" s="2"/>
+      <c r="H68" s="2"/>
+      <c r="I68" s="2"/>
+      <c r="J68" s="2"/>
+      <c r="K68" s="2"/>
+      <c r="L68" s="2"/>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H70" t="s">
+        <v>44</v>
+      </c>
+      <c r="I70" s="4">
         <v>90</v>
       </c>
-      <c r="H64" s="4" t="s">
+      <c r="J70" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="I64" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="J64" t="s">
+      <c r="K70" s="4" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F65" t="s">
+      <c r="L70" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H71" t="s">
+        <v>52</v>
+      </c>
+      <c r="I71" s="4">
+        <v>0.22</v>
+      </c>
+      <c r="J71" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G65" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="H65" s="4" t="s">
+      <c r="K71" s="7"/>
+      <c r="L71" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H72" t="s">
+        <v>50</v>
+      </c>
+      <c r="I72" s="4">
+        <v>3.4</v>
+      </c>
+      <c r="J72" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="K72" s="7"/>
+      <c r="L72" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H73" t="s">
+        <v>51</v>
+      </c>
+      <c r="I73" s="4">
+        <v>5</v>
+      </c>
+      <c r="J73" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="I65" s="7"/>
-      <c r="J65" t="s">
+      <c r="K73" s="7"/>
+      <c r="L73" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I74" s="4"/>
+      <c r="J74" s="4"/>
+      <c r="K74" s="7"/>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H75" t="s">
+        <v>55</v>
+      </c>
+      <c r="I75" s="4">
+        <v>0.61</v>
+      </c>
+      <c r="J75" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="K75" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="L75" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="76" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H76" t="s">
+        <v>56</v>
+      </c>
+      <c r="I76" s="4">
+        <v>0.99</v>
+      </c>
+      <c r="J76" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="K76" s="7"/>
+      <c r="L76" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I77" s="4"/>
+      <c r="J77" s="4"/>
+      <c r="K77" s="7"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H78" t="s">
+        <v>99</v>
+      </c>
+      <c r="I78" s="4">
+        <v>94</v>
+      </c>
+      <c r="J78" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="K78" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="L78" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H79" t="s">
+        <v>98</v>
+      </c>
+      <c r="I79" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="J79" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="K79" s="7"/>
+      <c r="L79" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H80" t="s">
+        <v>96</v>
+      </c>
+      <c r="I80" s="4">
+        <f>0.9*(1/3.6)</f>
+        <v>0.25</v>
+      </c>
+      <c r="J80" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="K80" s="7"/>
+      <c r="L80" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C82" t="s">
+        <v>8</v>
+      </c>
+      <c r="H82" t="s">
+        <v>39</v>
+      </c>
+      <c r="I82">
+        <v>63</v>
+      </c>
+      <c r="J82" t="s">
+        <v>72</v>
+      </c>
+      <c r="L82" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="83" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
+        <v>9</v>
+      </c>
+      <c r="H83" t="s">
+        <v>39</v>
+      </c>
+      <c r="I83">
+        <v>59</v>
+      </c>
+      <c r="J83" t="s">
+        <v>72</v>
+      </c>
+      <c r="L83" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="84" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C84" t="s">
+        <v>10</v>
+      </c>
+      <c r="H84" t="s">
+        <v>39</v>
+      </c>
+      <c r="I84" s="6">
+        <f>I83</f>
+        <v>59</v>
+      </c>
+      <c r="J84" t="s">
+        <v>72</v>
+      </c>
+      <c r="K84" s="7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="85" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A85" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B85" s="4"/>
+      <c r="C85" t="s">
+        <v>61</v>
+      </c>
+      <c r="H85" t="s">
+        <v>39</v>
+      </c>
+      <c r="I85">
+        <v>56</v>
+      </c>
+      <c r="J85" t="s">
+        <v>72</v>
+      </c>
+      <c r="K85" t="s">
+        <v>82</v>
+      </c>
+      <c r="L85" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="86" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C86" t="s">
+        <v>46</v>
+      </c>
+      <c r="H86" t="s">
+        <v>39</v>
+      </c>
+      <c r="I86" s="4">
+        <v>65</v>
+      </c>
+      <c r="J86" t="s">
+        <v>72</v>
+      </c>
+      <c r="K86" t="s">
+        <v>81</v>
+      </c>
+      <c r="L86" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="87" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="I87" s="4"/>
+      <c r="J87" s="4"/>
+      <c r="K87" s="7"/>
+    </row>
+    <row r="88" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H88" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F66" t="s">
-        <v>51</v>
-      </c>
-      <c r="G66" s="4">
-        <v>5</v>
-      </c>
-      <c r="H66" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="I66" s="7"/>
-      <c r="J66" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F67" t="s">
-        <v>52</v>
-      </c>
-      <c r="G67" s="4">
-        <v>5</v>
-      </c>
-      <c r="H67" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="I67" s="7"/>
-      <c r="J67" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="G68" s="4"/>
-      <c r="H68" s="4"/>
-      <c r="I68" s="7"/>
-    </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F69" t="s">
-        <v>56</v>
-      </c>
-      <c r="G69" s="4">
-        <v>0.61</v>
-      </c>
-      <c r="H69" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I69" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="J69" t="s">
+      <c r="I88" s="11">
+        <f>238/0.74/1000</f>
+        <v>0.32162162162162161</v>
+      </c>
+      <c r="J88" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="K88" s="7"/>
+      <c r="L88" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="89" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H89" t="s">
+        <v>79</v>
+      </c>
+      <c r="I89" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="J89" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="K89" s="7"/>
+      <c r="L89" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="90" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="H90" t="s">
+        <v>68</v>
+      </c>
+      <c r="I90" s="13">
         <v>60</v>
       </c>
-    </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="F70" t="s">
-        <v>57</v>
-      </c>
-      <c r="G70" s="4">
-        <v>0.99</v>
-      </c>
-      <c r="H70" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="I70" s="7"/>
-    </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C72" t="s">
-        <v>8</v>
-      </c>
-      <c r="F72" t="s">
-        <v>39</v>
-      </c>
-      <c r="G72">
-        <v>63</v>
-      </c>
-      <c r="H72" t="s">
-        <v>12</v>
-      </c>
-      <c r="J72" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C73" t="s">
-        <v>9</v>
-      </c>
-      <c r="F73" t="s">
-        <v>39</v>
-      </c>
-      <c r="G73">
-        <v>59</v>
-      </c>
-      <c r="H73" t="s">
-        <v>12</v>
-      </c>
-      <c r="J73" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="C74" t="s">
-        <v>10</v>
-      </c>
-      <c r="F74" t="s">
-        <v>39</v>
-      </c>
-      <c r="G74" s="6">
-        <f>G73</f>
-        <v>59</v>
-      </c>
-      <c r="H74" t="s">
-        <v>12</v>
-      </c>
-      <c r="I74" s="7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A75" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B75" s="4"/>
-      <c r="C75" t="s">
-        <v>62</v>
-      </c>
-      <c r="F75" t="s">
-        <v>39</v>
-      </c>
-      <c r="G75">
-        <v>56</v>
-      </c>
-      <c r="H75" t="s">
-        <v>12</v>
-      </c>
-      <c r="I75" t="s">
-        <v>42</v>
-      </c>
-      <c r="J75" t="s">
-        <v>49</v>
+      <c r="J90" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="K90" s="7"/>
+      <c r="L90" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="92" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F92" t="s">
+        <v>85</v>
+      </c>
+      <c r="G92" t="s">
+        <v>87</v>
+      </c>
+      <c r="H92" t="s">
+        <v>86</v>
+      </c>
+      <c r="I92">
+        <v>2.75</v>
+      </c>
+      <c r="J92" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="93" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F93" t="s">
+        <v>85</v>
+      </c>
+      <c r="G93" t="s">
+        <v>88</v>
+      </c>
+      <c r="H93" t="s">
+        <v>86</v>
+      </c>
+      <c r="I93">
+        <v>0</v>
+      </c>
+      <c r="J93" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="94" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F94" t="s">
+        <v>85</v>
+      </c>
+      <c r="G94" t="s">
+        <v>89</v>
+      </c>
+      <c r="H94" t="s">
+        <v>86</v>
+      </c>
+      <c r="I94">
+        <v>0</v>
+      </c>
+      <c r="J94" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="95" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F95" t="s">
+        <v>85</v>
+      </c>
+      <c r="G95" t="s">
+        <v>90</v>
+      </c>
+      <c r="H95" t="s">
+        <v>86</v>
+      </c>
+      <c r="I95">
+        <v>0</v>
+      </c>
+      <c r="J95" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="97" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F97" t="s">
+        <v>92</v>
+      </c>
+      <c r="G97" t="s">
+        <v>92</v>
+      </c>
+      <c r="H97" t="s">
+        <v>86</v>
+      </c>
+      <c r="I97">
+        <v>0</v>
+      </c>
+      <c r="J97" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="98" spans="6:10" x14ac:dyDescent="0.25">
+      <c r="F98" t="s">
+        <v>93</v>
+      </c>
+      <c r="G98" t="s">
+        <v>93</v>
+      </c>
+      <c r="H98" t="s">
+        <v>86</v>
+      </c>
+      <c r="I98">
+        <v>0</v>
+      </c>
+      <c r="J98" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -1669,25 +2104,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A2:A4"/>
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A2:A5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>65</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
WasteAndCircularity: Some name changes waste -> feedstock
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="117">
   <si>
     <t>parameter</t>
   </si>
@@ -42,27 +42,9 @@
     <t>source</t>
   </si>
   <si>
-    <t>f_waste_level</t>
-  </si>
-  <si>
-    <t>f_waste_treatment</t>
-  </si>
-  <si>
     <t>treatment_share</t>
   </si>
   <si>
-    <t>household</t>
-  </si>
-  <si>
-    <t>retail</t>
-  </si>
-  <si>
-    <t>processing</t>
-  </si>
-  <si>
-    <t>carcasses</t>
-  </si>
-  <si>
     <t>%</t>
   </si>
   <si>
@@ -99,30 +81,9 @@
     <t>WASTE COMPOSITION</t>
   </si>
   <si>
-    <t>waste_VS</t>
-  </si>
-  <si>
-    <t>waste_N</t>
-  </si>
-  <si>
-    <t>waste_P</t>
-  </si>
-  <si>
-    <t>waste_K</t>
-  </si>
-  <si>
     <t>kg C/kg VS</t>
   </si>
   <si>
-    <t>f_waste</t>
-  </si>
-  <si>
-    <t>f_waste_group</t>
-  </si>
-  <si>
-    <t>waste_DM</t>
-  </si>
-  <si>
     <t>kg DM/kg</t>
   </si>
   <si>
@@ -138,9 +99,6 @@
     <t>kg K/kg DM</t>
   </si>
   <si>
-    <t>waste_C</t>
-  </si>
-  <si>
     <t>ANAEROBIC DIGESTION</t>
   </si>
   <si>
@@ -162,9 +120,6 @@
     <t>biogas_CH4_yield</t>
   </si>
   <si>
-    <t>primary</t>
-  </si>
-  <si>
     <t>manure</t>
   </si>
   <si>
@@ -174,9 +129,6 @@
     <t>Avfall Sverige (2009)</t>
   </si>
   <si>
-    <t>waste_B0</t>
-  </si>
-  <si>
     <t>biogas_flare_frac</t>
   </si>
   <si>
@@ -376,6 +328,54 @@
   </si>
   <si>
     <t>% of CH4</t>
+  </si>
+  <si>
+    <t>f_feedstock_type</t>
+  </si>
+  <si>
+    <t>animal carcasses</t>
+  </si>
+  <si>
+    <t>slaughterhouse waste</t>
+  </si>
+  <si>
+    <t>f_feedstock</t>
+  </si>
+  <si>
+    <t>f_feedstock_group</t>
+  </si>
+  <si>
+    <t>f_treatment</t>
+  </si>
+  <si>
+    <t>feedstock_C</t>
+  </si>
+  <si>
+    <t>feedstock_DM</t>
+  </si>
+  <si>
+    <t>feedstock_VS</t>
+  </si>
+  <si>
+    <t>feedstock_B0</t>
+  </si>
+  <si>
+    <t>feedstock_N</t>
+  </si>
+  <si>
+    <t>feedstock_P</t>
+  </si>
+  <si>
+    <t>feedstock_K</t>
+  </si>
+  <si>
+    <t>food waste, household</t>
+  </si>
+  <si>
+    <t>food waste, retail</t>
+  </si>
+  <si>
+    <t>food waste, processing</t>
   </si>
 </sst>
 </file>
@@ -772,11 +772,11 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O103"/>
+  <dimension ref="A1:O104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
     <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
@@ -789,31 +789,31 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
+        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>5</v>
+        <v>101</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>80</v>
+        <v>64</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>93</v>
+        <v>77</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>0</v>
@@ -833,7 +833,7 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -851,1230 +851,1231 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J5" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K5" s="3">
         <v>0</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" t="s">
         <v>8</v>
       </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
       <c r="J7" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K7">
         <v>40</v>
       </c>
       <c r="L7" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M7" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="N7" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="E8" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="J8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K8">
         <v>5</v>
       </c>
       <c r="L8" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J9" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K9">
         <v>50</v>
       </c>
       <c r="L9" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="E10" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K10">
         <v>5</v>
       </c>
       <c r="L10" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="E12" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K12">
         <v>40</v>
       </c>
       <c r="L12" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M12" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="N12" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E13" t="s">
         <v>9</v>
       </c>
-      <c r="E13" t="s">
-        <v>15</v>
-      </c>
       <c r="J13" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K13">
         <v>5</v>
       </c>
       <c r="L13" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J14" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K14">
         <v>50</v>
       </c>
       <c r="L14" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="E15" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J15" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K15">
         <v>5</v>
       </c>
       <c r="L15" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="E17" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="J17" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K17">
         <v>40</v>
       </c>
       <c r="L17" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="M17" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="N17" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="E18" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="J18" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K18">
         <v>5</v>
       </c>
       <c r="L18" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
+        <v>116</v>
+      </c>
+      <c r="E19" t="s">
         <v>10</v>
       </c>
-      <c r="E19" t="s">
-        <v>16</v>
-      </c>
       <c r="J19" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K19">
         <v>50</v>
       </c>
       <c r="L19" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="E20" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="J20" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K20">
         <v>5</v>
       </c>
       <c r="L20" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" t="s">
-        <v>14</v>
-      </c>
-      <c r="J22" t="s">
+      <c r="C22" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
+      <c r="J22" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K22" s="7">
+        <v>100</v>
+      </c>
+      <c r="L22" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C23" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
+      <c r="J23" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="K23" s="7">
+        <v>100</v>
+      </c>
+      <c r="L23" s="7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>31</v>
+      </c>
+      <c r="E25" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" t="s">
+        <v>5</v>
+      </c>
+      <c r="K25">
+        <v>100</v>
+      </c>
+      <c r="L25" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" s="5"/>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="5"/>
+      <c r="N27" s="5"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" t="s">
+        <v>43</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="J29" t="s">
+        <v>5</v>
+      </c>
+      <c r="K29">
+        <v>100</v>
+      </c>
+      <c r="L29" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B31" s="2"/>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J33" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="K33" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L33" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M33" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="K22">
-        <v>100</v>
-      </c>
-      <c r="L22" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C24" t="s">
-        <v>46</v>
-      </c>
-      <c r="E24" t="s">
-        <v>14</v>
-      </c>
-      <c r="J24" t="s">
-        <v>7</v>
-      </c>
-      <c r="K24">
-        <v>100</v>
-      </c>
-      <c r="L24" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A26" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="5"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="5"/>
-      <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-      <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
-      <c r="K26" s="5"/>
-      <c r="L26" s="5"/>
-      <c r="M26" s="5"/>
-      <c r="N26" s="5"/>
-    </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B28" s="4"/>
-      <c r="C28" t="s">
-        <v>59</v>
-      </c>
-      <c r="E28" t="s">
-        <v>14</v>
-      </c>
-      <c r="J28" t="s">
-        <v>7</v>
-      </c>
-      <c r="K28">
-        <v>100</v>
-      </c>
-      <c r="L28" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A30" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" s="2"/>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J32" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K32" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="L32" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="M32" s="3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="4"/>
-      <c r="C34" t="s">
-        <v>8</v>
-      </c>
-      <c r="J34" t="s">
-        <v>31</v>
-      </c>
-      <c r="K34">
-        <v>0.33</v>
-      </c>
-      <c r="L34" t="s">
-        <v>32</v>
-      </c>
-      <c r="M34" t="s">
-        <v>40</v>
-      </c>
-      <c r="N34" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
       <c r="B35" s="4"/>
       <c r="C35" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="J35" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="K35">
+        <v>0.33</v>
+      </c>
+      <c r="L35" t="s">
+        <v>19</v>
+      </c>
+      <c r="M35" t="s">
+        <v>26</v>
+      </c>
+      <c r="N35" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" t="s">
+        <v>114</v>
+      </c>
+      <c r="J36" t="s">
+        <v>109</v>
+      </c>
+      <c r="K36">
         <v>0.85</v>
       </c>
-      <c r="L35" t="s">
+      <c r="L36" t="s">
+        <v>20</v>
+      </c>
+      <c r="N36" t="s">
         <v>33</v>
       </c>
-      <c r="N35" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C36" t="s">
-        <v>8</v>
-      </c>
-      <c r="J36" t="s">
-        <v>49</v>
-      </c>
-      <c r="K36">
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C37" t="s">
+        <v>114</v>
+      </c>
+      <c r="J37" t="s">
+        <v>110</v>
+      </c>
+      <c r="K37">
         <v>0.46100000000000002</v>
       </c>
-      <c r="L36" t="s">
-        <v>43</v>
-      </c>
-      <c r="N36" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="4"/>
-      <c r="B37" s="4"/>
-      <c r="C37" t="s">
-        <v>8</v>
-      </c>
-      <c r="J37" t="s">
-        <v>25</v>
-      </c>
-      <c r="K37" s="8">
-        <f>8.3/1000/0.33</f>
-        <v>2.515151515151515E-2</v>
-      </c>
       <c r="L37" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="N37" t="s">
-        <v>60</v>
-      </c>
-      <c r="O37" t="s">
-        <v>64</v>
+        <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A38" s="4"/>
       <c r="B38" s="4"/>
       <c r="C38" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="J38" t="s">
-        <v>26</v>
+        <v>111</v>
       </c>
       <c r="K38" s="8">
-        <f>1/1000/0.33</f>
-        <v>3.0303030303030303E-3</v>
+        <f>8.3/1000/0.33</f>
+        <v>2.515151515151515E-2</v>
       </c>
       <c r="L38" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="N38" t="s">
-        <v>60</v>
+        <v>44</v>
+      </c>
+      <c r="O38" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A39" s="4"/>
       <c r="B39" s="4"/>
       <c r="C39" t="s">
-        <v>8</v>
+        <v>114</v>
       </c>
       <c r="J39" t="s">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="K39" s="8">
+        <f>1/1000/0.33</f>
+        <v>3.0303030303030303E-3</v>
+      </c>
+      <c r="L39" t="s">
+        <v>22</v>
+      </c>
+      <c r="N39" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A40" s="4"/>
+      <c r="B40" s="4"/>
+      <c r="C40" t="s">
+        <v>114</v>
+      </c>
+      <c r="J40" t="s">
+        <v>113</v>
+      </c>
+      <c r="K40" s="8">
         <f>2.6/1000/0.33</f>
         <v>7.8787878787878775E-3</v>
       </c>
-      <c r="L39" t="s">
-        <v>36</v>
-      </c>
-      <c r="N39" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="4"/>
-      <c r="B41" s="4"/>
-      <c r="C41" t="s">
-        <v>9</v>
-      </c>
-      <c r="J41" t="s">
-        <v>31</v>
-      </c>
-      <c r="K41">
-        <v>0.15</v>
-      </c>
-      <c r="L41" t="s">
-        <v>32</v>
-      </c>
-      <c r="N41" t="s">
-        <v>60</v>
+      <c r="L40" t="s">
+        <v>23</v>
+      </c>
+      <c r="N40" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="J42" t="s">
-        <v>24</v>
-      </c>
-      <c r="K42" s="10">
+        <v>108</v>
+      </c>
+      <c r="K42">
+        <v>0.15</v>
+      </c>
+      <c r="L42" t="s">
+        <v>19</v>
+      </c>
+      <c r="N42" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" t="s">
+        <v>115</v>
+      </c>
+      <c r="J43" t="s">
+        <v>109</v>
+      </c>
+      <c r="K43" s="10">
         <v>0.9</v>
       </c>
-      <c r="L42" t="s">
-        <v>33</v>
-      </c>
-      <c r="M42" s="7"/>
-      <c r="N42" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C43" t="s">
-        <v>9</v>
-      </c>
-      <c r="J43" t="s">
-        <v>49</v>
-      </c>
-      <c r="K43" s="8">
+      <c r="L43" t="s">
+        <v>20</v>
+      </c>
+      <c r="M43" s="7"/>
+      <c r="N43" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="C44" t="s">
+        <v>115</v>
+      </c>
+      <c r="J44" t="s">
+        <v>110</v>
+      </c>
+      <c r="K44" s="8">
         <v>0.55000000000000004</v>
       </c>
-      <c r="L43" t="s">
-        <v>43</v>
-      </c>
-      <c r="N43" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="4"/>
-      <c r="B44" s="4"/>
-      <c r="C44" t="s">
-        <v>9</v>
-      </c>
-      <c r="J44" t="s">
-        <v>25</v>
-      </c>
-      <c r="K44" s="8">
-        <f>3.8/1000/0.15</f>
-        <v>2.5333333333333333E-2</v>
-      </c>
       <c r="L44" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="N44" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A45" s="4"/>
       <c r="B45" s="4"/>
       <c r="C45" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="J45" t="s">
-        <v>26</v>
+        <v>111</v>
       </c>
       <c r="K45" s="8">
-        <f>0.5/1000/0.15</f>
-        <v>3.3333333333333335E-3</v>
+        <f>3.8/1000/0.15</f>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L45" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="N45" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="4"/>
       <c r="B46" s="4"/>
       <c r="C46" t="s">
-        <v>9</v>
+        <v>115</v>
       </c>
       <c r="J46" t="s">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="K46" s="8">
+        <f>0.5/1000/0.15</f>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L46" t="s">
+        <v>22</v>
+      </c>
+      <c r="N46" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A47" s="4"/>
+      <c r="B47" s="4"/>
+      <c r="C47" t="s">
+        <v>115</v>
+      </c>
+      <c r="J47" t="s">
+        <v>113</v>
+      </c>
+      <c r="K47" s="8">
         <f>1.2/1000/0.15</f>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="L46" t="s">
-        <v>36</v>
-      </c>
-      <c r="N46" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="4"/>
-      <c r="C48" t="s">
-        <v>10</v>
-      </c>
-      <c r="J48" t="s">
-        <v>31</v>
-      </c>
-      <c r="K48" s="6">
-        <f t="shared" ref="K48:K53" si="0">K41</f>
-        <v>0.15</v>
-      </c>
-      <c r="L48" t="s">
-        <v>32</v>
-      </c>
-      <c r="M48" s="7" t="s">
-        <v>41</v>
+      <c r="L47" t="s">
+        <v>23</v>
+      </c>
+      <c r="N47" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="J49" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="K49" s="6">
-        <f t="shared" si="0"/>
-        <v>0.9</v>
+        <f t="shared" ref="K49:K54" si="0">K42</f>
+        <v>0.15</v>
       </c>
       <c r="L49" t="s">
-        <v>33</v>
+        <v>19</v>
+      </c>
+      <c r="M49" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="4"/>
       <c r="B50" s="4"/>
       <c r="C50" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="J50" t="s">
-        <v>49</v>
-      </c>
-      <c r="K50" s="9">
+        <v>109</v>
+      </c>
+      <c r="K50" s="6">
         <f t="shared" si="0"/>
-        <v>0.55000000000000004</v>
+        <v>0.9</v>
       </c>
       <c r="L50" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
       <c r="C51" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="J51" t="s">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="K51" s="9">
         <f t="shared" si="0"/>
-        <v>2.5333333333333333E-2</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="L51" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="J52" t="s">
-        <v>26</v>
+        <v>111</v>
       </c>
       <c r="K52" s="9">
         <f t="shared" si="0"/>
-        <v>3.3333333333333335E-3</v>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L52" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" t="s">
-        <v>10</v>
+        <v>116</v>
       </c>
       <c r="J53" t="s">
-        <v>27</v>
+        <v>112</v>
       </c>
       <c r="K53" s="9">
         <f t="shared" si="0"/>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L53" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54" s="4"/>
+      <c r="B54" s="4"/>
+      <c r="C54" t="s">
+        <v>116</v>
+      </c>
+      <c r="J54" t="s">
+        <v>113</v>
+      </c>
+      <c r="K54" s="9">
+        <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="L53" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A55" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B55" s="4"/>
-      <c r="C55" t="s">
-        <v>59</v>
-      </c>
-      <c r="J55" t="s">
-        <v>31</v>
-      </c>
-      <c r="K55">
-        <v>1</v>
-      </c>
-      <c r="L55" t="s">
-        <v>32</v>
+      <c r="L54" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B56" s="4"/>
       <c r="C56" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="J56" t="s">
-        <v>24</v>
+        <v>108</v>
       </c>
       <c r="K56">
-        <v>0.88</v>
+        <v>1</v>
       </c>
       <c r="L56" t="s">
-        <v>33</v>
-      </c>
-      <c r="N56" t="s">
-        <v>48</v>
+        <v>19</v>
       </c>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B57" s="4"/>
       <c r="C57" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="J57" t="s">
-        <v>49</v>
-      </c>
-      <c r="K57" s="8">
-        <v>0.3</v>
+        <v>109</v>
+      </c>
+      <c r="K57">
+        <v>0.88</v>
       </c>
       <c r="L57" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="N57" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B58" s="4"/>
       <c r="C58" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="J58" t="s">
-        <v>25</v>
-      </c>
-      <c r="K58" s="4">
+        <v>110</v>
+      </c>
+      <c r="K58" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="L58" t="s">
+        <v>29</v>
+      </c>
+      <c r="N58" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B59" s="4"/>
+      <c r="C59" t="s">
+        <v>43</v>
+      </c>
+      <c r="J59" t="s">
+        <v>111</v>
+      </c>
+      <c r="K59" s="4">
         <f>2.1/100</f>
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="L58" t="s">
-        <v>34</v>
-      </c>
-      <c r="N58" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
+      <c r="L59" t="s">
         <v>21</v>
       </c>
-      <c r="B59" s="4"/>
-      <c r="C59" t="s">
-        <v>59</v>
-      </c>
-      <c r="J59" t="s">
-        <v>26</v>
-      </c>
-      <c r="K59" s="11">
+      <c r="N59" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B60" s="4"/>
+      <c r="C60" t="s">
+        <v>43</v>
+      </c>
+      <c r="J60" t="s">
+        <v>112</v>
+      </c>
+      <c r="K60" s="11">
         <f>0.27/100</f>
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="L59" t="s">
-        <v>35</v>
-      </c>
-      <c r="N59" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B60" s="4"/>
-      <c r="C60" t="s">
-        <v>59</v>
-      </c>
-      <c r="J60" t="s">
-        <v>27</v>
-      </c>
-      <c r="K60" s="11">
+      <c r="L60" t="s">
+        <v>22</v>
+      </c>
+      <c r="N60" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A61" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B61" s="4"/>
+      <c r="C61" t="s">
+        <v>43</v>
+      </c>
+      <c r="J61" t="s">
+        <v>113</v>
+      </c>
+      <c r="K61" s="11">
         <f>2.34/100</f>
         <v>2.3399999999999997E-2</v>
       </c>
-      <c r="L60" t="s">
-        <v>36</v>
-      </c>
-      <c r="N60" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A61" s="4"/>
-      <c r="B61" s="4"/>
-      <c r="K61" s="11"/>
+      <c r="L61" t="s">
+        <v>23</v>
+      </c>
+      <c r="N61" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A62" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-      <c r="G62" s="2"/>
-      <c r="H62" s="2"/>
-      <c r="I62" s="2"/>
-      <c r="J62" s="2"/>
-      <c r="K62" s="2"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
-      <c r="N62" s="2"/>
+      <c r="A62" s="4"/>
+      <c r="B62" s="4"/>
+      <c r="K62" s="11"/>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A63" s="4"/>
-      <c r="B63" s="4"/>
-      <c r="C63" s="4"/>
-      <c r="D63" s="4"/>
-      <c r="E63" s="4"/>
-      <c r="F63" s="4"/>
-      <c r="G63" s="4"/>
-      <c r="H63" s="4"/>
-      <c r="I63" s="4"/>
-      <c r="J63" s="4"/>
-      <c r="K63" s="4"/>
-      <c r="L63" s="4"/>
-      <c r="M63" s="4"/>
-      <c r="N63" s="4"/>
+      <c r="A63" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B63" s="2"/>
+      <c r="C63" s="2"/>
+      <c r="D63" s="2"/>
+      <c r="E63" s="2"/>
+      <c r="F63" s="2"/>
+      <c r="G63" s="2"/>
+      <c r="H63" s="2"/>
+      <c r="I63" s="2"/>
+      <c r="J63" s="2"/>
+      <c r="K63" s="2"/>
+      <c r="L63" s="2"/>
+      <c r="M63" s="2"/>
+      <c r="N63" s="2"/>
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
-      <c r="J64" t="s">
-        <v>72</v>
-      </c>
-      <c r="K64" s="11">
-        <v>0.71750000000000003</v>
-      </c>
-      <c r="L64" t="s">
-        <v>73</v>
-      </c>
-      <c r="N64" t="s">
-        <v>57</v>
-      </c>
+      <c r="C64" s="4"/>
+      <c r="D64" s="4"/>
+      <c r="E64" s="4"/>
+      <c r="F64" s="4"/>
+      <c r="G64" s="4"/>
+      <c r="H64" s="4"/>
+      <c r="I64" s="4"/>
+      <c r="J64" s="4"/>
+      <c r="K64" s="4"/>
+      <c r="L64" s="4"/>
+      <c r="M64" s="4"/>
+      <c r="N64" s="4"/>
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="J65" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="K65" s="11">
-        <v>1.9496</v>
+        <v>0.71750000000000003</v>
       </c>
       <c r="L65" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="N65" t="s">
-        <v>57</v>
+        <v>41</v>
       </c>
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
       <c r="J66" t="s">
-        <v>112</v>
-      </c>
-      <c r="K66" s="13">
+        <v>58</v>
+      </c>
+      <c r="K66" s="11">
+        <v>1.9496</v>
+      </c>
+      <c r="L66" t="s">
+        <v>57</v>
+      </c>
+      <c r="N66" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A67" s="4"/>
+      <c r="B67" s="4"/>
+      <c r="J67" t="s">
+        <v>96</v>
+      </c>
+      <c r="K67" s="13">
         <f>50*(1/3.6)</f>
         <v>13.888888888888889</v>
       </c>
-      <c r="L66" t="s">
-        <v>108</v>
-      </c>
-      <c r="M66" t="s">
-        <v>107</v>
-      </c>
-      <c r="N66" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A68" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="B68" s="2"/>
-      <c r="C68" s="2"/>
-      <c r="D68" s="2"/>
-      <c r="E68" s="2"/>
-      <c r="F68" s="2"/>
-      <c r="G68" s="2"/>
-      <c r="H68" s="2"/>
-      <c r="I68" s="2"/>
-      <c r="J68" s="2"/>
-      <c r="K68" s="2"/>
-      <c r="L68" s="2"/>
-      <c r="M68" s="2"/>
-      <c r="N68" s="2"/>
+      <c r="L67" t="s">
+        <v>92</v>
+      </c>
+      <c r="M67" t="s">
+        <v>91</v>
+      </c>
+      <c r="N67" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="14" t="s">
-        <v>101</v>
-      </c>
+      <c r="A69" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
+      <c r="I69" s="2"/>
+      <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
+      <c r="L69" s="2"/>
+      <c r="M69" s="2"/>
+      <c r="N69" s="2"/>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J70" t="s">
-        <v>44</v>
-      </c>
-      <c r="K70" s="4">
-        <v>90</v>
-      </c>
-      <c r="L70" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M70" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="N70" t="s">
-        <v>60</v>
+      <c r="A70" s="14" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J71" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="K71" s="4">
-        <v>0.22</v>
+        <v>90</v>
       </c>
       <c r="L71" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="M71" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="M71" s="4" t="s">
+        <v>46</v>
+      </c>
       <c r="N71" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J72" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="K72" s="4">
-        <v>3.4</v>
+        <v>0.22</v>
       </c>
       <c r="L72" s="4" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="M72" s="7"/>
       <c r="N72" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J73" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="K73" s="4">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="L73" s="4" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="M73" s="7"/>
       <c r="N73" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A74" s="14" t="s">
-        <v>102</v>
-      </c>
-      <c r="K74" s="4"/>
-      <c r="L74" s="4"/>
+      <c r="J74" t="s">
+        <v>35</v>
+      </c>
+      <c r="K74" s="4">
+        <v>5</v>
+      </c>
+      <c r="L74" s="4" t="s">
+        <v>38</v>
+      </c>
       <c r="M74" s="7"/>
+      <c r="N74" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I75" t="s">
-        <v>94</v>
-      </c>
-      <c r="J75" t="s">
-        <v>96</v>
-      </c>
-      <c r="K75" s="4">
-        <v>0.61</v>
-      </c>
-      <c r="L75" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M75" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="N75" t="s">
-        <v>57</v>
-      </c>
+      <c r="A75" s="14" t="s">
+        <v>86</v>
+      </c>
+      <c r="K75" s="4"/>
+      <c r="L75" s="4"/>
+      <c r="M75" s="7"/>
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.25">
       <c r="I76" t="s">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="J76" t="s">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="K76" s="4">
+        <v>0.61</v>
+      </c>
+      <c r="L76" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M76" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="N76" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I77" t="s">
+        <v>79</v>
+      </c>
+      <c r="J77" t="s">
+        <v>80</v>
+      </c>
+      <c r="K77" s="4">
         <v>0.99</v>
       </c>
-      <c r="L76" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="M76" s="7"/>
-      <c r="N76" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A77" s="14" t="s">
-        <v>104</v>
+      <c r="L77" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M77" s="7"/>
+      <c r="N77" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C78" t="s">
-        <v>8</v>
-      </c>
-      <c r="J78" t="s">
-        <v>39</v>
-      </c>
-      <c r="K78">
-        <v>63</v>
-      </c>
-      <c r="L78" t="s">
-        <v>70</v>
-      </c>
-      <c r="N78" t="s">
-        <v>48</v>
+      <c r="A78" s="14" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C79" t="s">
-        <v>9</v>
+        <v>114</v>
       </c>
       <c r="J79" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="K79">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="L79" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="N79" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C80" t="s">
-        <v>10</v>
+        <v>115</v>
       </c>
       <c r="J80" t="s">
-        <v>39</v>
-      </c>
-      <c r="K80" s="6">
-        <f>K79</f>
+        <v>25</v>
+      </c>
+      <c r="K80">
         <v>59</v>
       </c>
       <c r="L80" t="s">
-        <v>70</v>
-      </c>
-      <c r="M80" s="7" t="s">
-        <v>41</v>
+        <v>54</v>
+      </c>
+      <c r="N80" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A81" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B81" s="4"/>
       <c r="C81" t="s">
+        <v>116</v>
+      </c>
+      <c r="J81" t="s">
+        <v>25</v>
+      </c>
+      <c r="K81" s="6">
+        <f>K80</f>
         <v>59</v>
       </c>
-      <c r="J81" t="s">
-        <v>39</v>
-      </c>
-      <c r="K81">
+      <c r="L81" t="s">
+        <v>54</v>
+      </c>
+      <c r="M81" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A82" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B82" s="4"/>
+      <c r="C82" t="s">
+        <v>43</v>
+      </c>
+      <c r="J82" t="s">
+        <v>25</v>
+      </c>
+      <c r="K82">
         <v>56</v>
       </c>
-      <c r="L81" t="s">
-        <v>70</v>
-      </c>
-      <c r="M81" t="s">
-        <v>78</v>
-      </c>
-      <c r="N81" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C82" t="s">
-        <v>46</v>
-      </c>
-      <c r="J82" t="s">
-        <v>39</v>
-      </c>
-      <c r="K82" s="4">
+      <c r="L82" t="s">
+        <v>54</v>
+      </c>
+      <c r="M82" t="s">
+        <v>62</v>
+      </c>
+      <c r="N82" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C83" t="s">
+        <v>31</v>
+      </c>
+      <c r="J83" t="s">
+        <v>25</v>
+      </c>
+      <c r="K83" s="4">
         <v>65</v>
       </c>
-      <c r="L82" t="s">
-        <v>70</v>
-      </c>
-      <c r="M82" t="s">
-        <v>77</v>
-      </c>
-      <c r="N82" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A83" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="K83" s="4"/>
-      <c r="L83" s="4"/>
-      <c r="M83" s="7"/>
+      <c r="L83" t="s">
+        <v>54</v>
+      </c>
+      <c r="M83" t="s">
+        <v>61</v>
+      </c>
+      <c r="N83" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H84" t="s">
-        <v>100</v>
-      </c>
-      <c r="J84" t="s">
-        <v>97</v>
-      </c>
-      <c r="K84" s="13">
+      <c r="A84" s="14" t="s">
+        <v>87</v>
+      </c>
+      <c r="K84" s="4"/>
+      <c r="L84" s="4"/>
+      <c r="M84" s="7"/>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H85" t="s">
+        <v>84</v>
+      </c>
+      <c r="J85" t="s">
+        <v>81</v>
+      </c>
+      <c r="K85" s="13">
         <f>1041/(50+3+1041)*100</f>
         <v>95.155393053016454</v>
       </c>
-      <c r="L84" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M84" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="N84" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H85" t="s">
-        <v>95</v>
-      </c>
-      <c r="J85" t="s">
-        <v>97</v>
-      </c>
-      <c r="K85" s="12">
+      <c r="L85" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M85" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="N85" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H86" t="s">
+        <v>79</v>
+      </c>
+      <c r="J86" t="s">
+        <v>81</v>
+      </c>
+      <c r="K86" s="12">
         <f>50/(50+3+1041)*100</f>
         <v>4.5703839122486292</v>
       </c>
-      <c r="L85" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M85" s="4"/>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H86" t="s">
-        <v>94</v>
-      </c>
-      <c r="J86" t="s">
-        <v>97</v>
-      </c>
-      <c r="K86" s="12">
+      <c r="L86" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M86" s="4"/>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H87" t="s">
+        <v>78</v>
+      </c>
+      <c r="J87" t="s">
+        <v>81</v>
+      </c>
+      <c r="K87" s="12">
         <f>3/(50+3+1041)*100</f>
         <v>0.27422303473491771</v>
       </c>
-      <c r="L86" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="M86" s="4"/>
-    </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A87" s="14" t="s">
-        <v>110</v>
-      </c>
-      <c r="K87" s="4"/>
-      <c r="L87" s="4"/>
+      <c r="L87" s="4" t="s">
+        <v>6</v>
+      </c>
       <c r="M87" s="4"/>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A88" s="15"/>
-      <c r="B88" s="3"/>
-      <c r="C88" s="3"/>
-      <c r="D88" s="3"/>
-      <c r="E88" s="3"/>
-      <c r="F88" s="3"/>
-      <c r="G88" s="3"/>
-      <c r="H88" s="3"/>
-      <c r="I88" s="3"/>
-      <c r="J88" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="K88" s="3">
-        <v>0</v>
-      </c>
-      <c r="L88" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="M88" s="3" t="s">
-        <v>109</v>
-      </c>
+      <c r="A88" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="K88" s="4"/>
+      <c r="L88" s="4"/>
+      <c r="M88" s="4"/>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A89" s="15"/>
@@ -2087,214 +2088,237 @@
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
       <c r="J89" s="3" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="K89" s="3">
         <v>0</v>
       </c>
       <c r="L89" s="3" t="s">
-        <v>113</v>
+        <v>6</v>
       </c>
       <c r="M89" s="3" t="s">
-        <v>109</v>
+        <v>93</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H90" t="s">
-        <v>100</v>
-      </c>
-      <c r="J90" t="s">
-        <v>98</v>
-      </c>
-      <c r="K90" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="L90" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="M90" s="7"/>
-      <c r="N90" t="s">
-        <v>69</v>
+      <c r="A90" s="15"/>
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="H90" s="3"/>
+      <c r="I90" s="3"/>
+      <c r="J90" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="K90" s="3">
+        <v>0</v>
+      </c>
+      <c r="L90" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="M90" s="3" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H91" t="s">
+        <v>84</v>
+      </c>
+      <c r="J91" t="s">
+        <v>82</v>
+      </c>
+      <c r="K91" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="L91" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="I91" t="s">
-        <v>94</v>
-      </c>
-      <c r="J91" t="s">
-        <v>99</v>
-      </c>
-      <c r="K91" s="10">
+      <c r="M91" s="7"/>
+      <c r="N91" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H92" t="s">
+        <v>84</v>
+      </c>
+      <c r="I92" t="s">
+        <v>78</v>
+      </c>
+      <c r="J92" t="s">
+        <v>83</v>
+      </c>
+      <c r="K92" s="10">
         <f>0.9 * (1/3.6) / 0.6 / 0.718</f>
         <v>0.5803156917363046</v>
       </c>
-      <c r="L91" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="M91" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="N91" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A92" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="K92" s="4"/>
-      <c r="L92" s="4"/>
-      <c r="M92" s="7"/>
+      <c r="L92" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="M92" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="N92" t="s">
+        <v>53</v>
+      </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J93" t="s">
-        <v>65</v>
-      </c>
-      <c r="K93" s="11">
+      <c r="A93" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="K93" s="4"/>
+      <c r="L93" s="4"/>
+      <c r="M93" s="7"/>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J94" t="s">
+        <v>49</v>
+      </c>
+      <c r="K94" s="11">
         <f>238/0.74/1000</f>
         <v>0.32162162162162161</v>
       </c>
-      <c r="L93" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="M93" s="7"/>
-      <c r="N93" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J94" t="s">
-        <v>75</v>
-      </c>
-      <c r="K94" s="12">
-        <v>1.5</v>
-      </c>
       <c r="L94" s="4" t="s">
-        <v>76</v>
+        <v>29</v>
       </c>
       <c r="M94" s="7"/>
       <c r="N94" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J95" t="s">
-        <v>66</v>
-      </c>
-      <c r="K95" s="13">
+        <v>59</v>
+      </c>
+      <c r="K95" s="12">
+        <v>1.5</v>
+      </c>
+      <c r="L95" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="L95" s="4" t="s">
-        <v>67</v>
       </c>
       <c r="M95" s="7"/>
       <c r="N95" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="97" spans="6:12" x14ac:dyDescent="0.25">
-      <c r="F97" t="s">
-        <v>81</v>
-      </c>
-      <c r="G97" t="s">
-        <v>83</v>
-      </c>
-      <c r="J97" t="s">
-        <v>82</v>
-      </c>
-      <c r="K97">
-        <v>2.75</v>
-      </c>
-      <c r="L97" t="s">
-        <v>67</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J96" t="s">
+        <v>50</v>
+      </c>
+      <c r="K96" s="13">
+        <v>60</v>
+      </c>
+      <c r="L96" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M96" s="7"/>
+      <c r="N96" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="98" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F98" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G98" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
       <c r="J98" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="K98">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="L98" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
     </row>
     <row r="99" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F99" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G99" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="J99" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="K99">
         <v>0</v>
       </c>
       <c r="L99" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="100" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F100" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G100" t="s">
-        <v>86</v>
+        <v>69</v>
       </c>
       <c r="J100" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="K100">
         <v>0</v>
       </c>
       <c r="L100" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="102" spans="6:12" x14ac:dyDescent="0.25">
-      <c r="F102" t="s">
-        <v>88</v>
-      </c>
-      <c r="G102" t="s">
-        <v>88</v>
-      </c>
-      <c r="J102" t="s">
-        <v>82</v>
-      </c>
-      <c r="K102">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="101" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F101" t="s">
+        <v>65</v>
+      </c>
+      <c r="G101" t="s">
+        <v>70</v>
+      </c>
+      <c r="J101" t="s">
+        <v>66</v>
+      </c>
+      <c r="K101">
         <v>0</v>
       </c>
-      <c r="L102" t="s">
-        <v>90</v>
+      <c r="L101" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="103" spans="6:12" x14ac:dyDescent="0.25">
       <c r="F103" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="G103" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="J103" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="K103">
         <v>0</v>
       </c>
       <c r="L103" t="s">
-        <v>91</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="104" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="F104" t="s">
+        <v>73</v>
+      </c>
+      <c r="G104" t="s">
+        <v>73</v>
+      </c>
+      <c r="J104" t="s">
+        <v>66</v>
+      </c>
+      <c r="K104">
+        <v>0</v>
+      </c>
+      <c r="L104" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -2311,22 +2335,22 @@
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added references to all data
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="122">
   <si>
     <t>parameter</t>
   </si>
@@ -376,6 +376,21 @@
   </si>
   <si>
     <t>food waste, processing</t>
+  </si>
+  <si>
+    <t>Energigas Sverige (2023), Tabell 6</t>
+  </si>
+  <si>
+    <t>Energigas Sverige (2023) Produktion av biogas och rötrester och dess användning år 2022</t>
+  </si>
+  <si>
+    <t>NIR 2022, Table 5.18</t>
+  </si>
+  <si>
+    <t>Swedish IIR 2023 Table 5-12</t>
+  </si>
+  <si>
+    <t>Assumed same as anaerobically digested manure</t>
   </si>
 </sst>
 </file>
@@ -509,7 +524,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -2034,7 +2049,7 @@
         <v>90</v>
       </c>
       <c r="N85" t="s">
-        <v>76</v>
+        <v>117</v>
       </c>
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.25">
@@ -2052,6 +2067,9 @@
         <v>6</v>
       </c>
       <c r="M86" s="4"/>
+      <c r="N86" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H87" t="s">
@@ -2068,6 +2086,9 @@
         <v>6</v>
       </c>
       <c r="M87" s="4"/>
+      <c r="N87" t="s">
+        <v>117</v>
+      </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A88" s="14" t="s">
@@ -2219,7 +2240,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="98" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="98" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F98" t="s">
         <v>65</v>
       </c>
@@ -2235,8 +2256,14 @@
       <c r="L98" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="99" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="M98" t="s">
+        <v>121</v>
+      </c>
+      <c r="N98" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="99" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F99" t="s">
         <v>65</v>
       </c>
@@ -2253,7 +2280,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="100" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="100" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F100" t="s">
         <v>65</v>
       </c>
@@ -2270,7 +2297,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="101" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="101" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F101" t="s">
         <v>65</v>
       </c>
@@ -2286,8 +2313,11 @@
       <c r="L101" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="103" spans="6:12" x14ac:dyDescent="0.25">
+      <c r="N101" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="103" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F103" t="s">
         <v>72</v>
       </c>
@@ -2304,7 +2334,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="104" spans="6:12" x14ac:dyDescent="0.25">
+    <row r="104" spans="6:14" x14ac:dyDescent="0.25">
       <c r="F104" t="s">
         <v>73</v>
       </c>
@@ -2330,7 +2360,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="A2:A5"/>
+  <dimension ref="A2:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2340,16 +2370,21 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>52</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implemented and parametrised surpluss by-products to waste treatment
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Documents\#1 Projekt\MISTRA Food Futures WP5\CIBUSmod Food Systems Model\CIBUSmod\data\default\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="325" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="131">
   <si>
     <t>parameter</t>
   </si>
@@ -391,6 +391,33 @@
   </si>
   <si>
     <t>Assumed same as anaerobically digested manure</t>
+  </si>
+  <si>
+    <t>Slaughterhouse waste</t>
+  </si>
+  <si>
+    <t>slaughterhouse by-products</t>
+  </si>
+  <si>
+    <t>Dairy waste</t>
+  </si>
+  <si>
+    <t>Brewaries spent grain</t>
+  </si>
+  <si>
+    <t>cereal by-products</t>
+  </si>
+  <si>
+    <t>dairy by-products</t>
+  </si>
+  <si>
+    <t>by-product waste</t>
+  </si>
+  <si>
+    <t>other by-products</t>
+  </si>
+  <si>
+    <t>Food waste, grocery stores</t>
   </si>
 </sst>
 </file>
@@ -489,7 +516,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -506,6 +533,8 @@
     <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -524,7 +553,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office-tema">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -787,7 +816,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O104"/>
+  <dimension ref="A1:O138"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -1162,129 +1191,110 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="C27" t="s">
+        <v>128</v>
+      </c>
+      <c r="E27" t="s">
+        <v>8</v>
+      </c>
+      <c r="J27" t="s">
+        <v>5</v>
+      </c>
+      <c r="K27">
+        <v>100</v>
+      </c>
+      <c r="L27" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B27" s="5"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="5"/>
-      <c r="E27" s="5"/>
-      <c r="F27" s="5"/>
-      <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-      <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
-      <c r="K27" s="5"/>
-      <c r="L27" s="5"/>
-      <c r="M27" s="5"/>
-      <c r="N27" s="5"/>
-    </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="4" t="s">
+      <c r="B29" s="5"/>
+      <c r="C29" s="5"/>
+      <c r="D29" s="5"/>
+      <c r="E29" s="5"/>
+      <c r="F29" s="5"/>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+      <c r="N29" s="5"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A31" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B29" s="4"/>
-      <c r="C29" t="s">
+      <c r="B31" s="4"/>
+      <c r="C31" t="s">
         <v>43</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E31" t="s">
         <v>8</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J31" t="s">
         <v>5</v>
       </c>
-      <c r="K29">
+      <c r="K31">
         <v>100</v>
       </c>
-      <c r="L29" t="s">
+      <c r="L31" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="2" t="s">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-      <c r="G31" s="2"/>
-      <c r="H31" s="2"/>
-      <c r="I31" s="2"/>
-      <c r="J31" s="2"/>
-      <c r="K31" s="2"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J33" s="3" t="s">
+      <c r="B33" s="2"/>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="2"/>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J35" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="K33" s="3">
+      <c r="K35" s="3">
         <v>0.5</v>
       </c>
-      <c r="L33" s="3" t="s">
+      <c r="L35" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="M33" s="3" t="s">
+      <c r="M35" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="4"/>
-      <c r="B35" s="4"/>
-      <c r="C35" t="s">
-        <v>114</v>
-      </c>
-      <c r="J35" t="s">
-        <v>108</v>
-      </c>
-      <c r="K35">
-        <v>0.33</v>
-      </c>
-      <c r="L35" t="s">
-        <v>19</v>
-      </c>
-      <c r="M35" t="s">
-        <v>26</v>
-      </c>
-      <c r="N35" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="4"/>
-      <c r="B36" s="4"/>
-      <c r="C36" t="s">
-        <v>114</v>
-      </c>
-      <c r="J36" t="s">
-        <v>109</v>
-      </c>
-      <c r="K36">
-        <v>0.85</v>
-      </c>
-      <c r="L36" t="s">
-        <v>20</v>
-      </c>
-      <c r="N36" t="s">
-        <v>33</v>
-      </c>
-    </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
       <c r="C37" t="s">
         <v>114</v>
       </c>
       <c r="J37" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="K37">
-        <v>0.46100000000000002</v>
+        <v>0.33</v>
       </c>
       <c r="L37" t="s">
-        <v>29</v>
+        <v>19</v>
+      </c>
+      <c r="M37" t="s">
+        <v>26</v>
       </c>
       <c r="N37" t="s">
         <v>33</v>
@@ -1297,40 +1307,33 @@
         <v>114</v>
       </c>
       <c r="J38" t="s">
-        <v>111</v>
-      </c>
-      <c r="K38" s="8">
-        <f>8.3/1000/0.33</f>
-        <v>2.515151515151515E-2</v>
+        <v>109</v>
+      </c>
+      <c r="K38">
+        <v>0.85</v>
       </c>
       <c r="L38" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N38" t="s">
-        <v>44</v>
-      </c>
-      <c r="O38" t="s">
-        <v>48</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="4"/>
-      <c r="B39" s="4"/>
       <c r="C39" t="s">
         <v>114</v>
       </c>
       <c r="J39" t="s">
-        <v>112</v>
-      </c>
-      <c r="K39" s="8">
-        <f>1/1000/0.33</f>
-        <v>3.0303030303030303E-3</v>
+        <v>110</v>
+      </c>
+      <c r="K39">
+        <v>0.46100000000000002</v>
       </c>
       <c r="L39" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="N39" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
@@ -1340,16 +1343,39 @@
         <v>114</v>
       </c>
       <c r="J40" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="K40" s="8">
-        <f>2.6/1000/0.33</f>
-        <v>7.8787878787878775E-3</v>
+        <f>8.3/1000/0.33</f>
+        <v>2.515151515151515E-2</v>
       </c>
       <c r="L40" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N40" t="s">
+        <v>44</v>
+      </c>
+      <c r="O40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A41" s="4"/>
+      <c r="B41" s="4"/>
+      <c r="C41" t="s">
+        <v>114</v>
+      </c>
+      <c r="J41" t="s">
+        <v>112</v>
+      </c>
+      <c r="K41" s="8">
+        <f>1/1000/0.33</f>
+        <v>3.0303030303030303E-3</v>
+      </c>
+      <c r="L41" t="s">
+        <v>22</v>
+      </c>
+      <c r="N41" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1357,53 +1383,39 @@
       <c r="A42" s="4"/>
       <c r="B42" s="4"/>
       <c r="C42" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J42" t="s">
-        <v>108</v>
-      </c>
-      <c r="K42">
-        <v>0.15</v>
+        <v>113</v>
+      </c>
+      <c r="K42" s="8">
+        <f>2.6/1000/0.33</f>
+        <v>7.8787878787878775E-3</v>
       </c>
       <c r="L42" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="N42" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="4"/>
-      <c r="B43" s="4"/>
-      <c r="C43" t="s">
-        <v>115</v>
-      </c>
-      <c r="J43" t="s">
-        <v>109</v>
-      </c>
-      <c r="K43" s="10">
-        <v>0.9</v>
-      </c>
-      <c r="L43" t="s">
-        <v>20</v>
-      </c>
-      <c r="M43" s="7"/>
-      <c r="N43" t="s">
-        <v>44</v>
-      </c>
-    </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A44" s="4"/>
+      <c r="B44" s="4"/>
       <c r="C44" t="s">
         <v>115</v>
       </c>
       <c r="J44" t="s">
-        <v>110</v>
-      </c>
-      <c r="K44" s="8">
-        <v>0.55000000000000004</v>
+        <v>108</v>
+      </c>
+      <c r="K44">
+        <v>0.15</v>
       </c>
       <c r="L44" t="s">
-        <v>29</v>
+        <v>19</v>
+      </c>
+      <c r="M44" t="s">
+        <v>130</v>
       </c>
       <c r="N44" t="s">
         <v>44</v>
@@ -1416,34 +1428,31 @@
         <v>115</v>
       </c>
       <c r="J45" t="s">
-        <v>111</v>
-      </c>
-      <c r="K45" s="8">
-        <f>3.8/1000/0.15</f>
-        <v>2.5333333333333333E-2</v>
+        <v>109</v>
+      </c>
+      <c r="K45" s="10">
+        <v>0.9</v>
       </c>
       <c r="L45" t="s">
-        <v>21</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="M45" s="7"/>
       <c r="N45" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="4"/>
-      <c r="B46" s="4"/>
       <c r="C46" t="s">
         <v>115</v>
       </c>
       <c r="J46" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="K46" s="8">
-        <f>0.5/1000/0.15</f>
-        <v>3.3333333333333335E-3</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="L46" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="N46" t="s">
         <v>44</v>
@@ -1456,16 +1465,36 @@
         <v>115</v>
       </c>
       <c r="J47" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="K47" s="8">
-        <f>1.2/1000/0.15</f>
-        <v>8.0000000000000002E-3</v>
+        <f>3.8/1000/0.15</f>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L47" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N47" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A48" s="4"/>
+      <c r="B48" s="4"/>
+      <c r="C48" t="s">
+        <v>115</v>
+      </c>
+      <c r="J48" t="s">
+        <v>112</v>
+      </c>
+      <c r="K48" s="8">
+        <f>0.5/1000/0.15</f>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L48" t="s">
+        <v>22</v>
+      </c>
+      <c r="N48" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1473,37 +1502,20 @@
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J49" t="s">
-        <v>108</v>
-      </c>
-      <c r="K49" s="6">
-        <f t="shared" ref="K49:K54" si="0">K42</f>
-        <v>0.15</v>
+        <v>113</v>
+      </c>
+      <c r="K49" s="8">
+        <f>1.2/1000/0.15</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="L49" t="s">
-        <v>19</v>
-      </c>
-      <c r="M49" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A50" s="4"/>
-      <c r="B50" s="4"/>
-      <c r="C50" t="s">
-        <v>116</v>
-      </c>
-      <c r="J50" t="s">
-        <v>109</v>
-      </c>
-      <c r="K50" s="6">
-        <f t="shared" si="0"/>
-        <v>0.9</v>
-      </c>
-      <c r="L50" t="s">
-        <v>20</v>
+        <v>23</v>
+      </c>
+      <c r="N49" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -1513,14 +1525,17 @@
         <v>116</v>
       </c>
       <c r="J51" t="s">
-        <v>110</v>
-      </c>
-      <c r="K51" s="9">
-        <f t="shared" si="0"/>
-        <v>0.55000000000000004</v>
+        <v>108</v>
+      </c>
+      <c r="K51" s="6">
+        <f t="shared" ref="K51:K56" si="0">K44</f>
+        <v>0.15</v>
       </c>
       <c r="L51" t="s">
-        <v>29</v>
+        <v>19</v>
+      </c>
+      <c r="M51" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
@@ -1530,14 +1545,14 @@
         <v>116</v>
       </c>
       <c r="J52" t="s">
-        <v>111</v>
-      </c>
-      <c r="K52" s="9">
+        <v>109</v>
+      </c>
+      <c r="K52" s="16">
         <f t="shared" si="0"/>
-        <v>2.5333333333333333E-2</v>
+        <v>0.9</v>
       </c>
       <c r="L52" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
@@ -1547,14 +1562,14 @@
         <v>116</v>
       </c>
       <c r="J53" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="K53" s="9">
         <f t="shared" si="0"/>
-        <v>3.3333333333333335E-3</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="L53" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
@@ -1564,790 +1579,1397 @@
         <v>116</v>
       </c>
       <c r="J54" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="K54" s="9">
         <f t="shared" si="0"/>
-        <v>8.0000000000000002E-3</v>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L54" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A55" s="4"/>
+      <c r="B55" s="4"/>
+      <c r="C55" t="s">
+        <v>116</v>
+      </c>
+      <c r="J55" t="s">
+        <v>112</v>
+      </c>
+      <c r="K55" s="9">
+        <f t="shared" si="0"/>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L55" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="A56" s="4"/>
       <c r="B56" s="4"/>
       <c r="C56" t="s">
+        <v>116</v>
+      </c>
+      <c r="J56" t="s">
+        <v>113</v>
+      </c>
+      <c r="K56" s="9">
+        <f t="shared" si="0"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="L56" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B58" t="s">
+        <v>123</v>
+      </c>
+      <c r="C58" t="s">
+        <v>128</v>
+      </c>
+      <c r="J58" t="s">
+        <v>108</v>
+      </c>
+      <c r="K58">
+        <v>0.16</v>
+      </c>
+      <c r="L58" t="s">
+        <v>19</v>
+      </c>
+      <c r="M58" t="s">
+        <v>122</v>
+      </c>
+      <c r="N58" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>123</v>
+      </c>
+      <c r="C59" t="s">
+        <v>128</v>
+      </c>
+      <c r="J59" t="s">
+        <v>109</v>
+      </c>
+      <c r="K59" s="17">
+        <v>0.9</v>
+      </c>
+      <c r="L59" t="s">
+        <v>20</v>
+      </c>
+      <c r="N59" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B60" t="s">
+        <v>123</v>
+      </c>
+      <c r="C60" t="s">
+        <v>128</v>
+      </c>
+      <c r="J60" t="s">
+        <v>110</v>
+      </c>
+      <c r="K60">
+        <v>0.434</v>
+      </c>
+      <c r="L60" t="s">
+        <v>29</v>
+      </c>
+      <c r="N60" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>123</v>
+      </c>
+      <c r="C61" t="s">
+        <v>128</v>
+      </c>
+      <c r="J61" t="s">
+        <v>111</v>
+      </c>
+      <c r="K61" s="8">
+        <f>3.8/1000/0.16</f>
+        <v>2.375E-2</v>
+      </c>
+      <c r="L61" t="s">
+        <v>21</v>
+      </c>
+      <c r="N61" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B62" t="s">
+        <v>123</v>
+      </c>
+      <c r="C62" t="s">
+        <v>128</v>
+      </c>
+      <c r="J62" t="s">
+        <v>112</v>
+      </c>
+      <c r="K62" s="8">
+        <f>0.4/1000/0.16</f>
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="L62" t="s">
+        <v>22</v>
+      </c>
+      <c r="N62" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B63" t="s">
+        <v>123</v>
+      </c>
+      <c r="C63" t="s">
+        <v>128</v>
+      </c>
+      <c r="J63" t="s">
+        <v>113</v>
+      </c>
+      <c r="K63" s="8">
+        <f>0.7/1000/0.16</f>
+        <v>4.3749999999999995E-3</v>
+      </c>
+      <c r="L63" t="s">
+        <v>23</v>
+      </c>
+      <c r="N63" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>127</v>
+      </c>
+      <c r="C65" t="s">
+        <v>128</v>
+      </c>
+      <c r="J65" t="s">
+        <v>108</v>
+      </c>
+      <c r="K65">
+        <v>0.06</v>
+      </c>
+      <c r="L65" t="s">
+        <v>19</v>
+      </c>
+      <c r="M65" t="s">
+        <v>124</v>
+      </c>
+      <c r="N65" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>127</v>
+      </c>
+      <c r="C66" t="s">
+        <v>128</v>
+      </c>
+      <c r="J66" t="s">
+        <v>109</v>
+      </c>
+      <c r="K66" s="17">
+        <v>0.95</v>
+      </c>
+      <c r="L66" t="s">
+        <v>20</v>
+      </c>
+      <c r="N66" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>127</v>
+      </c>
+      <c r="C67" t="s">
+        <v>128</v>
+      </c>
+      <c r="J67" t="s">
+        <v>110</v>
+      </c>
+      <c r="K67" s="8">
+        <v>0.52</v>
+      </c>
+      <c r="L67" t="s">
+        <v>29</v>
+      </c>
+      <c r="N67" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>127</v>
+      </c>
+      <c r="C68" t="s">
+        <v>128</v>
+      </c>
+      <c r="J68" t="s">
+        <v>111</v>
+      </c>
+      <c r="K68" s="8">
+        <f>3.5/1000/0.06</f>
+        <v>5.8333333333333334E-2</v>
+      </c>
+      <c r="L68" t="s">
+        <v>21</v>
+      </c>
+      <c r="N68" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>127</v>
+      </c>
+      <c r="C69" t="s">
+        <v>128</v>
+      </c>
+      <c r="J69" t="s">
+        <v>112</v>
+      </c>
+      <c r="K69" s="8">
+        <f>0.3/1000/0.06</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="L69" t="s">
+        <v>22</v>
+      </c>
+      <c r="N69" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B70" t="s">
+        <v>127</v>
+      </c>
+      <c r="C70" t="s">
+        <v>128</v>
+      </c>
+      <c r="J70" t="s">
+        <v>113</v>
+      </c>
+      <c r="K70" s="8">
+        <f>0.6/1000/0.06</f>
+        <v>0.01</v>
+      </c>
+      <c r="L70" t="s">
+        <v>23</v>
+      </c>
+      <c r="N70" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="72" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B72" t="s">
+        <v>126</v>
+      </c>
+      <c r="C72" t="s">
+        <v>128</v>
+      </c>
+      <c r="J72" t="s">
+        <v>108</v>
+      </c>
+      <c r="K72">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L72" t="s">
+        <v>19</v>
+      </c>
+      <c r="M72" t="s">
+        <v>125</v>
+      </c>
+      <c r="N72" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="73" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B73" t="s">
+        <v>126</v>
+      </c>
+      <c r="C73" t="s">
+        <v>128</v>
+      </c>
+      <c r="J73" t="s">
+        <v>109</v>
+      </c>
+      <c r="K73" s="17">
+        <v>0.97</v>
+      </c>
+      <c r="L73" t="s">
+        <v>20</v>
+      </c>
+      <c r="N73" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="74" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B74" t="s">
+        <v>126</v>
+      </c>
+      <c r="C74" t="s">
+        <v>128</v>
+      </c>
+      <c r="J74" t="s">
+        <v>110</v>
+      </c>
+      <c r="K74">
+        <v>0.32300000000000001</v>
+      </c>
+      <c r="L74" t="s">
+        <v>29</v>
+      </c>
+      <c r="N74" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="75" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B75" t="s">
+        <v>126</v>
+      </c>
+      <c r="C75" t="s">
+        <v>128</v>
+      </c>
+      <c r="J75" t="s">
+        <v>111</v>
+      </c>
+      <c r="K75" s="8">
+        <f>3.7/1000/0.07</f>
+        <v>5.2857142857142853E-2</v>
+      </c>
+      <c r="L75" t="s">
+        <v>21</v>
+      </c>
+      <c r="N75" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="76" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B76" t="s">
+        <v>126</v>
+      </c>
+      <c r="C76" t="s">
+        <v>128</v>
+      </c>
+      <c r="J76" t="s">
+        <v>112</v>
+      </c>
+      <c r="K76" s="8">
+        <f>0.3/1000/0.07</f>
+        <v>4.2857142857142851E-3</v>
+      </c>
+      <c r="L76" t="s">
+        <v>22</v>
+      </c>
+      <c r="N76" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B77" t="s">
+        <v>126</v>
+      </c>
+      <c r="C77" t="s">
+        <v>128</v>
+      </c>
+      <c r="J77" t="s">
+        <v>113</v>
+      </c>
+      <c r="K77" s="8">
+        <f>0.5/1000/0.07</f>
+        <v>7.1428571428571426E-3</v>
+      </c>
+      <c r="L77" t="s">
+        <v>23</v>
+      </c>
+      <c r="N77" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>129</v>
+      </c>
+      <c r="C79" t="s">
+        <v>128</v>
+      </c>
+      <c r="J79" t="s">
+        <v>108</v>
+      </c>
+      <c r="K79" s="6">
+        <f>K44</f>
+        <v>0.15</v>
+      </c>
+      <c r="L79" t="s">
+        <v>19</v>
+      </c>
+      <c r="M79" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>129</v>
+      </c>
+      <c r="C80" t="s">
+        <v>128</v>
+      </c>
+      <c r="J80" t="s">
+        <v>109</v>
+      </c>
+      <c r="K80" s="6">
+        <f t="shared" ref="K80:K84" si="1">K45</f>
+        <v>0.9</v>
+      </c>
+      <c r="L80" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>129</v>
+      </c>
+      <c r="C81" t="s">
+        <v>128</v>
+      </c>
+      <c r="J81" t="s">
+        <v>110</v>
+      </c>
+      <c r="K81" s="9">
+        <f t="shared" si="1"/>
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="L81" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>129</v>
+      </c>
+      <c r="C82" t="s">
+        <v>128</v>
+      </c>
+      <c r="J82" t="s">
+        <v>111</v>
+      </c>
+      <c r="K82" s="9">
+        <f t="shared" si="1"/>
+        <v>2.5333333333333333E-2</v>
+      </c>
+      <c r="L82" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>129</v>
+      </c>
+      <c r="C83" t="s">
+        <v>128</v>
+      </c>
+      <c r="J83" t="s">
+        <v>112</v>
+      </c>
+      <c r="K83" s="9">
+        <f t="shared" si="1"/>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L83" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B84" t="s">
+        <v>129</v>
+      </c>
+      <c r="C84" t="s">
+        <v>128</v>
+      </c>
+      <c r="J84" t="s">
+        <v>113</v>
+      </c>
+      <c r="K84" s="9">
+        <f t="shared" si="1"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="L84" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A86" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B86" s="4"/>
+      <c r="C86" t="s">
         <v>43</v>
       </c>
-      <c r="J56" t="s">
+      <c r="J86" t="s">
         <v>108</v>
       </c>
-      <c r="K56">
+      <c r="K86">
         <v>1</v>
       </c>
-      <c r="L56" t="s">
+      <c r="L86" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A57" s="4" t="s">
+    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A87" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B57" s="4"/>
-      <c r="C57" t="s">
+      <c r="B87" s="4"/>
+      <c r="C87" t="s">
         <v>43</v>
       </c>
-      <c r="J57" t="s">
+      <c r="J87" t="s">
         <v>109</v>
       </c>
-      <c r="K57">
+      <c r="K87">
         <v>0.88</v>
       </c>
-      <c r="L57" t="s">
+      <c r="L87" t="s">
         <v>20</v>
       </c>
-      <c r="N57" t="s">
+      <c r="N87" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A58" s="4" t="s">
+    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A88" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B58" s="4"/>
-      <c r="C58" t="s">
+      <c r="B88" s="4"/>
+      <c r="C88" t="s">
         <v>43</v>
       </c>
-      <c r="J58" t="s">
+      <c r="J88" t="s">
         <v>110</v>
       </c>
-      <c r="K58" s="8">
+      <c r="K88" s="8">
         <v>0.3</v>
       </c>
-      <c r="L58" t="s">
+      <c r="L88" t="s">
         <v>29</v>
       </c>
-      <c r="N58" t="s">
+      <c r="N88" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A59" s="4" t="s">
+    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A89" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B59" s="4"/>
-      <c r="C59" t="s">
+      <c r="B89" s="4"/>
+      <c r="C89" t="s">
         <v>43</v>
       </c>
-      <c r="J59" t="s">
+      <c r="J89" t="s">
         <v>111</v>
       </c>
-      <c r="K59" s="4">
+      <c r="K89" s="4">
         <f>2.1/100</f>
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="L59" t="s">
+      <c r="L89" t="s">
         <v>21</v>
       </c>
-      <c r="N59" t="s">
+      <c r="N89" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A60" s="4" t="s">
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A90" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B60" s="4"/>
-      <c r="C60" t="s">
+      <c r="B90" s="4"/>
+      <c r="C90" t="s">
         <v>43</v>
       </c>
-      <c r="J60" t="s">
+      <c r="J90" t="s">
         <v>112</v>
       </c>
-      <c r="K60" s="11">
+      <c r="K90" s="11">
         <f>0.27/100</f>
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="L60" t="s">
+      <c r="L90" t="s">
         <v>22</v>
       </c>
-      <c r="N60" t="s">
+      <c r="N90" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A61" s="4" t="s">
+    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A91" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B61" s="4"/>
-      <c r="C61" t="s">
+      <c r="B91" s="4"/>
+      <c r="C91" t="s">
         <v>43</v>
       </c>
-      <c r="J61" t="s">
+      <c r="J91" t="s">
         <v>113</v>
       </c>
-      <c r="K61" s="11">
+      <c r="K91" s="11">
         <f>2.34/100</f>
         <v>2.3399999999999997E-2</v>
       </c>
-      <c r="L61" t="s">
+      <c r="L91" t="s">
         <v>23</v>
       </c>
-      <c r="N61" t="s">
+      <c r="N91" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A62" s="4"/>
-      <c r="B62" s="4"/>
-      <c r="K62" s="11"/>
-    </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A63" s="2" t="s">
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92" s="4"/>
+      <c r="B92" s="4"/>
+      <c r="K92" s="11"/>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B63" s="2"/>
-      <c r="C63" s="2"/>
-      <c r="D63" s="2"/>
-      <c r="E63" s="2"/>
-      <c r="F63" s="2"/>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2"/>
-      <c r="K63" s="2"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-      <c r="N63" s="2"/>
-    </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A64" s="4"/>
-      <c r="B64" s="4"/>
-      <c r="C64" s="4"/>
-      <c r="D64" s="4"/>
-      <c r="E64" s="4"/>
-      <c r="F64" s="4"/>
-      <c r="G64" s="4"/>
-      <c r="H64" s="4"/>
-      <c r="I64" s="4"/>
-      <c r="J64" s="4"/>
-      <c r="K64" s="4"/>
-      <c r="L64" s="4"/>
-      <c r="M64" s="4"/>
-      <c r="N64" s="4"/>
-    </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A65" s="4"/>
-      <c r="B65" s="4"/>
-      <c r="J65" t="s">
+      <c r="B93" s="2"/>
+      <c r="C93" s="2"/>
+      <c r="D93" s="2"/>
+      <c r="E93" s="2"/>
+      <c r="F93" s="2"/>
+      <c r="G93" s="2"/>
+      <c r="H93" s="2"/>
+      <c r="I93" s="2"/>
+      <c r="J93" s="2"/>
+      <c r="K93" s="2"/>
+      <c r="L93" s="2"/>
+      <c r="M93" s="2"/>
+      <c r="N93" s="2"/>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94" s="4"/>
+      <c r="B94" s="4"/>
+      <c r="C94" s="4"/>
+      <c r="D94" s="4"/>
+      <c r="E94" s="4"/>
+      <c r="F94" s="4"/>
+      <c r="G94" s="4"/>
+      <c r="H94" s="4"/>
+      <c r="I94" s="4"/>
+      <c r="J94" s="4"/>
+      <c r="K94" s="4"/>
+      <c r="L94" s="4"/>
+      <c r="M94" s="4"/>
+      <c r="N94" s="4"/>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95" s="4"/>
+      <c r="B95" s="4"/>
+      <c r="J95" t="s">
         <v>56</v>
       </c>
-      <c r="K65" s="11">
+      <c r="K95" s="11">
         <v>0.71750000000000003</v>
       </c>
-      <c r="L65" t="s">
+      <c r="L95" t="s">
         <v>57</v>
       </c>
-      <c r="N65" t="s">
+      <c r="N95" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A66" s="4"/>
-      <c r="B66" s="4"/>
-      <c r="J66" t="s">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" s="4"/>
+      <c r="B96" s="4"/>
+      <c r="J96" t="s">
         <v>58</v>
       </c>
-      <c r="K66" s="11">
+      <c r="K96" s="11">
         <v>1.9496</v>
       </c>
-      <c r="L66" t="s">
+      <c r="L96" t="s">
         <v>57</v>
       </c>
-      <c r="N66" t="s">
+      <c r="N96" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A67" s="4"/>
-      <c r="B67" s="4"/>
-      <c r="J67" t="s">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97" s="4"/>
+      <c r="B97" s="4"/>
+      <c r="J97" t="s">
         <v>96</v>
       </c>
-      <c r="K67" s="13">
+      <c r="K97" s="13">
         <f>50*(1/3.6)</f>
         <v>13.888888888888889</v>
       </c>
-      <c r="L67" t="s">
+      <c r="L97" t="s">
         <v>92</v>
       </c>
-      <c r="M67" t="s">
+      <c r="M97" t="s">
         <v>91</v>
       </c>
-      <c r="N67" t="s">
+      <c r="N97" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A69" s="2" t="s">
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B69" s="2"/>
-      <c r="C69" s="2"/>
-      <c r="D69" s="2"/>
-      <c r="E69" s="2"/>
-      <c r="F69" s="2"/>
-      <c r="G69" s="2"/>
-      <c r="H69" s="2"/>
-      <c r="I69" s="2"/>
-      <c r="J69" s="2"/>
-      <c r="K69" s="2"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
-      <c r="N69" s="2"/>
-    </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A70" s="14" t="s">
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+      <c r="H99" s="2"/>
+      <c r="I99" s="2"/>
+      <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
+      <c r="L99" s="2"/>
+      <c r="M99" s="2"/>
+      <c r="N99" s="2"/>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100" s="14" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J71" t="s">
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J101" t="s">
         <v>30</v>
       </c>
-      <c r="K71" s="4">
+      <c r="K101" s="4">
         <v>90</v>
       </c>
-      <c r="L71" s="4" t="s">
+      <c r="L101" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M71" s="4" t="s">
+      <c r="M101" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="N71" t="s">
+      <c r="N101" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J72" t="s">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J102" t="s">
         <v>36</v>
       </c>
-      <c r="K72" s="4">
+      <c r="K102" s="4">
         <v>0.22</v>
       </c>
-      <c r="L72" s="4" t="s">
+      <c r="L102" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="M72" s="7"/>
-      <c r="N72" t="s">
+      <c r="M102" s="7"/>
+      <c r="N102" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J73" t="s">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J103" t="s">
         <v>34</v>
       </c>
-      <c r="K73" s="4">
+      <c r="K103" s="4">
         <v>3.4</v>
       </c>
-      <c r="L73" s="4" t="s">
+      <c r="L103" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="M73" s="7"/>
-      <c r="N73" t="s">
+      <c r="M103" s="7"/>
+      <c r="N103" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J74" t="s">
+    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J104" t="s">
         <v>35</v>
       </c>
-      <c r="K74" s="4">
+      <c r="K104" s="4">
         <v>5</v>
       </c>
-      <c r="L74" s="4" t="s">
+      <c r="L104" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="M74" s="7"/>
-      <c r="N74" t="s">
+      <c r="M104" s="7"/>
+      <c r="N104" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A75" s="14" t="s">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A105" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="K75" s="4"/>
-      <c r="L75" s="4"/>
-      <c r="M75" s="7"/>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I76" t="s">
+      <c r="K105" s="4"/>
+      <c r="L105" s="4"/>
+      <c r="M105" s="7"/>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I106" t="s">
         <v>78</v>
       </c>
-      <c r="J76" t="s">
+      <c r="J106" t="s">
         <v>80</v>
       </c>
-      <c r="K76" s="4">
+      <c r="K106" s="4">
         <v>0.61</v>
       </c>
-      <c r="L76" s="4" t="s">
+      <c r="L106" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M76" s="4" t="s">
+      <c r="M106" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N76" t="s">
+      <c r="N106" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I77" t="s">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I107" t="s">
         <v>79</v>
       </c>
-      <c r="J77" t="s">
+      <c r="J107" t="s">
         <v>80</v>
       </c>
-      <c r="K77" s="4">
+      <c r="K107" s="4">
         <v>0.99</v>
       </c>
-      <c r="L77" s="4" t="s">
+      <c r="L107" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M77" s="7"/>
-      <c r="N77" t="s">
+      <c r="M107" s="7"/>
+      <c r="N107" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A78" s="14" t="s">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A108" s="14" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="79" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C79" t="s">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C109" t="s">
         <v>114</v>
       </c>
-      <c r="J79" t="s">
+      <c r="J109" t="s">
         <v>25</v>
       </c>
-      <c r="K79">
+      <c r="K109">
         <v>63</v>
       </c>
-      <c r="L79" t="s">
+      <c r="L109" t="s">
         <v>54</v>
       </c>
-      <c r="N79" t="s">
+      <c r="N109" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="80" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C80" t="s">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C110" t="s">
         <v>115</v>
       </c>
-      <c r="J80" t="s">
+      <c r="J110" t="s">
         <v>25</v>
       </c>
-      <c r="K80">
+      <c r="K110">
         <v>59</v>
       </c>
-      <c r="L80" t="s">
+      <c r="L110" t="s">
         <v>54</v>
       </c>
-      <c r="N80" t="s">
+      <c r="N110" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C81" t="s">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C111" t="s">
         <v>116</v>
       </c>
-      <c r="J81" t="s">
+      <c r="J111" t="s">
         <v>25</v>
       </c>
-      <c r="K81" s="6">
-        <f>K80</f>
+      <c r="K111" s="6">
+        <f>K110</f>
         <v>59</v>
       </c>
-      <c r="L81" t="s">
+      <c r="L111" t="s">
         <v>54</v>
       </c>
-      <c r="M81" s="7" t="s">
+      <c r="M111" s="7" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A82" s="4" t="s">
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B112" t="s">
+        <v>123</v>
+      </c>
+      <c r="C112" t="s">
+        <v>128</v>
+      </c>
+      <c r="J112" t="s">
+        <v>25</v>
+      </c>
+      <c r="K112" s="4">
+        <v>65</v>
+      </c>
+      <c r="L112" t="s">
+        <v>54</v>
+      </c>
+      <c r="M112" s="7"/>
+      <c r="N112" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B113" t="s">
+        <v>127</v>
+      </c>
+      <c r="C113" t="s">
+        <v>128</v>
+      </c>
+      <c r="J113" t="s">
+        <v>25</v>
+      </c>
+      <c r="K113" s="4">
+        <v>65</v>
+      </c>
+      <c r="L113" t="s">
+        <v>54</v>
+      </c>
+      <c r="M113" s="7"/>
+      <c r="N113" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B114" t="s">
+        <v>126</v>
+      </c>
+      <c r="C114" t="s">
+        <v>128</v>
+      </c>
+      <c r="J114" t="s">
+        <v>25</v>
+      </c>
+      <c r="K114" s="4">
+        <v>65</v>
+      </c>
+      <c r="L114" t="s">
+        <v>54</v>
+      </c>
+      <c r="M114" s="7"/>
+      <c r="N114" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B115" t="s">
+        <v>129</v>
+      </c>
+      <c r="C115" t="s">
+        <v>128</v>
+      </c>
+      <c r="J115" t="s">
+        <v>25</v>
+      </c>
+      <c r="K115" s="6">
+        <f>K110</f>
+        <v>59</v>
+      </c>
+      <c r="L115" t="s">
+        <v>54</v>
+      </c>
+      <c r="M115" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A116" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B82" s="4"/>
-      <c r="C82" t="s">
+      <c r="B116" s="4"/>
+      <c r="C116" t="s">
         <v>43</v>
       </c>
-      <c r="J82" t="s">
+      <c r="J116" t="s">
         <v>25</v>
       </c>
-      <c r="K82">
+      <c r="K116">
         <v>56</v>
       </c>
-      <c r="L82" t="s">
+      <c r="L116" t="s">
         <v>54</v>
       </c>
-      <c r="M82" t="s">
+      <c r="M116" t="s">
         <v>62</v>
       </c>
-      <c r="N82" t="s">
+      <c r="N116" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C83" t="s">
+    <row r="117" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C117" t="s">
         <v>31</v>
       </c>
-      <c r="J83" t="s">
+      <c r="J117" t="s">
         <v>25</v>
       </c>
-      <c r="K83" s="4">
+      <c r="K117" s="4">
         <v>65</v>
       </c>
-      <c r="L83" t="s">
+      <c r="L117" t="s">
         <v>54</v>
       </c>
-      <c r="M83" t="s">
+      <c r="M117" t="s">
         <v>61</v>
       </c>
-      <c r="N83" t="s">
+      <c r="N117" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A84" s="14" t="s">
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A118" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="K84" s="4"/>
-      <c r="L84" s="4"/>
-      <c r="M84" s="7"/>
-    </row>
-    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H85" t="s">
+      <c r="K118" s="4"/>
+      <c r="L118" s="4"/>
+      <c r="M118" s="7"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H119" t="s">
         <v>84</v>
       </c>
-      <c r="J85" t="s">
+      <c r="J119" t="s">
         <v>81</v>
       </c>
-      <c r="K85" s="13">
+      <c r="K119" s="13">
         <f>1041/(50+3+1041)*100</f>
         <v>95.155393053016454</v>
       </c>
-      <c r="L85" s="4" t="s">
+      <c r="L119" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M85" s="4" t="s">
+      <c r="M119" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="N85" t="s">
+      <c r="N119" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H86" t="s">
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H120" t="s">
         <v>79</v>
       </c>
-      <c r="J86" t="s">
+      <c r="J120" t="s">
         <v>81</v>
       </c>
-      <c r="K86" s="12">
+      <c r="K120" s="12">
         <f>50/(50+3+1041)*100</f>
         <v>4.5703839122486292</v>
       </c>
-      <c r="L86" s="4" t="s">
+      <c r="L120" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M86" s="4"/>
-      <c r="N86" t="s">
+      <c r="M120" s="4"/>
+      <c r="N120" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="87" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H87" t="s">
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H121" t="s">
         <v>78</v>
       </c>
-      <c r="J87" t="s">
+      <c r="J121" t="s">
         <v>81</v>
       </c>
-      <c r="K87" s="12">
+      <c r="K121" s="12">
         <f>3/(50+3+1041)*100</f>
         <v>0.27422303473491771</v>
       </c>
-      <c r="L87" s="4" t="s">
+      <c r="L121" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M87" s="4"/>
-      <c r="N87" t="s">
+      <c r="M121" s="4"/>
+      <c r="N121" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="88" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A88" s="14" t="s">
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A122" s="14" t="s">
         <v>94</v>
       </c>
-      <c r="K88" s="4"/>
-      <c r="L88" s="4"/>
-      <c r="M88" s="4"/>
-    </row>
-    <row r="89" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A89" s="15"/>
-      <c r="B89" s="3"/>
-      <c r="C89" s="3"/>
-      <c r="D89" s="3"/>
-      <c r="E89" s="3"/>
-      <c r="F89" s="3"/>
-      <c r="G89" s="3"/>
-      <c r="H89" s="3"/>
-      <c r="I89" s="3"/>
-      <c r="J89" s="3" t="s">
+      <c r="K122" s="4"/>
+      <c r="L122" s="4"/>
+      <c r="M122" s="4"/>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A123" s="15"/>
+      <c r="B123" s="3"/>
+      <c r="C123" s="3"/>
+      <c r="D123" s="3"/>
+      <c r="E123" s="3"/>
+      <c r="F123" s="3"/>
+      <c r="G123" s="3"/>
+      <c r="H123" s="3"/>
+      <c r="I123" s="3"/>
+      <c r="J123" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="K89" s="3">
+      <c r="K123" s="3">
         <v>0</v>
       </c>
-      <c r="L89" s="3" t="s">
+      <c r="L123" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="M89" s="3" t="s">
+      <c r="M123" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A90" s="15"/>
-      <c r="B90" s="3"/>
-      <c r="C90" s="3"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="3"/>
-      <c r="F90" s="3"/>
-      <c r="G90" s="3"/>
-      <c r="H90" s="3"/>
-      <c r="I90" s="3"/>
-      <c r="J90" s="3" t="s">
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A124" s="15"/>
+      <c r="B124" s="3"/>
+      <c r="C124" s="3"/>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3"/>
+      <c r="F124" s="3"/>
+      <c r="G124" s="3"/>
+      <c r="H124" s="3"/>
+      <c r="I124" s="3"/>
+      <c r="J124" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="K90" s="3">
+      <c r="K124" s="3">
         <v>0</v>
       </c>
-      <c r="L90" s="3" t="s">
+      <c r="L124" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="M90" s="3" t="s">
+      <c r="M124" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H91" t="s">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H125" t="s">
         <v>84</v>
       </c>
-      <c r="J91" t="s">
+      <c r="J125" t="s">
         <v>82</v>
       </c>
-      <c r="K91" s="4">
+      <c r="K125" s="4">
         <v>0.5</v>
       </c>
-      <c r="L91" s="4" t="s">
+      <c r="L125" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="M91" s="7"/>
-      <c r="N91" t="s">
+      <c r="M125" s="7"/>
+      <c r="N125" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H92" t="s">
+    <row r="126" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H126" t="s">
         <v>84</v>
       </c>
-      <c r="I92" t="s">
+      <c r="I126" t="s">
         <v>78</v>
       </c>
-      <c r="J92" t="s">
+      <c r="J126" t="s">
         <v>83</v>
       </c>
-      <c r="K92" s="10">
+      <c r="K126" s="10">
         <f>0.9 * (1/3.6) / 0.6 / 0.718</f>
         <v>0.5803156917363046</v>
       </c>
-      <c r="L92" s="4" t="s">
+      <c r="L126" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="M92" s="4" t="s">
+      <c r="M126" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="N92" t="s">
+      <c r="N126" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A93" s="14" t="s">
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A127" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="K93" s="4"/>
-      <c r="L93" s="4"/>
-      <c r="M93" s="7"/>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J94" t="s">
+      <c r="K127" s="4"/>
+      <c r="L127" s="4"/>
+      <c r="M127" s="7"/>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J128" t="s">
         <v>49</v>
       </c>
-      <c r="K94" s="11">
+      <c r="K128" s="11">
         <f>238/0.74/1000</f>
         <v>0.32162162162162161</v>
       </c>
-      <c r="L94" s="4" t="s">
+      <c r="L128" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M94" s="7"/>
-      <c r="N94" t="s">
+      <c r="M128" s="7"/>
+      <c r="N128" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J95" t="s">
+    <row r="129" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="J129" t="s">
         <v>59</v>
       </c>
-      <c r="K95" s="12">
+      <c r="K129" s="12">
         <v>1.5</v>
       </c>
-      <c r="L95" s="4" t="s">
+      <c r="L129" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M95" s="7"/>
-      <c r="N95" t="s">
+      <c r="M129" s="7"/>
+      <c r="N129" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J96" t="s">
+    <row r="130" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="J130" t="s">
         <v>50</v>
       </c>
-      <c r="K96" s="13">
+      <c r="K130" s="13">
         <v>60</v>
       </c>
-      <c r="L96" s="4" t="s">
+      <c r="L130" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="M96" s="7"/>
-      <c r="N96" t="s">
+      <c r="M130" s="7"/>
+      <c r="N130" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="98" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F98" t="s">
+    <row r="132" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F132" t="s">
         <v>65</v>
       </c>
-      <c r="G98" t="s">
+      <c r="G132" t="s">
         <v>67</v>
       </c>
-      <c r="J98" t="s">
+      <c r="J132" t="s">
         <v>66</v>
       </c>
-      <c r="K98">
+      <c r="K132">
         <v>2.75</v>
       </c>
-      <c r="L98" t="s">
+      <c r="L132" t="s">
         <v>51</v>
       </c>
-      <c r="M98" t="s">
+      <c r="M132" t="s">
         <v>121</v>
       </c>
-      <c r="N98" t="s">
+      <c r="N132" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="99" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F99" t="s">
+    <row r="133" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F133" t="s">
         <v>65</v>
       </c>
-      <c r="G99" t="s">
+      <c r="G133" t="s">
         <v>68</v>
       </c>
-      <c r="J99" t="s">
+      <c r="J133" t="s">
         <v>66</v>
       </c>
-      <c r="K99">
+      <c r="K133">
         <v>0</v>
       </c>
-      <c r="L99" t="s">
+      <c r="L133" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="100" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F100" t="s">
+    <row r="134" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F134" t="s">
         <v>65</v>
       </c>
-      <c r="G100" t="s">
+      <c r="G134" t="s">
         <v>69</v>
       </c>
-      <c r="J100" t="s">
+      <c r="J134" t="s">
         <v>66</v>
       </c>
-      <c r="K100">
+      <c r="K134">
         <v>0</v>
       </c>
-      <c r="L100" t="s">
+      <c r="L134" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="101" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F101" t="s">
+    <row r="135" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F135" t="s">
         <v>65</v>
       </c>
-      <c r="G101" t="s">
+      <c r="G135" t="s">
         <v>70</v>
       </c>
-      <c r="J101" t="s">
+      <c r="J135" t="s">
         <v>66</v>
       </c>
-      <c r="K101">
+      <c r="K135">
         <v>0</v>
       </c>
-      <c r="L101" t="s">
+      <c r="L135" t="s">
         <v>71</v>
       </c>
-      <c r="N101" t="s">
+      <c r="N135" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="103" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F103" t="s">
+    <row r="137" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F137" t="s">
         <v>72</v>
       </c>
-      <c r="G103" t="s">
+      <c r="G137" t="s">
         <v>72</v>
       </c>
-      <c r="J103" t="s">
+      <c r="J137" t="s">
         <v>66</v>
       </c>
-      <c r="K103">
+      <c r="K137">
         <v>0</v>
       </c>
-      <c r="L103" t="s">
+      <c r="L137" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="104" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F104" t="s">
+    <row r="138" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F138" t="s">
         <v>73</v>
       </c>
-      <c r="G104" t="s">
+      <c r="G138" t="s">
         <v>73</v>
       </c>
-      <c r="J104" t="s">
+      <c r="J138" t="s">
         <v>66</v>
       </c>
-      <c r="K104">
+      <c r="K138">
         <v>0</v>
       </c>
-      <c r="L104" t="s">
+      <c r="L138" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Function for 'incineration' + data (draft)
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -15,7 +15,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="references" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="468" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="145">
   <si>
     <t>parameter</t>
   </si>
@@ -418,6 +418,48 @@
   </si>
   <si>
     <t>Food waste, grocery stores</t>
+  </si>
+  <si>
+    <t>INCINERATION</t>
+  </si>
+  <si>
+    <t>2.5 kWh/kg wet weight</t>
+  </si>
+  <si>
+    <t>kWh/kg VS</t>
+  </si>
+  <si>
+    <t>incineration_efficiency</t>
+  </si>
+  <si>
+    <t>incineration_heating_value</t>
+  </si>
+  <si>
+    <t>incineration_emissions</t>
+  </si>
+  <si>
+    <t>kg/kWh</t>
+  </si>
+  <si>
+    <t>N2O</t>
+  </si>
+  <si>
+    <t>NOx</t>
+  </si>
+  <si>
+    <t>NH3</t>
+  </si>
+  <si>
+    <t>Miljöfaktaboken 2011, Tabell 17</t>
+  </si>
+  <si>
+    <t>Miljöfaktaboken 2011, s. 43</t>
+  </si>
+  <si>
+    <t>VS</t>
+  </si>
+  <si>
+    <t>CH4bio</t>
   </si>
 </sst>
 </file>
@@ -490,7 +532,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -500,6 +542,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -516,7 +570,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -535,6 +589,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -816,7 +874,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O138"/>
+  <dimension ref="A1:O153"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -826,6 +884,7 @@
     <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="9" width="21.28515625" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="32.42578125" customWidth="1"/>
     <col min="14" max="14" width="20.7109375" customWidth="1"/>
@@ -2330,22 +2389,22 @@
       </c>
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A99" s="2" t="s">
+      <c r="A99" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B99" s="2"/>
-      <c r="C99" s="2"/>
-      <c r="D99" s="2"/>
-      <c r="E99" s="2"/>
-      <c r="F99" s="2"/>
-      <c r="G99" s="2"/>
-      <c r="H99" s="2"/>
-      <c r="I99" s="2"/>
-      <c r="J99" s="2"/>
-      <c r="K99" s="2"/>
-      <c r="L99" s="2"/>
-      <c r="M99" s="2"/>
-      <c r="N99" s="2"/>
+      <c r="B99" s="19"/>
+      <c r="C99" s="19"/>
+      <c r="D99" s="19"/>
+      <c r="E99" s="19"/>
+      <c r="F99" s="19"/>
+      <c r="G99" s="19"/>
+      <c r="H99" s="19"/>
+      <c r="I99" s="19"/>
+      <c r="J99" s="19"/>
+      <c r="K99" s="19"/>
+      <c r="L99" s="19"/>
+      <c r="M99" s="19"/>
+      <c r="N99" s="19"/>
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="14" t="s">
@@ -2832,7 +2891,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="129" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J129" t="s">
         <v>59</v>
       </c>
@@ -2847,7 +2906,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="130" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J130" t="s">
         <v>50</v>
       </c>
@@ -2862,52 +2921,47 @@
         <v>53</v>
       </c>
     </row>
-    <row r="132" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F132" t="s">
-        <v>65</v>
-      </c>
-      <c r="G132" t="s">
-        <v>67</v>
-      </c>
-      <c r="J132" t="s">
+    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J132" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="K132">
-        <v>2.75</v>
-      </c>
-      <c r="L132" t="s">
-        <v>51</v>
-      </c>
-      <c r="M132" t="s">
-        <v>121</v>
-      </c>
-      <c r="N132" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="133" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="K132" s="3">
+        <v>0</v>
+      </c>
+      <c r="L132" s="3"/>
+      <c r="M132" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F133" t="s">
         <v>65</v>
       </c>
       <c r="G133" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="J133" t="s">
         <v>66</v>
       </c>
       <c r="K133">
-        <v>0</v>
+        <v>2.75</v>
       </c>
       <c r="L133" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="134" spans="6:14" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+      <c r="M133" t="s">
+        <v>121</v>
+      </c>
+      <c r="N133" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F134" t="s">
         <v>65</v>
       </c>
       <c r="G134" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J134" t="s">
         <v>66</v>
@@ -2916,15 +2970,15 @@
         <v>0</v>
       </c>
       <c r="L134" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="135" spans="6:14" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F135" t="s">
         <v>65</v>
       </c>
       <c r="G135" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J135" t="s">
         <v>66</v>
@@ -2933,35 +2987,35 @@
         <v>0</v>
       </c>
       <c r="L135" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F136" t="s">
+        <v>65</v>
+      </c>
+      <c r="G136" t="s">
+        <v>70</v>
+      </c>
+      <c r="J136" t="s">
+        <v>66</v>
+      </c>
+      <c r="K136">
+        <v>0</v>
+      </c>
+      <c r="L136" t="s">
         <v>71</v>
       </c>
-      <c r="N135" t="s">
+      <c r="N136" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="137" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F137" t="s">
+    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F138" t="s">
         <v>72</v>
       </c>
-      <c r="G137" t="s">
+      <c r="G138" t="s">
         <v>72</v>
-      </c>
-      <c r="J137" t="s">
-        <v>66</v>
-      </c>
-      <c r="K137">
-        <v>0</v>
-      </c>
-      <c r="L137" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="138" spans="6:14" x14ac:dyDescent="0.25">
-      <c r="F138" t="s">
-        <v>73</v>
-      </c>
-      <c r="G138" t="s">
-        <v>73</v>
       </c>
       <c r="J138" t="s">
         <v>66</v>
@@ -2970,7 +3024,205 @@
         <v>0</v>
       </c>
       <c r="L138" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F139" t="s">
+        <v>73</v>
+      </c>
+      <c r="G139" t="s">
+        <v>73</v>
+      </c>
+      <c r="J139" t="s">
+        <v>66</v>
+      </c>
+      <c r="K139">
+        <v>0</v>
+      </c>
+      <c r="L139" t="s">
         <v>75</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A141" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="B141" s="18"/>
+      <c r="C141" s="18"/>
+      <c r="D141" s="18"/>
+      <c r="E141" s="18"/>
+      <c r="F141" s="18"/>
+      <c r="G141" s="18"/>
+      <c r="H141" s="18"/>
+      <c r="I141" s="18"/>
+      <c r="J141" s="18"/>
+      <c r="K141" s="18"/>
+      <c r="L141" s="18"/>
+      <c r="M141" s="18"/>
+      <c r="N141" s="18"/>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J143" t="s">
+        <v>135</v>
+      </c>
+      <c r="K143" s="20">
+        <f>2.5/0.33/0.85</f>
+        <v>8.9126559714795004</v>
+      </c>
+      <c r="L143" t="s">
+        <v>133</v>
+      </c>
+      <c r="M143" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="145" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="J145" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="K145" s="3">
+        <v>0</v>
+      </c>
+      <c r="L145" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="M145" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="146" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="H146" t="s">
+        <v>78</v>
+      </c>
+      <c r="J146" t="s">
+        <v>134</v>
+      </c>
+      <c r="K146" s="8">
+        <f>0.94*0.184</f>
+        <v>0.17295999999999997</v>
+      </c>
+      <c r="L146" t="s">
+        <v>97</v>
+      </c>
+      <c r="N146" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="147" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="H147" t="s">
+        <v>79</v>
+      </c>
+      <c r="J147" t="s">
+        <v>134</v>
+      </c>
+      <c r="K147" s="8">
+        <f>0.94*0.816</f>
+        <v>0.76703999999999994</v>
+      </c>
+      <c r="L147" t="s">
+        <v>97</v>
+      </c>
+      <c r="N147" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="149" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="J149" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="K149" s="3">
+        <v>0</v>
+      </c>
+      <c r="L149" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="M149" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="150" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F150" t="s">
+        <v>143</v>
+      </c>
+      <c r="G150" t="s">
+        <v>144</v>
+      </c>
+      <c r="J150" t="s">
+        <v>136</v>
+      </c>
+      <c r="K150" s="21">
+        <f>(0.00234-0.000502)/1000/(1/3.6)</f>
+        <v>6.6168000000000008E-6</v>
+      </c>
+      <c r="L150" t="s">
+        <v>137</v>
+      </c>
+      <c r="N150" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="151" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F151" t="s">
+        <v>65</v>
+      </c>
+      <c r="G151" t="s">
+        <v>138</v>
+      </c>
+      <c r="J151" t="s">
+        <v>136</v>
+      </c>
+      <c r="K151" s="21">
+        <f>(0.000364 -0.00000236)/1000/(1/3.6)</f>
+        <v>1.3019039999999999E-6</v>
+      </c>
+      <c r="L151" t="s">
+        <v>137</v>
+      </c>
+      <c r="N151" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="152" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F152" t="s">
+        <v>65</v>
+      </c>
+      <c r="G152" t="s">
+        <v>139</v>
+      </c>
+      <c r="J152" t="s">
+        <v>136</v>
+      </c>
+      <c r="K152" s="21">
+        <f>(0.0376-0.00437)/1000/(1/3.6)</f>
+        <v>1.1962800000000001E-4</v>
+      </c>
+      <c r="L152" t="s">
+        <v>137</v>
+      </c>
+      <c r="N152" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="153" spans="6:14" x14ac:dyDescent="0.25">
+      <c r="F153" t="s">
+        <v>65</v>
+      </c>
+      <c r="G153" t="s">
+        <v>140</v>
+      </c>
+      <c r="J153" t="s">
+        <v>136</v>
+      </c>
+      <c r="K153" s="21">
+        <f>(0.00171-0.00000236)/1000/(1/3.6)</f>
+        <v>6.1475039999999993E-6</v>
+      </c>
+      <c r="L153" t="s">
+        <v>137</v>
+      </c>
+      <c r="N153" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added 'landfill' treatment function + data
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="508" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="156">
   <si>
     <t>parameter</t>
   </si>
@@ -460,15 +460,50 @@
   </si>
   <si>
     <t>CH4bio</t>
+  </si>
+  <si>
+    <t>LANDFILL</t>
+  </si>
+  <si>
+    <t>kg/kg VS</t>
+  </si>
+  <si>
+    <t>landfill_emissions</t>
+  </si>
+  <si>
+    <t>NO3</t>
+  </si>
+  <si>
+    <t>PO4</t>
+  </si>
+  <si>
+    <t>Ecoinvent. treatment of municipal solid waste, sanitary landfill (SE).https://ecoquery.ecoinvent.org/3.11/cutoff/dataset/92891/documentation</t>
+  </si>
+  <si>
+    <t>Emissions from ecoinvent</t>
+  </si>
+  <si>
+    <t>landfill of municipal solid waste</t>
+  </si>
+  <si>
+    <t>assuming 0.43 kg VS/kg</t>
+  </si>
+  <si>
+    <t>0.54 kgDM/kg (ecoinvent) * 0.8 kgVS/kgDM</t>
+  </si>
+  <si>
+    <t>NH4</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
+    <numFmt numFmtId="170" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -532,7 +567,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -557,6 +592,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -570,7 +611,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -593,6 +634,11 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="165" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,7 +920,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O153"/>
+  <dimension ref="A1:O165"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -884,7 +930,7 @@
     <col min="5" max="5" width="21.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="9" width="21.28515625" customWidth="1"/>
     <col min="10" max="10" width="25.7109375" customWidth="1"/>
-    <col min="11" max="11" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="32.42578125" customWidth="1"/>
     <col min="14" max="14" width="20.7109375" customWidth="1"/>
@@ -3077,7 +3123,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="145" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J145" s="3" t="s">
         <v>134</v>
       </c>
@@ -3091,7 +3137,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="146" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H146" t="s">
         <v>78</v>
       </c>
@@ -3109,7 +3155,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="147" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H147" t="s">
         <v>79</v>
       </c>
@@ -3127,7 +3173,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="149" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
       <c r="J149" s="3" t="s">
         <v>136</v>
       </c>
@@ -3141,7 +3187,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="150" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F150" t="s">
         <v>143</v>
       </c>
@@ -3162,7 +3208,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="151" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F151" t="s">
         <v>65</v>
       </c>
@@ -3183,7 +3229,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="152" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F152" t="s">
         <v>65</v>
       </c>
@@ -3204,7 +3250,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="153" spans="6:14" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="F153" t="s">
         <v>65</v>
       </c>
@@ -3223,6 +3269,194 @@
       </c>
       <c r="N153" t="s">
         <v>141</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A155" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="B155" s="23"/>
+      <c r="C155" s="23"/>
+      <c r="D155" s="23"/>
+      <c r="E155" s="23"/>
+      <c r="F155" s="23"/>
+      <c r="G155" s="23"/>
+      <c r="H155" s="23"/>
+      <c r="I155" s="23"/>
+      <c r="J155" s="23"/>
+      <c r="K155" s="23"/>
+      <c r="L155" s="23"/>
+      <c r="M155" s="23"/>
+      <c r="N155" s="23"/>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J157" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="K157" s="3">
+        <v>0</v>
+      </c>
+      <c r="L157" s="3" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F158" t="s">
+        <v>143</v>
+      </c>
+      <c r="G158" t="s">
+        <v>144</v>
+      </c>
+      <c r="J158" t="s">
+        <v>147</v>
+      </c>
+      <c r="K158" s="17">
+        <f>(0.00144+0.0129)/0.43</f>
+        <v>3.3348837209302325E-2</v>
+      </c>
+      <c r="L158" t="s">
+        <v>146</v>
+      </c>
+      <c r="M158" t="s">
+        <v>151</v>
+      </c>
+      <c r="N158" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F159" t="s">
+        <v>65</v>
+      </c>
+      <c r="G159" t="s">
+        <v>138</v>
+      </c>
+      <c r="J159" t="s">
+        <v>147</v>
+      </c>
+      <c r="K159" s="26">
+        <f>(0)/0.43</f>
+        <v>0</v>
+      </c>
+      <c r="L159" t="s">
+        <v>146</v>
+      </c>
+      <c r="M159" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F160" t="s">
+        <v>65</v>
+      </c>
+      <c r="G160" t="s">
+        <v>139</v>
+      </c>
+      <c r="J160" t="s">
+        <v>147</v>
+      </c>
+      <c r="K160" s="24">
+        <f>(0.00000208)/0.43</f>
+        <v>4.8372093023255818E-6</v>
+      </c>
+      <c r="L160" t="s">
+        <v>146</v>
+      </c>
+      <c r="M160" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="161" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F161" t="s">
+        <v>65</v>
+      </c>
+      <c r="G161" t="s">
+        <v>140</v>
+      </c>
+      <c r="J161" t="s">
+        <v>147</v>
+      </c>
+      <c r="K161" s="26">
+        <f t="shared" ref="K161:K165" si="2">(0)/0.43</f>
+        <v>0</v>
+      </c>
+      <c r="L161" t="s">
+        <v>146</v>
+      </c>
+      <c r="M161" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="162" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F162" t="s">
+        <v>65</v>
+      </c>
+      <c r="G162" t="s">
+        <v>155</v>
+      </c>
+      <c r="J162" t="s">
+        <v>147</v>
+      </c>
+      <c r="K162" s="8">
+        <f>(0.00152)/0.43</f>
+        <v>3.534883720930233E-3</v>
+      </c>
+      <c r="L162" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="163" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F163" t="s">
+        <v>65</v>
+      </c>
+      <c r="G163" t="s">
+        <v>148</v>
+      </c>
+      <c r="J163" t="s">
+        <v>147</v>
+      </c>
+      <c r="K163" s="25">
+        <f>(0.00016)/0.43</f>
+        <v>3.7209302325581399E-4</v>
+      </c>
+      <c r="L163" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="164" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F164" t="s">
+        <v>72</v>
+      </c>
+      <c r="G164" t="s">
+        <v>149</v>
+      </c>
+      <c r="J164" t="s">
+        <v>147</v>
+      </c>
+      <c r="K164" s="8">
+        <f>(0.000218)/0.43</f>
+        <v>5.0697674418604657E-4</v>
+      </c>
+      <c r="L164" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="165" spans="6:13" x14ac:dyDescent="0.25">
+      <c r="F165" t="s">
+        <v>73</v>
+      </c>
+      <c r="G165" t="s">
+        <v>73</v>
+      </c>
+      <c r="J165" t="s">
+        <v>147</v>
+      </c>
+      <c r="K165" s="17">
+        <f>(0.00343)/0.43</f>
+        <v>7.9767441860465107E-3</v>
+      </c>
+      <c r="L165" t="s">
+        <v>146</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Lost animals to waste treatment
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -15,7 +15,7 @@
     <sheet name="default" sheetId="1" r:id="rId1"/>
     <sheet name="references" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913" iterateDelta="1E-4"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="156">
   <si>
     <t>parameter</t>
   </si>
@@ -336,9 +336,6 @@
     <t>animal carcasses</t>
   </si>
   <si>
-    <t>slaughterhouse waste</t>
-  </si>
-  <si>
     <t>f_feedstock</t>
   </si>
   <si>
@@ -493,6 +490,9 @@
   </si>
   <si>
     <t>NH4</t>
+  </si>
+  <si>
+    <t>Live weight of animals lost before slughter</t>
   </si>
 </sst>
 </file>
@@ -502,8 +502,8 @@
   <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="168" formatCode="0.000000"/>
-    <numFmt numFmtId="170" formatCode="0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -636,8 +636,8 @@
     <xf numFmtId="11" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -920,7 +920,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:O165"/>
+  <dimension ref="A1:O172"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.42578125" customWidth="1"/>
@@ -938,10 +938,10 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>105</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>101</v>
@@ -950,7 +950,7 @@
         <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>63</v>
@@ -1014,7 +1014,7 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
@@ -1037,7 +1037,7 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E8" t="s">
         <v>9</v>
@@ -1054,7 +1054,7 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" t="s">
         <v>10</v>
@@ -1071,7 +1071,7 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
@@ -1088,7 +1088,7 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E12" t="s">
         <v>8</v>
@@ -1111,7 +1111,7 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E13" t="s">
         <v>9</v>
@@ -1128,7 +1128,7 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E14" t="s">
         <v>10</v>
@@ -1145,7 +1145,7 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
@@ -1162,7 +1162,7 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E17" t="s">
         <v>8</v>
@@ -1185,7 +1185,7 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E18" t="s">
         <v>9</v>
@@ -1202,7 +1202,7 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E19" t="s">
         <v>10</v>
@@ -1219,7 +1219,7 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E20" t="s">
         <v>11</v>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="D22" s="7"/>
       <c r="E22" s="7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -1255,252 +1255,260 @@
       <c r="L22" s="7" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C23" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7" t="s">
+      <c r="M22" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>31</v>
+      </c>
+      <c r="E24" t="s">
         <v>8</v>
       </c>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="7" t="s">
+      <c r="J24" t="s">
         <v>5</v>
       </c>
-      <c r="K23" s="7">
+      <c r="K24">
         <v>100</v>
       </c>
-      <c r="L23" s="7" t="s">
+      <c r="L24" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C25" t="s">
-        <v>31</v>
-      </c>
-      <c r="E25" t="s">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C26" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J25" t="s">
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="K25">
+      <c r="K26" s="7">
         <v>100</v>
       </c>
-      <c r="L25" t="s">
+      <c r="L26" s="7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C27" t="s">
-        <v>128</v>
-      </c>
-      <c r="E27" t="s">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="5"/>
+      <c r="C28" s="5"/>
+      <c r="D28" s="5"/>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5"/>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+      <c r="N28" s="5"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A30" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B30" s="4"/>
+      <c r="C30" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" t="s">
         <v>8</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J30" t="s">
         <v>5</v>
       </c>
-      <c r="K27">
+      <c r="K30">
         <v>100</v>
       </c>
-      <c r="L27" t="s">
+      <c r="L30" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B29" s="5"/>
-      <c r="C29" s="5"/>
-      <c r="D29" s="5"/>
-      <c r="E29" s="5"/>
-      <c r="F29" s="5"/>
-      <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-      <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
-      <c r="K29" s="5"/>
-      <c r="L29" s="5"/>
-      <c r="M29" s="5"/>
-      <c r="N29" s="5"/>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" s="4"/>
-      <c r="C31" t="s">
-        <v>43</v>
-      </c>
-      <c r="E31" t="s">
-        <v>8</v>
-      </c>
-      <c r="J31" t="s">
-        <v>5</v>
-      </c>
-      <c r="K31">
-        <v>100</v>
-      </c>
-      <c r="L31" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="2" t="s">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-      <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-    </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="J35" s="3" t="s">
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+      <c r="G32" s="2"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2"/>
+      <c r="J32" s="2"/>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="J34" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="K34" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="L34" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M34" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" t="s">
+        <v>113</v>
+      </c>
+      <c r="J36" t="s">
         <v>107</v>
       </c>
-      <c r="K35" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="L35" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="M35" s="3" t="s">
-        <v>7</v>
+      <c r="K36">
+        <v>0.33</v>
+      </c>
+      <c r="L36" t="s">
+        <v>19</v>
+      </c>
+      <c r="M36" t="s">
+        <v>26</v>
+      </c>
+      <c r="N36" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J37" t="s">
         <v>108</v>
       </c>
       <c r="K37">
-        <v>0.33</v>
+        <v>0.85</v>
       </c>
       <c r="L37" t="s">
-        <v>19</v>
-      </c>
-      <c r="M37" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="N37" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="4"/>
-      <c r="B38" s="4"/>
       <c r="C38" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J38" t="s">
         <v>109</v>
       </c>
       <c r="K38">
-        <v>0.85</v>
+        <v>0.46100000000000002</v>
       </c>
       <c r="L38" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="N38" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
       <c r="C39" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J39" t="s">
         <v>110</v>
       </c>
-      <c r="K39">
-        <v>0.46100000000000002</v>
+      <c r="K39" s="8">
+        <f>8.3/1000/0.33</f>
+        <v>2.515151515151515E-2</v>
       </c>
       <c r="L39" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="N39" t="s">
-        <v>33</v>
+        <v>44</v>
+      </c>
+      <c r="O39" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J40" t="s">
         <v>111</v>
       </c>
       <c r="K40" s="8">
-        <f>8.3/1000/0.33</f>
-        <v>2.515151515151515E-2</v>
+        <f>1/1000/0.33</f>
+        <v>3.0303030303030303E-3</v>
       </c>
       <c r="L40" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N40" t="s">
         <v>44</v>
-      </c>
-      <c r="O40" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J41" t="s">
         <v>112</v>
       </c>
       <c r="K41" s="8">
-        <f>1/1000/0.33</f>
-        <v>3.0303030303030303E-3</v>
+        <f>2.6/1000/0.33</f>
+        <v>7.8787878787878775E-3</v>
       </c>
       <c r="L41" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N41" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="4"/>
-      <c r="B42" s="4"/>
-      <c r="C42" t="s">
+    <row r="43" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A43" s="4"/>
+      <c r="B43" s="4"/>
+      <c r="C43" t="s">
         <v>114</v>
       </c>
-      <c r="J42" t="s">
-        <v>113</v>
-      </c>
-      <c r="K42" s="8">
-        <f>2.6/1000/0.33</f>
-        <v>7.8787878787878775E-3</v>
-      </c>
-      <c r="L42" t="s">
-        <v>23</v>
-      </c>
-      <c r="N42" t="s">
+      <c r="J43" t="s">
+        <v>107</v>
+      </c>
+      <c r="K43">
+        <v>0.15</v>
+      </c>
+      <c r="L43" t="s">
+        <v>19</v>
+      </c>
+      <c r="M43" t="s">
+        <v>129</v>
+      </c>
+      <c r="N43" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1508,56 +1516,54 @@
       <c r="A44" s="4"/>
       <c r="B44" s="4"/>
       <c r="C44" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J44" t="s">
         <v>108</v>
       </c>
-      <c r="K44">
-        <v>0.15</v>
+      <c r="K44" s="10">
+        <v>0.9</v>
       </c>
       <c r="L44" t="s">
-        <v>19</v>
-      </c>
-      <c r="M44" t="s">
-        <v>130</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="M44" s="7"/>
       <c r="N44" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="4"/>
-      <c r="B45" s="4"/>
       <c r="C45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J45" t="s">
         <v>109</v>
       </c>
-      <c r="K45" s="10">
-        <v>0.9</v>
+      <c r="K45" s="8">
+        <v>0.55000000000000004</v>
       </c>
       <c r="L45" t="s">
-        <v>20</v>
-      </c>
-      <c r="M45" s="7"/>
+        <v>29</v>
+      </c>
       <c r="N45" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+      <c r="B46" s="4"/>
       <c r="C46" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J46" t="s">
         <v>110</v>
       </c>
       <c r="K46" s="8">
-        <v>0.55000000000000004</v>
+        <f>3.8/1000/0.15</f>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L46" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="N46" t="s">
         <v>44</v>
@@ -1567,17 +1573,17 @@
       <c r="A47" s="4"/>
       <c r="B47" s="4"/>
       <c r="C47" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J47" t="s">
         <v>111</v>
       </c>
       <c r="K47" s="8">
-        <f>3.8/1000/0.15</f>
-        <v>2.5333333333333333E-2</v>
+        <f>0.5/1000/0.15</f>
+        <v>3.3333333333333335E-3</v>
       </c>
       <c r="L47" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N47" t="s">
         <v>44</v>
@@ -1587,396 +1593,384 @@
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J48" t="s">
         <v>112</v>
       </c>
       <c r="K48" s="8">
-        <f>0.5/1000/0.15</f>
-        <v>3.3333333333333335E-3</v>
+        <f>1.2/1000/0.15</f>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="L48" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="N48" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A49" s="4"/>
-      <c r="B49" s="4"/>
-      <c r="C49" t="s">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="4"/>
+      <c r="B50" s="4"/>
+      <c r="C50" t="s">
         <v>115</v>
       </c>
-      <c r="J49" t="s">
-        <v>113</v>
-      </c>
-      <c r="K49" s="8">
-        <f>1.2/1000/0.15</f>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="L49" t="s">
-        <v>23</v>
-      </c>
-      <c r="N49" t="s">
-        <v>44</v>
+      <c r="J50" t="s">
+        <v>107</v>
+      </c>
+      <c r="K50" s="6">
+        <f t="shared" ref="K50:K55" si="0">K43</f>
+        <v>0.15</v>
+      </c>
+      <c r="L50" t="s">
+        <v>19</v>
+      </c>
+      <c r="M50" s="4" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="4"/>
       <c r="B51" s="4"/>
       <c r="C51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J51" t="s">
         <v>108</v>
       </c>
-      <c r="K51" s="6">
-        <f t="shared" ref="K51:K56" si="0">K44</f>
-        <v>0.15</v>
+      <c r="K51" s="16">
+        <f t="shared" si="0"/>
+        <v>0.9</v>
       </c>
       <c r="L51" t="s">
-        <v>19</v>
-      </c>
-      <c r="M51" s="7" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="4"/>
       <c r="B52" s="4"/>
       <c r="C52" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J52" t="s">
         <v>109</v>
       </c>
-      <c r="K52" s="16">
+      <c r="K52" s="9">
         <f t="shared" si="0"/>
-        <v>0.9</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="L52" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="4"/>
       <c r="B53" s="4"/>
       <c r="C53" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J53" t="s">
         <v>110</v>
       </c>
       <c r="K53" s="9">
         <f t="shared" si="0"/>
-        <v>0.55000000000000004</v>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L53" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="4"/>
       <c r="B54" s="4"/>
       <c r="C54" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J54" t="s">
         <v>111</v>
       </c>
       <c r="K54" s="9">
         <f t="shared" si="0"/>
-        <v>2.5333333333333333E-2</v>
+        <v>3.3333333333333335E-3</v>
       </c>
       <c r="L54" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
       <c r="C55" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J55" t="s">
         <v>112</v>
       </c>
       <c r="K55" s="9">
         <f t="shared" si="0"/>
-        <v>3.3333333333333335E-3</v>
+        <v>8.0000000000000002E-3</v>
       </c>
       <c r="L55" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
-      <c r="B56" s="4"/>
-      <c r="C56" t="s">
-        <v>116</v>
-      </c>
-      <c r="J56" t="s">
-        <v>113</v>
-      </c>
-      <c r="K56" s="9">
-        <f t="shared" si="0"/>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="L56" t="s">
         <v>23</v>
       </c>
     </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C57" t="s">
+        <v>102</v>
+      </c>
+      <c r="J57" t="s">
+        <v>107</v>
+      </c>
+      <c r="K57" s="6">
+        <f>K64</f>
+        <v>0.16</v>
+      </c>
+      <c r="L57" t="s">
+        <v>19</v>
+      </c>
+      <c r="M57" t="s">
+        <v>121</v>
+      </c>
+      <c r="N57" t="s">
+        <v>44</v>
+      </c>
+    </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B58" t="s">
-        <v>123</v>
-      </c>
       <c r="C58" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="J58" t="s">
         <v>108</v>
       </c>
-      <c r="K58">
-        <v>0.16</v>
+      <c r="K58" s="6">
+        <f t="shared" ref="K58:K62" si="1">K65</f>
+        <v>0.9</v>
       </c>
       <c r="L58" t="s">
-        <v>19</v>
-      </c>
-      <c r="M58" t="s">
-        <v>122</v>
+        <v>20</v>
       </c>
       <c r="N58" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B59" t="s">
-        <v>123</v>
-      </c>
       <c r="C59" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="J59" t="s">
         <v>109</v>
       </c>
-      <c r="K59" s="17">
-        <v>0.9</v>
+      <c r="K59" s="6">
+        <f t="shared" si="1"/>
+        <v>0.434</v>
       </c>
       <c r="L59" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="N59" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B60" t="s">
-        <v>123</v>
-      </c>
       <c r="C60" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="J60" t="s">
         <v>110</v>
       </c>
-      <c r="K60">
-        <v>0.434</v>
+      <c r="K60" s="6">
+        <f t="shared" si="1"/>
+        <v>2.375E-2</v>
       </c>
       <c r="L60" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="N60" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B61" t="s">
-        <v>123</v>
-      </c>
       <c r="C61" t="s">
-        <v>128</v>
+        <v>102</v>
       </c>
       <c r="J61" t="s">
         <v>111</v>
       </c>
-      <c r="K61" s="8">
+      <c r="K61" s="6">
+        <f t="shared" si="1"/>
+        <v>2.5000000000000001E-3</v>
+      </c>
+      <c r="L61" t="s">
+        <v>22</v>
+      </c>
+      <c r="N61" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C62" t="s">
+        <v>102</v>
+      </c>
+      <c r="J62" t="s">
+        <v>112</v>
+      </c>
+      <c r="K62" s="6">
+        <f t="shared" si="1"/>
+        <v>4.3749999999999995E-3</v>
+      </c>
+      <c r="L62" t="s">
+        <v>23</v>
+      </c>
+      <c r="N62" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B64" t="s">
+        <v>122</v>
+      </c>
+      <c r="C64" t="s">
+        <v>127</v>
+      </c>
+      <c r="J64" t="s">
+        <v>107</v>
+      </c>
+      <c r="K64">
+        <v>0.16</v>
+      </c>
+      <c r="L64" t="s">
+        <v>19</v>
+      </c>
+      <c r="M64" t="s">
+        <v>121</v>
+      </c>
+      <c r="N64" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B65" t="s">
+        <v>122</v>
+      </c>
+      <c r="C65" t="s">
+        <v>127</v>
+      </c>
+      <c r="J65" t="s">
+        <v>108</v>
+      </c>
+      <c r="K65" s="17">
+        <v>0.9</v>
+      </c>
+      <c r="L65" t="s">
+        <v>20</v>
+      </c>
+      <c r="N65" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B66" t="s">
+        <v>122</v>
+      </c>
+      <c r="C66" t="s">
+        <v>127</v>
+      </c>
+      <c r="J66" t="s">
+        <v>109</v>
+      </c>
+      <c r="K66">
+        <v>0.434</v>
+      </c>
+      <c r="L66" t="s">
+        <v>29</v>
+      </c>
+      <c r="N66" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B67" t="s">
+        <v>122</v>
+      </c>
+      <c r="C67" t="s">
+        <v>127</v>
+      </c>
+      <c r="J67" t="s">
+        <v>110</v>
+      </c>
+      <c r="K67" s="8">
         <f>3.8/1000/0.16</f>
         <v>2.375E-2</v>
       </c>
-      <c r="L61" t="s">
+      <c r="L67" t="s">
         <v>21</v>
       </c>
-      <c r="N61" t="s">
+      <c r="N67" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B62" t="s">
-        <v>123</v>
-      </c>
-      <c r="C62" t="s">
-        <v>128</v>
-      </c>
-      <c r="J62" t="s">
-        <v>112</v>
-      </c>
-      <c r="K62" s="8">
+    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B68" t="s">
+        <v>122</v>
+      </c>
+      <c r="C68" t="s">
+        <v>127</v>
+      </c>
+      <c r="J68" t="s">
+        <v>111</v>
+      </c>
+      <c r="K68" s="8">
         <f>0.4/1000/0.16</f>
         <v>2.5000000000000001E-3</v>
       </c>
-      <c r="L62" t="s">
+      <c r="L68" t="s">
         <v>22</v>
       </c>
-      <c r="N62" t="s">
+      <c r="N68" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B63" t="s">
-        <v>123</v>
-      </c>
-      <c r="C63" t="s">
-        <v>128</v>
-      </c>
-      <c r="J63" t="s">
-        <v>113</v>
-      </c>
-      <c r="K63" s="8">
+    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B69" t="s">
+        <v>122</v>
+      </c>
+      <c r="C69" t="s">
+        <v>127</v>
+      </c>
+      <c r="J69" t="s">
+        <v>112</v>
+      </c>
+      <c r="K69" s="8">
         <f>0.7/1000/0.16</f>
         <v>4.3749999999999995E-3</v>
       </c>
-      <c r="L63" t="s">
+      <c r="L69" t="s">
         <v>23</v>
-      </c>
-      <c r="N63" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="65" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B65" t="s">
-        <v>127</v>
-      </c>
-      <c r="C65" t="s">
-        <v>128</v>
-      </c>
-      <c r="J65" t="s">
-        <v>108</v>
-      </c>
-      <c r="K65">
-        <v>0.06</v>
-      </c>
-      <c r="L65" t="s">
-        <v>19</v>
-      </c>
-      <c r="M65" t="s">
-        <v>124</v>
-      </c>
-      <c r="N65" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="66" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B66" t="s">
-        <v>127</v>
-      </c>
-      <c r="C66" t="s">
-        <v>128</v>
-      </c>
-      <c r="J66" t="s">
-        <v>109</v>
-      </c>
-      <c r="K66" s="17">
-        <v>0.95</v>
-      </c>
-      <c r="L66" t="s">
-        <v>20</v>
-      </c>
-      <c r="N66" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="67" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B67" t="s">
-        <v>127</v>
-      </c>
-      <c r="C67" t="s">
-        <v>128</v>
-      </c>
-      <c r="J67" t="s">
-        <v>110</v>
-      </c>
-      <c r="K67" s="8">
-        <v>0.52</v>
-      </c>
-      <c r="L67" t="s">
-        <v>29</v>
-      </c>
-      <c r="N67" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="68" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B68" t="s">
-        <v>127</v>
-      </c>
-      <c r="C68" t="s">
-        <v>128</v>
-      </c>
-      <c r="J68" t="s">
-        <v>111</v>
-      </c>
-      <c r="K68" s="8">
-        <f>3.5/1000/0.06</f>
-        <v>5.8333333333333334E-2</v>
-      </c>
-      <c r="L68" t="s">
-        <v>21</v>
-      </c>
-      <c r="N68" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="69" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B69" t="s">
-        <v>127</v>
-      </c>
-      <c r="C69" t="s">
-        <v>128</v>
-      </c>
-      <c r="J69" t="s">
-        <v>112</v>
-      </c>
-      <c r="K69" s="8">
-        <f>0.3/1000/0.06</f>
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="L69" t="s">
-        <v>22</v>
       </c>
       <c r="N69" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="70" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B70" t="s">
+    <row r="71" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B71" t="s">
+        <v>126</v>
+      </c>
+      <c r="C71" t="s">
         <v>127</v>
       </c>
-      <c r="C70" t="s">
-        <v>128</v>
-      </c>
-      <c r="J70" t="s">
-        <v>113</v>
-      </c>
-      <c r="K70" s="8">
-        <f>0.6/1000/0.06</f>
-        <v>0.01</v>
-      </c>
-      <c r="L70" t="s">
-        <v>23</v>
-      </c>
-      <c r="N70" t="s">
+      <c r="J71" t="s">
+        <v>107</v>
+      </c>
+      <c r="K71">
+        <v>0.06</v>
+      </c>
+      <c r="L71" t="s">
+        <v>19</v>
+      </c>
+      <c r="M71" t="s">
+        <v>123</v>
+      </c>
+      <c r="N71" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1985,19 +1979,16 @@
         <v>126</v>
       </c>
       <c r="C72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J72" t="s">
         <v>108</v>
       </c>
-      <c r="K72">
-        <v>7.0000000000000007E-2</v>
+      <c r="K72" s="17">
+        <v>0.95</v>
       </c>
       <c r="L72" t="s">
-        <v>19</v>
-      </c>
-      <c r="M72" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
       <c r="N72" t="s">
         <v>44</v>
@@ -2008,16 +1999,16 @@
         <v>126</v>
       </c>
       <c r="C73" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J73" t="s">
         <v>109</v>
       </c>
-      <c r="K73" s="17">
-        <v>0.97</v>
+      <c r="K73" s="8">
+        <v>0.52</v>
       </c>
       <c r="L73" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="N73" t="s">
         <v>44</v>
@@ -2028,16 +2019,17 @@
         <v>126</v>
       </c>
       <c r="C74" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J74" t="s">
         <v>110</v>
       </c>
-      <c r="K74">
-        <v>0.32300000000000001</v>
+      <c r="K74" s="8">
+        <f>3.5/1000/0.06</f>
+        <v>5.8333333333333334E-2</v>
       </c>
       <c r="L74" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="N74" t="s">
         <v>44</v>
@@ -2048,17 +2040,17 @@
         <v>126</v>
       </c>
       <c r="C75" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J75" t="s">
         <v>111</v>
       </c>
       <c r="K75" s="8">
-        <f>3.7/1000/0.07</f>
-        <v>5.2857142857142853E-2</v>
+        <f>0.3/1000/0.06</f>
+        <v>5.0000000000000001E-3</v>
       </c>
       <c r="L75" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N75" t="s">
         <v>44</v>
@@ -2069,1259 +2061,1285 @@
         <v>126</v>
       </c>
       <c r="C76" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="J76" t="s">
         <v>112</v>
       </c>
       <c r="K76" s="8">
+        <f>0.6/1000/0.06</f>
+        <v>0.01</v>
+      </c>
+      <c r="L76" t="s">
+        <v>23</v>
+      </c>
+      <c r="N76" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="78" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B78" t="s">
+        <v>125</v>
+      </c>
+      <c r="C78" t="s">
+        <v>127</v>
+      </c>
+      <c r="J78" t="s">
+        <v>107</v>
+      </c>
+      <c r="K78">
+        <v>7.0000000000000007E-2</v>
+      </c>
+      <c r="L78" t="s">
+        <v>19</v>
+      </c>
+      <c r="M78" t="s">
+        <v>124</v>
+      </c>
+      <c r="N78" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B79" t="s">
+        <v>125</v>
+      </c>
+      <c r="C79" t="s">
+        <v>127</v>
+      </c>
+      <c r="J79" t="s">
+        <v>108</v>
+      </c>
+      <c r="K79" s="17">
+        <v>0.97</v>
+      </c>
+      <c r="L79" t="s">
+        <v>20</v>
+      </c>
+      <c r="N79" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="B80" t="s">
+        <v>125</v>
+      </c>
+      <c r="C80" t="s">
+        <v>127</v>
+      </c>
+      <c r="J80" t="s">
+        <v>109</v>
+      </c>
+      <c r="K80">
+        <v>0.32300000000000001</v>
+      </c>
+      <c r="L80" t="s">
+        <v>29</v>
+      </c>
+      <c r="N80" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B81" t="s">
+        <v>125</v>
+      </c>
+      <c r="C81" t="s">
+        <v>127</v>
+      </c>
+      <c r="J81" t="s">
+        <v>110</v>
+      </c>
+      <c r="K81" s="8">
+        <f>3.7/1000/0.07</f>
+        <v>5.2857142857142853E-2</v>
+      </c>
+      <c r="L81" t="s">
+        <v>21</v>
+      </c>
+      <c r="N81" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B82" t="s">
+        <v>125</v>
+      </c>
+      <c r="C82" t="s">
+        <v>127</v>
+      </c>
+      <c r="J82" t="s">
+        <v>111</v>
+      </c>
+      <c r="K82" s="8">
         <f>0.3/1000/0.07</f>
         <v>4.2857142857142851E-3</v>
       </c>
-      <c r="L76" t="s">
+      <c r="L82" t="s">
         <v>22</v>
       </c>
-      <c r="N76" t="s">
+      <c r="N82" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="77" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B77" t="s">
-        <v>126</v>
-      </c>
-      <c r="C77" t="s">
-        <v>128</v>
-      </c>
-      <c r="J77" t="s">
-        <v>113</v>
-      </c>
-      <c r="K77" s="8">
+    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B83" t="s">
+        <v>125</v>
+      </c>
+      <c r="C83" t="s">
+        <v>127</v>
+      </c>
+      <c r="J83" t="s">
+        <v>112</v>
+      </c>
+      <c r="K83" s="8">
         <f>0.5/1000/0.07</f>
         <v>7.1428571428571426E-3</v>
       </c>
-      <c r="L77" t="s">
+      <c r="L83" t="s">
         <v>23</v>
       </c>
-      <c r="N77" t="s">
+      <c r="N83" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="79" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B79" t="s">
-        <v>129</v>
-      </c>
-      <c r="C79" t="s">
+    <row r="85" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B85" t="s">
         <v>128</v>
       </c>
-      <c r="J79" t="s">
-        <v>108</v>
-      </c>
-      <c r="K79" s="6">
-        <f>K44</f>
+      <c r="C85" t="s">
+        <v>127</v>
+      </c>
+      <c r="J85" t="s">
+        <v>107</v>
+      </c>
+      <c r="K85" s="6">
+        <f>K43</f>
         <v>0.15</v>
       </c>
-      <c r="L79" t="s">
+      <c r="L85" t="s">
         <v>19</v>
       </c>
-      <c r="M79" s="7" t="s">
+      <c r="M85" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="80" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="B80" t="s">
-        <v>129</v>
-      </c>
-      <c r="C80" t="s">
+    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B86" t="s">
         <v>128</v>
       </c>
-      <c r="J80" t="s">
-        <v>109</v>
-      </c>
-      <c r="K80" s="6">
-        <f t="shared" ref="K80:K84" si="1">K45</f>
-        <v>0.9</v>
-      </c>
-      <c r="L80" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="81" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B81" t="s">
-        <v>129</v>
-      </c>
-      <c r="C81" t="s">
-        <v>128</v>
-      </c>
-      <c r="J81" t="s">
-        <v>110</v>
-      </c>
-      <c r="K81" s="9">
-        <f t="shared" si="1"/>
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="L81" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="82" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B82" t="s">
-        <v>129</v>
-      </c>
-      <c r="C82" t="s">
-        <v>128</v>
-      </c>
-      <c r="J82" t="s">
-        <v>111</v>
-      </c>
-      <c r="K82" s="9">
-        <f t="shared" si="1"/>
-        <v>2.5333333333333333E-2</v>
-      </c>
-      <c r="L82" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="83" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B83" t="s">
-        <v>129</v>
-      </c>
-      <c r="C83" t="s">
-        <v>128</v>
-      </c>
-      <c r="J83" t="s">
-        <v>112</v>
-      </c>
-      <c r="K83" s="9">
-        <f t="shared" si="1"/>
-        <v>3.3333333333333335E-3</v>
-      </c>
-      <c r="L83" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="84" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B84" t="s">
-        <v>129</v>
-      </c>
-      <c r="C84" t="s">
-        <v>128</v>
-      </c>
-      <c r="J84" t="s">
-        <v>113</v>
-      </c>
-      <c r="K84" s="9">
-        <f t="shared" si="1"/>
-        <v>8.0000000000000002E-3</v>
-      </c>
-      <c r="L84" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="86" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A86" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B86" s="4"/>
       <c r="C86" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="J86" t="s">
         <v>108</v>
       </c>
-      <c r="K86">
-        <v>1</v>
+      <c r="K86" s="6">
+        <f t="shared" ref="K86:K90" si="2">K44</f>
+        <v>0.9</v>
       </c>
       <c r="L86" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A87" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B87" s="4"/>
+      <c r="B87" t="s">
+        <v>128</v>
+      </c>
       <c r="C87" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="J87" t="s">
         <v>109</v>
       </c>
-      <c r="K87">
-        <v>0.88</v>
+      <c r="K87" s="9">
+        <f t="shared" si="2"/>
+        <v>0.55000000000000004</v>
       </c>
       <c r="L87" t="s">
-        <v>20</v>
-      </c>
-      <c r="N87" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A88" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B88" s="4"/>
+      <c r="B88" t="s">
+        <v>128</v>
+      </c>
       <c r="C88" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="J88" t="s">
         <v>110</v>
       </c>
-      <c r="K88" s="8">
-        <v>0.3</v>
+      <c r="K88" s="9">
+        <f t="shared" si="2"/>
+        <v>2.5333333333333333E-2</v>
       </c>
       <c r="L88" t="s">
-        <v>29</v>
-      </c>
-      <c r="N88" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A89" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B89" s="4"/>
+      <c r="B89" t="s">
+        <v>128</v>
+      </c>
       <c r="C89" t="s">
-        <v>43</v>
+        <v>127</v>
       </c>
       <c r="J89" t="s">
         <v>111</v>
       </c>
-      <c r="K89" s="4">
+      <c r="K89" s="9">
+        <f t="shared" si="2"/>
+        <v>3.3333333333333335E-3</v>
+      </c>
+      <c r="L89" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B90" t="s">
+        <v>128</v>
+      </c>
+      <c r="C90" t="s">
+        <v>127</v>
+      </c>
+      <c r="J90" t="s">
+        <v>112</v>
+      </c>
+      <c r="K90" s="9">
+        <f t="shared" si="2"/>
+        <v>8.0000000000000002E-3</v>
+      </c>
+      <c r="L90" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A92" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B92" s="4"/>
+      <c r="C92" t="s">
+        <v>43</v>
+      </c>
+      <c r="J92" t="s">
+        <v>107</v>
+      </c>
+      <c r="K92">
+        <v>1</v>
+      </c>
+      <c r="L92" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A93" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B93" s="4"/>
+      <c r="C93" t="s">
+        <v>43</v>
+      </c>
+      <c r="J93" t="s">
+        <v>108</v>
+      </c>
+      <c r="K93">
+        <v>0.88</v>
+      </c>
+      <c r="L93" t="s">
+        <v>20</v>
+      </c>
+      <c r="N93" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A94" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B94" s="4"/>
+      <c r="C94" t="s">
+        <v>43</v>
+      </c>
+      <c r="J94" t="s">
+        <v>109</v>
+      </c>
+      <c r="K94" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="L94" t="s">
+        <v>29</v>
+      </c>
+      <c r="N94" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A95" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B95" s="4"/>
+      <c r="C95" t="s">
+        <v>43</v>
+      </c>
+      <c r="J95" t="s">
+        <v>110</v>
+      </c>
+      <c r="K95" s="4">
         <f>2.1/100</f>
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="L89" t="s">
+      <c r="L95" t="s">
         <v>21</v>
       </c>
-      <c r="N89" t="s">
+      <c r="N95" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="90" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A90" s="4" t="s">
+    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A96" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B90" s="4"/>
-      <c r="C90" t="s">
+      <c r="B96" s="4"/>
+      <c r="C96" t="s">
         <v>43</v>
       </c>
-      <c r="J90" t="s">
-        <v>112</v>
-      </c>
-      <c r="K90" s="11">
+      <c r="J96" t="s">
+        <v>111</v>
+      </c>
+      <c r="K96" s="11">
         <f>0.27/100</f>
         <v>2.7000000000000001E-3</v>
       </c>
-      <c r="L90" t="s">
+      <c r="L96" t="s">
         <v>22</v>
       </c>
-      <c r="N90" t="s">
+      <c r="N96" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="91" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A91" s="4" t="s">
+    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A97" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B91" s="4"/>
-      <c r="C91" t="s">
+      <c r="B97" s="4"/>
+      <c r="C97" t="s">
         <v>43</v>
       </c>
-      <c r="J91" t="s">
-        <v>113</v>
-      </c>
-      <c r="K91" s="11">
+      <c r="J97" t="s">
+        <v>112</v>
+      </c>
+      <c r="K97" s="11">
         <f>2.34/100</f>
         <v>2.3399999999999997E-2</v>
       </c>
-      <c r="L91" t="s">
+      <c r="L97" t="s">
         <v>23</v>
       </c>
-      <c r="N91" t="s">
+      <c r="N97" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="92" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A92" s="4"/>
-      <c r="B92" s="4"/>
-      <c r="K92" s="11"/>
-    </row>
-    <row r="93" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A93" s="2" t="s">
+    <row r="98" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A98" s="4"/>
+      <c r="B98" s="4"/>
+      <c r="K98" s="11"/>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="B93" s="2"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="2"/>
-      <c r="G93" s="2"/>
-      <c r="H93" s="2"/>
-      <c r="I93" s="2"/>
-      <c r="J93" s="2"/>
-      <c r="K93" s="2"/>
-      <c r="L93" s="2"/>
-      <c r="M93" s="2"/>
-      <c r="N93" s="2"/>
-    </row>
-    <row r="94" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A94" s="4"/>
-      <c r="B94" s="4"/>
-      <c r="C94" s="4"/>
-      <c r="D94" s="4"/>
-      <c r="E94" s="4"/>
-      <c r="F94" s="4"/>
-      <c r="G94" s="4"/>
-      <c r="H94" s="4"/>
-      <c r="I94" s="4"/>
-      <c r="J94" s="4"/>
-      <c r="K94" s="4"/>
-      <c r="L94" s="4"/>
-      <c r="M94" s="4"/>
-      <c r="N94" s="4"/>
-    </row>
-    <row r="95" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A95" s="4"/>
-      <c r="B95" s="4"/>
-      <c r="J95" t="s">
+      <c r="B99" s="2"/>
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+      <c r="H99" s="2"/>
+      <c r="I99" s="2"/>
+      <c r="J99" s="2"/>
+      <c r="K99" s="2"/>
+      <c r="L99" s="2"/>
+      <c r="M99" s="2"/>
+      <c r="N99" s="2"/>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A100" s="4"/>
+      <c r="B100" s="4"/>
+      <c r="C100" s="4"/>
+      <c r="D100" s="4"/>
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="4"/>
+      <c r="J100" s="4"/>
+      <c r="K100" s="4"/>
+      <c r="L100" s="4"/>
+      <c r="M100" s="4"/>
+      <c r="N100" s="4"/>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A101" s="4"/>
+      <c r="B101" s="4"/>
+      <c r="J101" t="s">
         <v>56</v>
       </c>
-      <c r="K95" s="11">
+      <c r="K101" s="11">
         <v>0.71750000000000003</v>
       </c>
-      <c r="L95" t="s">
+      <c r="L101" t="s">
         <v>57</v>
       </c>
-      <c r="N95" t="s">
+      <c r="N101" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="96" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A96" s="4"/>
-      <c r="B96" s="4"/>
-      <c r="J96" t="s">
+    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A102" s="4"/>
+      <c r="B102" s="4"/>
+      <c r="J102" t="s">
         <v>58</v>
       </c>
-      <c r="K96" s="11">
+      <c r="K102" s="11">
         <v>1.9496</v>
       </c>
-      <c r="L96" t="s">
+      <c r="L102" t="s">
         <v>57</v>
       </c>
-      <c r="N96" t="s">
+      <c r="N102" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="97" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A97" s="4"/>
-      <c r="B97" s="4"/>
-      <c r="J97" t="s">
+    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A103" s="4"/>
+      <c r="B103" s="4"/>
+      <c r="J103" t="s">
         <v>96</v>
       </c>
-      <c r="K97" s="13">
+      <c r="K103" s="13">
         <f>50*(1/3.6)</f>
         <v>13.888888888888889</v>
       </c>
-      <c r="L97" t="s">
+      <c r="L103" t="s">
         <v>92</v>
       </c>
-      <c r="M97" t="s">
+      <c r="M103" t="s">
         <v>91</v>
       </c>
-      <c r="N97" t="s">
+      <c r="N103" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="99" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A99" s="19" t="s">
+    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A105" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B99" s="19"/>
-      <c r="C99" s="19"/>
-      <c r="D99" s="19"/>
-      <c r="E99" s="19"/>
-      <c r="F99" s="19"/>
-      <c r="G99" s="19"/>
-      <c r="H99" s="19"/>
-      <c r="I99" s="19"/>
-      <c r="J99" s="19"/>
-      <c r="K99" s="19"/>
-      <c r="L99" s="19"/>
-      <c r="M99" s="19"/>
-      <c r="N99" s="19"/>
-    </row>
-    <row r="100" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A100" s="14" t="s">
+      <c r="B105" s="19"/>
+      <c r="C105" s="19"/>
+      <c r="D105" s="19"/>
+      <c r="E105" s="19"/>
+      <c r="F105" s="19"/>
+      <c r="G105" s="19"/>
+      <c r="H105" s="19"/>
+      <c r="I105" s="19"/>
+      <c r="J105" s="19"/>
+      <c r="K105" s="19"/>
+      <c r="L105" s="19"/>
+      <c r="M105" s="19"/>
+      <c r="N105" s="19"/>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A106" s="14" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="101" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J101" t="s">
+    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J107" t="s">
         <v>30</v>
       </c>
-      <c r="K101" s="4">
+      <c r="K107" s="4">
         <v>90</v>
       </c>
-      <c r="L101" s="4" t="s">
+      <c r="L107" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="M101" s="4" t="s">
+      <c r="M107" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="N101" t="s">
+      <c r="N107" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="102" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J102" t="s">
+    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J108" t="s">
         <v>36</v>
       </c>
-      <c r="K102" s="4">
+      <c r="K108" s="4">
         <v>0.22</v>
       </c>
-      <c r="L102" s="4" t="s">
+      <c r="L108" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="M102" s="7"/>
-      <c r="N102" t="s">
+      <c r="M108" s="7"/>
+      <c r="N108" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="103" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J103" t="s">
+    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J109" t="s">
         <v>34</v>
       </c>
-      <c r="K103" s="4">
+      <c r="K109" s="4">
         <v>3.4</v>
       </c>
-      <c r="L103" s="4" t="s">
+      <c r="L109" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="M103" s="7"/>
-      <c r="N103" t="s">
+      <c r="M109" s="7"/>
+      <c r="N109" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="104" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J104" t="s">
+    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J110" t="s">
         <v>35</v>
       </c>
-      <c r="K104" s="4">
+      <c r="K110" s="4">
         <v>5</v>
       </c>
-      <c r="L104" s="4" t="s">
+      <c r="L110" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="M104" s="7"/>
-      <c r="N104" t="s">
+      <c r="M110" s="7"/>
+      <c r="N110" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="105" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A105" s="14" t="s">
+    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A111" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="K105" s="4"/>
-      <c r="L105" s="4"/>
-      <c r="M105" s="7"/>
-    </row>
-    <row r="106" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I106" t="s">
+      <c r="K111" s="4"/>
+      <c r="L111" s="4"/>
+      <c r="M111" s="7"/>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I112" t="s">
         <v>78</v>
       </c>
-      <c r="J106" t="s">
+      <c r="J112" t="s">
         <v>80</v>
       </c>
-      <c r="K106" s="4">
+      <c r="K112" s="4">
         <v>0.61</v>
       </c>
-      <c r="L106" s="4" t="s">
+      <c r="L112" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="M106" s="4" t="s">
+      <c r="M112" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="N106" t="s">
+      <c r="N112" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="107" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="I107" t="s">
+    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="I113" t="s">
         <v>79</v>
       </c>
-      <c r="J107" t="s">
+      <c r="J113" t="s">
         <v>80</v>
       </c>
-      <c r="K107" s="4">
+      <c r="K113" s="4">
         <v>0.99</v>
       </c>
-      <c r="L107" s="4" t="s">
+      <c r="L113" s="4" t="s">
         <v>39</v>
-      </c>
-      <c r="M107" s="7"/>
-      <c r="N107" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="108" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A108" s="14" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="109" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C109" t="s">
-        <v>114</v>
-      </c>
-      <c r="J109" t="s">
-        <v>25</v>
-      </c>
-      <c r="K109">
-        <v>63</v>
-      </c>
-      <c r="L109" t="s">
-        <v>54</v>
-      </c>
-      <c r="N109" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="110" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C110" t="s">
-        <v>115</v>
-      </c>
-      <c r="J110" t="s">
-        <v>25</v>
-      </c>
-      <c r="K110">
-        <v>59</v>
-      </c>
-      <c r="L110" t="s">
-        <v>54</v>
-      </c>
-      <c r="N110" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="111" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C111" t="s">
-        <v>116</v>
-      </c>
-      <c r="J111" t="s">
-        <v>25</v>
-      </c>
-      <c r="K111" s="6">
-        <f>K110</f>
-        <v>59</v>
-      </c>
-      <c r="L111" t="s">
-        <v>54</v>
-      </c>
-      <c r="M111" s="7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="112" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B112" t="s">
-        <v>123</v>
-      </c>
-      <c r="C112" t="s">
-        <v>128</v>
-      </c>
-      <c r="J112" t="s">
-        <v>25</v>
-      </c>
-      <c r="K112" s="4">
-        <v>65</v>
-      </c>
-      <c r="L112" t="s">
-        <v>54</v>
-      </c>
-      <c r="M112" s="7"/>
-      <c r="N112" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="113" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B113" t="s">
-        <v>127</v>
-      </c>
-      <c r="C113" t="s">
-        <v>128</v>
-      </c>
-      <c r="J113" t="s">
-        <v>25</v>
-      </c>
-      <c r="K113" s="4">
-        <v>65</v>
-      </c>
-      <c r="L113" t="s">
-        <v>54</v>
       </c>
       <c r="M113" s="7"/>
       <c r="N113" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B114" t="s">
-        <v>126</v>
-      </c>
-      <c r="C114" t="s">
-        <v>128</v>
-      </c>
-      <c r="J114" t="s">
-        <v>25</v>
-      </c>
-      <c r="K114" s="4">
-        <v>65</v>
-      </c>
-      <c r="L114" t="s">
-        <v>54</v>
-      </c>
-      <c r="M114" s="7"/>
-      <c r="N114" t="s">
-        <v>44</v>
+      <c r="A114" s="14" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B115" t="s">
-        <v>129</v>
-      </c>
       <c r="C115" t="s">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="J115" t="s">
         <v>25</v>
       </c>
-      <c r="K115" s="6">
-        <f>K110</f>
-        <v>59</v>
+      <c r="K115">
+        <v>63</v>
       </c>
       <c r="L115" t="s">
         <v>54</v>
       </c>
-      <c r="M115" s="7" t="s">
-        <v>27</v>
+      <c r="N115" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A116" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B116" s="4"/>
       <c r="C116" t="s">
-        <v>43</v>
+        <v>114</v>
       </c>
       <c r="J116" t="s">
         <v>25</v>
       </c>
       <c r="K116">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="L116" t="s">
         <v>54</v>
       </c>
-      <c r="M116" t="s">
-        <v>62</v>
-      </c>
       <c r="N116" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.25">
       <c r="C117" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="J117" t="s">
         <v>25</v>
       </c>
-      <c r="K117" s="4">
-        <v>65</v>
+      <c r="K117" s="6">
+        <f>K116</f>
+        <v>59</v>
       </c>
       <c r="L117" t="s">
         <v>54</v>
       </c>
-      <c r="M117" t="s">
+      <c r="M117" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C118" t="s">
+        <v>102</v>
+      </c>
+      <c r="J118" t="s">
+        <v>25</v>
+      </c>
+      <c r="K118" s="6">
+        <f>K119</f>
+        <v>65</v>
+      </c>
+      <c r="L118" t="s">
+        <v>54</v>
+      </c>
+      <c r="M118" s="7"/>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B119" t="s">
+        <v>122</v>
+      </c>
+      <c r="C119" t="s">
+        <v>127</v>
+      </c>
+      <c r="J119" t="s">
+        <v>25</v>
+      </c>
+      <c r="K119" s="4">
+        <v>65</v>
+      </c>
+      <c r="L119" t="s">
+        <v>54</v>
+      </c>
+      <c r="M119" s="7"/>
+      <c r="N119" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B120" t="s">
+        <v>126</v>
+      </c>
+      <c r="C120" t="s">
+        <v>127</v>
+      </c>
+      <c r="J120" t="s">
+        <v>25</v>
+      </c>
+      <c r="K120" s="4">
+        <v>65</v>
+      </c>
+      <c r="L120" t="s">
+        <v>54</v>
+      </c>
+      <c r="M120" s="7"/>
+      <c r="N120" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B121" t="s">
+        <v>125</v>
+      </c>
+      <c r="C121" t="s">
+        <v>127</v>
+      </c>
+      <c r="J121" t="s">
+        <v>25</v>
+      </c>
+      <c r="K121" s="4">
+        <v>65</v>
+      </c>
+      <c r="L121" t="s">
+        <v>54</v>
+      </c>
+      <c r="M121" s="7"/>
+      <c r="N121" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B122" t="s">
+        <v>128</v>
+      </c>
+      <c r="C122" t="s">
+        <v>127</v>
+      </c>
+      <c r="J122" t="s">
+        <v>25</v>
+      </c>
+      <c r="K122" s="6">
+        <f>K116</f>
+        <v>59</v>
+      </c>
+      <c r="L122" t="s">
+        <v>54</v>
+      </c>
+      <c r="M122" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A123" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B123" s="4"/>
+      <c r="C123" t="s">
+        <v>43</v>
+      </c>
+      <c r="J123" t="s">
+        <v>25</v>
+      </c>
+      <c r="K123">
+        <v>56</v>
+      </c>
+      <c r="L123" t="s">
+        <v>54</v>
+      </c>
+      <c r="M123" t="s">
+        <v>62</v>
+      </c>
+      <c r="N123" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="C124" t="s">
+        <v>31</v>
+      </c>
+      <c r="J124" t="s">
+        <v>25</v>
+      </c>
+      <c r="K124" s="4">
+        <v>65</v>
+      </c>
+      <c r="L124" t="s">
+        <v>54</v>
+      </c>
+      <c r="M124" t="s">
         <v>61</v>
       </c>
-      <c r="N117" t="s">
+      <c r="N124" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="118" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A118" s="14" t="s">
+    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A125" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="K118" s="4"/>
-      <c r="L118" s="4"/>
-      <c r="M118" s="7"/>
-    </row>
-    <row r="119" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H119" t="s">
-        <v>84</v>
-      </c>
-      <c r="J119" t="s">
-        <v>81</v>
-      </c>
-      <c r="K119" s="13">
-        <f>1041/(50+3+1041)*100</f>
-        <v>95.155393053016454</v>
-      </c>
-      <c r="L119" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="M119" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="N119" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="120" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H120" t="s">
-        <v>79</v>
-      </c>
-      <c r="J120" t="s">
-        <v>81</v>
-      </c>
-      <c r="K120" s="12">
-        <f>50/(50+3+1041)*100</f>
-        <v>4.5703839122486292</v>
-      </c>
-      <c r="L120" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="M120" s="4"/>
-      <c r="N120" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="121" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H121" t="s">
-        <v>78</v>
-      </c>
-      <c r="J121" t="s">
-        <v>81</v>
-      </c>
-      <c r="K121" s="12">
-        <f>3/(50+3+1041)*100</f>
-        <v>0.27422303473491771</v>
-      </c>
-      <c r="L121" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="M121" s="4"/>
-      <c r="N121" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="122" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A122" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="K122" s="4"/>
-      <c r="L122" s="4"/>
-      <c r="M122" s="4"/>
-    </row>
-    <row r="123" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A123" s="15"/>
-      <c r="B123" s="3"/>
-      <c r="C123" s="3"/>
-      <c r="D123" s="3"/>
-      <c r="E123" s="3"/>
-      <c r="F123" s="3"/>
-      <c r="G123" s="3"/>
-      <c r="H123" s="3"/>
-      <c r="I123" s="3"/>
-      <c r="J123" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="K123" s="3">
-        <v>0</v>
-      </c>
-      <c r="L123" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="M123" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="124" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A124" s="15"/>
-      <c r="B124" s="3"/>
-      <c r="C124" s="3"/>
-      <c r="D124" s="3"/>
-      <c r="E124" s="3"/>
-      <c r="F124" s="3"/>
-      <c r="G124" s="3"/>
-      <c r="H124" s="3"/>
-      <c r="I124" s="3"/>
-      <c r="J124" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="K124" s="3">
-        <v>0</v>
-      </c>
-      <c r="L124" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="M124" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="125" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H125" t="s">
-        <v>84</v>
-      </c>
-      <c r="J125" t="s">
-        <v>82</v>
-      </c>
-      <c r="K125" s="4">
-        <v>0.5</v>
-      </c>
-      <c r="L125" s="4" t="s">
-        <v>100</v>
-      </c>
+      <c r="K125" s="4"/>
+      <c r="L125" s="4"/>
       <c r="M125" s="7"/>
-      <c r="N125" t="s">
-        <v>53</v>
-      </c>
     </row>
     <row r="126" spans="1:14" x14ac:dyDescent="0.25">
       <c r="H126" t="s">
         <v>84</v>
       </c>
-      <c r="I126" t="s">
+      <c r="J126" t="s">
+        <v>81</v>
+      </c>
+      <c r="K126" s="13">
+        <f>1041/(50+3+1041)*100</f>
+        <v>95.155393053016454</v>
+      </c>
+      <c r="L126" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M126" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="N126" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H127" t="s">
+        <v>79</v>
+      </c>
+      <c r="J127" t="s">
+        <v>81</v>
+      </c>
+      <c r="K127" s="12">
+        <f>50/(50+3+1041)*100</f>
+        <v>4.5703839122486292</v>
+      </c>
+      <c r="L127" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M127" s="4"/>
+      <c r="N127" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H128" t="s">
         <v>78</v>
       </c>
-      <c r="J126" t="s">
+      <c r="J128" t="s">
+        <v>81</v>
+      </c>
+      <c r="K128" s="12">
+        <f>3/(50+3+1041)*100</f>
+        <v>0.27422303473491771</v>
+      </c>
+      <c r="L128" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="M128" s="4"/>
+      <c r="N128" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A129" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="K129" s="4"/>
+      <c r="L129" s="4"/>
+      <c r="M129" s="4"/>
+    </row>
+    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A130" s="15"/>
+      <c r="B130" s="3"/>
+      <c r="C130" s="3"/>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3"/>
+      <c r="G130" s="3"/>
+      <c r="H130" s="3"/>
+      <c r="I130" s="3"/>
+      <c r="J130" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="K130" s="3">
+        <v>0</v>
+      </c>
+      <c r="L130" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="M130" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A131" s="15"/>
+      <c r="B131" s="3"/>
+      <c r="C131" s="3"/>
+      <c r="D131" s="3"/>
+      <c r="E131" s="3"/>
+      <c r="F131" s="3"/>
+      <c r="G131" s="3"/>
+      <c r="H131" s="3"/>
+      <c r="I131" s="3"/>
+      <c r="J131" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="K126" s="10">
+      <c r="K131" s="3">
+        <v>0</v>
+      </c>
+      <c r="L131" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="M131" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H132" t="s">
+        <v>84</v>
+      </c>
+      <c r="J132" t="s">
+        <v>82</v>
+      </c>
+      <c r="K132" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="L132" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="M132" s="7"/>
+      <c r="N132" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H133" t="s">
+        <v>84</v>
+      </c>
+      <c r="I133" t="s">
+        <v>78</v>
+      </c>
+      <c r="J133" t="s">
+        <v>83</v>
+      </c>
+      <c r="K133" s="10">
         <f>0.9 * (1/3.6) / 0.6 / 0.718</f>
         <v>0.5803156917363046</v>
       </c>
-      <c r="L126" s="4" t="s">
+      <c r="L133" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="M126" s="4" t="s">
+      <c r="M133" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="N126" t="s">
+      <c r="N133" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="127" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A127" s="14" t="s">
+    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A134" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="K127" s="4"/>
-      <c r="L127" s="4"/>
-      <c r="M127" s="7"/>
-    </row>
-    <row r="128" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J128" t="s">
+      <c r="K134" s="4"/>
+      <c r="L134" s="4"/>
+      <c r="M134" s="7"/>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J135" t="s">
         <v>49</v>
       </c>
-      <c r="K128" s="11">
+      <c r="K135" s="11">
         <f>238/0.74/1000</f>
         <v>0.32162162162162161</v>
       </c>
-      <c r="L128" s="4" t="s">
+      <c r="L135" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="M128" s="7"/>
-      <c r="N128" t="s">
+      <c r="M135" s="7"/>
+      <c r="N135" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="129" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J129" t="s">
+    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J136" t="s">
         <v>59</v>
       </c>
-      <c r="K129" s="12">
+      <c r="K136" s="12">
         <v>1.5</v>
       </c>
-      <c r="L129" s="4" t="s">
+      <c r="L136" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="M129" s="7"/>
-      <c r="N129" t="s">
+      <c r="M136" s="7"/>
+      <c r="N136" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="130" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J130" t="s">
+    <row r="137" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J137" t="s">
         <v>50</v>
       </c>
-      <c r="K130" s="13">
+      <c r="K137" s="13">
         <v>60</v>
       </c>
-      <c r="L130" s="4" t="s">
+      <c r="L137" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="M130" s="7"/>
-      <c r="N130" t="s">
+      <c r="M137" s="7"/>
+      <c r="N137" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J132" s="3" t="s">
+    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J139" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="K132" s="3">
+      <c r="K139" s="3">
         <v>0</v>
       </c>
-      <c r="L132" s="3"/>
-      <c r="M132" s="3" t="s">
+      <c r="L139" s="3"/>
+      <c r="M139" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F133" t="s">
+    <row r="140" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F140" t="s">
         <v>65</v>
       </c>
-      <c r="G133" t="s">
+      <c r="G140" t="s">
         <v>67</v>
       </c>
-      <c r="J133" t="s">
+      <c r="J140" t="s">
         <v>66</v>
       </c>
-      <c r="K133">
+      <c r="K140">
         <v>2.75</v>
       </c>
-      <c r="L133" t="s">
+      <c r="L140" t="s">
         <v>51</v>
       </c>
-      <c r="M133" t="s">
-        <v>121</v>
-      </c>
-      <c r="N133" t="s">
+      <c r="M140" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F134" t="s">
+      <c r="N140" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F141" t="s">
         <v>65</v>
       </c>
-      <c r="G134" t="s">
+      <c r="G141" t="s">
         <v>68</v>
       </c>
-      <c r="J134" t="s">
+      <c r="J141" t="s">
         <v>66</v>
       </c>
-      <c r="K134">
+      <c r="K141">
         <v>0</v>
       </c>
-      <c r="L134" t="s">
+      <c r="L141" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F135" t="s">
+    <row r="142" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F142" t="s">
         <v>65</v>
       </c>
-      <c r="G135" t="s">
+      <c r="G142" t="s">
         <v>69</v>
       </c>
-      <c r="J135" t="s">
+      <c r="J142" t="s">
         <v>66</v>
       </c>
-      <c r="K135">
+      <c r="K142">
         <v>0</v>
       </c>
-      <c r="L135" t="s">
+      <c r="L142" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="136" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F136" t="s">
+    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F143" t="s">
         <v>65</v>
       </c>
-      <c r="G136" t="s">
+      <c r="G143" t="s">
         <v>70</v>
       </c>
-      <c r="J136" t="s">
+      <c r="J143" t="s">
         <v>66</v>
       </c>
-      <c r="K136">
+      <c r="K143">
         <v>0</v>
       </c>
-      <c r="L136" t="s">
+      <c r="L143" t="s">
         <v>71</v>
       </c>
-      <c r="N136" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="138" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F138" t="s">
+      <c r="N143" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F145" t="s">
         <v>72</v>
       </c>
-      <c r="G138" t="s">
+      <c r="G145" t="s">
         <v>72</v>
       </c>
-      <c r="J138" t="s">
+      <c r="J145" t="s">
         <v>66</v>
       </c>
-      <c r="K138">
+      <c r="K145">
         <v>0</v>
       </c>
-      <c r="L138" t="s">
+      <c r="L145" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="139" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F139" t="s">
+    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F146" t="s">
         <v>73</v>
       </c>
-      <c r="G139" t="s">
+      <c r="G146" t="s">
         <v>73</v>
       </c>
-      <c r="J139" t="s">
+      <c r="J146" t="s">
         <v>66</v>
       </c>
-      <c r="K139">
+      <c r="K146">
         <v>0</v>
       </c>
-      <c r="L139" t="s">
+      <c r="L146" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A141" s="18" t="s">
-        <v>131</v>
-      </c>
-      <c r="B141" s="18"/>
-      <c r="C141" s="18"/>
-      <c r="D141" s="18"/>
-      <c r="E141" s="18"/>
-      <c r="F141" s="18"/>
-      <c r="G141" s="18"/>
-      <c r="H141" s="18"/>
-      <c r="I141" s="18"/>
-      <c r="J141" s="18"/>
-      <c r="K141" s="18"/>
-      <c r="L141" s="18"/>
-      <c r="M141" s="18"/>
-      <c r="N141" s="18"/>
-    </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J143" t="s">
-        <v>135</v>
-      </c>
-      <c r="K143" s="20">
+    <row r="148" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A148" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="B148" s="18"/>
+      <c r="C148" s="18"/>
+      <c r="D148" s="18"/>
+      <c r="E148" s="18"/>
+      <c r="F148" s="18"/>
+      <c r="G148" s="18"/>
+      <c r="H148" s="18"/>
+      <c r="I148" s="18"/>
+      <c r="J148" s="18"/>
+      <c r="K148" s="18"/>
+      <c r="L148" s="18"/>
+      <c r="M148" s="18"/>
+      <c r="N148" s="18"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J150" t="s">
+        <v>134</v>
+      </c>
+      <c r="K150" s="20">
         <f>2.5/0.33/0.85</f>
         <v>8.9126559714795004</v>
       </c>
-      <c r="L143" t="s">
+      <c r="L150" t="s">
+        <v>132</v>
+      </c>
+      <c r="M150" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J152" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="M143" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="145" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J145" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="K145" s="3">
+      <c r="K152" s="3">
         <v>0</v>
       </c>
-      <c r="L145" s="3" t="s">
+      <c r="L152" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="M145" s="3" t="s">
+      <c r="M152" s="3" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="146" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H146" t="s">
+    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H153" t="s">
         <v>78</v>
       </c>
-      <c r="J146" t="s">
-        <v>134</v>
-      </c>
-      <c r="K146" s="8">
+      <c r="J153" t="s">
+        <v>133</v>
+      </c>
+      <c r="K153" s="8">
         <f>0.94*0.184</f>
         <v>0.17295999999999997</v>
       </c>
-      <c r="L146" t="s">
+      <c r="L153" t="s">
         <v>97</v>
       </c>
-      <c r="N146" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="147" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="H147" t="s">
+      <c r="N153" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="H154" t="s">
         <v>79</v>
       </c>
-      <c r="J147" t="s">
-        <v>134</v>
-      </c>
-      <c r="K147" s="8">
+      <c r="J154" t="s">
+        <v>133</v>
+      </c>
+      <c r="K154" s="8">
         <f>0.94*0.816</f>
         <v>0.76703999999999994</v>
       </c>
-      <c r="L147" t="s">
+      <c r="L154" t="s">
         <v>97</v>
       </c>
-      <c r="N147" t="s">
+      <c r="N154" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J156" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="K156" s="3">
+        <v>0</v>
+      </c>
+      <c r="L156" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="M156" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F157" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J149" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="K149" s="3">
-        <v>0</v>
-      </c>
-      <c r="L149" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="M149" s="3" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F150" t="s">
+      <c r="G157" t="s">
         <v>143</v>
       </c>
-      <c r="G150" t="s">
-        <v>144</v>
-      </c>
-      <c r="J150" t="s">
-        <v>136</v>
-      </c>
-      <c r="K150" s="21">
+      <c r="J157" t="s">
+        <v>135</v>
+      </c>
+      <c r="K157" s="21">
         <f>(0.00234-0.000502)/1000/(1/3.6)</f>
         <v>6.6168000000000008E-6</v>
       </c>
-      <c r="L150" t="s">
+      <c r="L157" t="s">
+        <v>136</v>
+      </c>
+      <c r="N157" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F158" t="s">
+        <v>65</v>
+      </c>
+      <c r="G158" t="s">
         <v>137</v>
       </c>
-      <c r="N150" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F151" t="s">
-        <v>65</v>
-      </c>
-      <c r="G151" t="s">
-        <v>138</v>
-      </c>
-      <c r="J151" t="s">
-        <v>136</v>
-      </c>
-      <c r="K151" s="21">
+      <c r="J158" t="s">
+        <v>135</v>
+      </c>
+      <c r="K158" s="21">
         <f>(0.000364 -0.00000236)/1000/(1/3.6)</f>
         <v>1.3019039999999999E-6</v>
       </c>
-      <c r="L151" t="s">
-        <v>137</v>
-      </c>
-      <c r="N151" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="152" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F152" t="s">
-        <v>65</v>
-      </c>
-      <c r="G152" t="s">
-        <v>139</v>
-      </c>
-      <c r="J152" t="s">
+      <c r="L158" t="s">
         <v>136</v>
       </c>
-      <c r="K152" s="21">
-        <f>(0.0376-0.00437)/1000/(1/3.6)</f>
-        <v>1.1962800000000001E-4</v>
-      </c>
-      <c r="L152" t="s">
-        <v>137</v>
-      </c>
-      <c r="N152" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="153" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F153" t="s">
-        <v>65</v>
-      </c>
-      <c r="G153" t="s">
+      <c r="N158" t="s">
         <v>140</v>
-      </c>
-      <c r="J153" t="s">
-        <v>136</v>
-      </c>
-      <c r="K153" s="21">
-        <f>(0.00171-0.00000236)/1000/(1/3.6)</f>
-        <v>6.1475039999999993E-6</v>
-      </c>
-      <c r="L153" t="s">
-        <v>137</v>
-      </c>
-      <c r="N153" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="155" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A155" s="22" t="s">
-        <v>145</v>
-      </c>
-      <c r="B155" s="23"/>
-      <c r="C155" s="23"/>
-      <c r="D155" s="23"/>
-      <c r="E155" s="23"/>
-      <c r="F155" s="23"/>
-      <c r="G155" s="23"/>
-      <c r="H155" s="23"/>
-      <c r="I155" s="23"/>
-      <c r="J155" s="23"/>
-      <c r="K155" s="23"/>
-      <c r="L155" s="23"/>
-      <c r="M155" s="23"/>
-      <c r="N155" s="23"/>
-    </row>
-    <row r="157" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J157" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="K157" s="3">
-        <v>0</v>
-      </c>
-      <c r="L157" s="3" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="F158" t="s">
-        <v>143</v>
-      </c>
-      <c r="G158" t="s">
-        <v>144</v>
-      </c>
-      <c r="J158" t="s">
-        <v>147</v>
-      </c>
-      <c r="K158" s="17">
-        <f>(0.00144+0.0129)/0.43</f>
-        <v>3.3348837209302325E-2</v>
-      </c>
-      <c r="L158" t="s">
-        <v>146</v>
-      </c>
-      <c r="M158" t="s">
-        <v>151</v>
-      </c>
-      <c r="N158" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="159" spans="1:14" x14ac:dyDescent="0.25">
@@ -3332,17 +3350,17 @@
         <v>138</v>
       </c>
       <c r="J159" t="s">
-        <v>147</v>
-      </c>
-      <c r="K159" s="26">
-        <f>(0)/0.43</f>
-        <v>0</v>
+        <v>135</v>
+      </c>
+      <c r="K159" s="21">
+        <f>(0.0376-0.00437)/1000/(1/3.6)</f>
+        <v>1.1962800000000001E-4</v>
       </c>
       <c r="L159" t="s">
-        <v>146</v>
-      </c>
-      <c r="M159" t="s">
-        <v>152</v>
+        <v>136</v>
+      </c>
+      <c r="N159" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="160" spans="1:14" x14ac:dyDescent="0.25">
@@ -3353,110 +3371,205 @@
         <v>139</v>
       </c>
       <c r="J160" t="s">
-        <v>147</v>
-      </c>
-      <c r="K160" s="24">
+        <v>135</v>
+      </c>
+      <c r="K160" s="21">
+        <f>(0.00171-0.00000236)/1000/(1/3.6)</f>
+        <v>6.1475039999999993E-6</v>
+      </c>
+      <c r="L160" t="s">
+        <v>136</v>
+      </c>
+      <c r="N160" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="162" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A162" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B162" s="23"/>
+      <c r="C162" s="23"/>
+      <c r="D162" s="23"/>
+      <c r="E162" s="23"/>
+      <c r="F162" s="23"/>
+      <c r="G162" s="23"/>
+      <c r="H162" s="23"/>
+      <c r="I162" s="23"/>
+      <c r="J162" s="23"/>
+      <c r="K162" s="23"/>
+      <c r="L162" s="23"/>
+      <c r="M162" s="23"/>
+      <c r="N162" s="23"/>
+    </row>
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J164" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="K164" s="3">
+        <v>0</v>
+      </c>
+      <c r="L164" s="3" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="165" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F165" t="s">
+        <v>142</v>
+      </c>
+      <c r="G165" t="s">
+        <v>143</v>
+      </c>
+      <c r="J165" t="s">
+        <v>146</v>
+      </c>
+      <c r="K165" s="17">
+        <f>(0.00144+0.0129)/0.43</f>
+        <v>3.3348837209302325E-2</v>
+      </c>
+      <c r="L165" t="s">
+        <v>145</v>
+      </c>
+      <c r="M165" t="s">
+        <v>150</v>
+      </c>
+      <c r="N165" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="166" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F166" t="s">
+        <v>65</v>
+      </c>
+      <c r="G166" t="s">
+        <v>137</v>
+      </c>
+      <c r="J166" t="s">
+        <v>146</v>
+      </c>
+      <c r="K166" s="26">
+        <f>(0)/0.43</f>
+        <v>0</v>
+      </c>
+      <c r="L166" t="s">
+        <v>145</v>
+      </c>
+      <c r="M166" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="167" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F167" t="s">
+        <v>65</v>
+      </c>
+      <c r="G167" t="s">
+        <v>138</v>
+      </c>
+      <c r="J167" t="s">
+        <v>146</v>
+      </c>
+      <c r="K167" s="24">
         <f>(0.00000208)/0.43</f>
         <v>4.8372093023255818E-6</v>
       </c>
-      <c r="L160" t="s">
+      <c r="L167" t="s">
+        <v>145</v>
+      </c>
+      <c r="M167" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="168" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F168" t="s">
+        <v>65</v>
+      </c>
+      <c r="G168" t="s">
+        <v>139</v>
+      </c>
+      <c r="J168" t="s">
         <v>146</v>
       </c>
-      <c r="M160" t="s">
+      <c r="K168" s="26">
+        <f t="shared" ref="K168" si="3">(0)/0.43</f>
+        <v>0</v>
+      </c>
+      <c r="L168" t="s">
+        <v>145</v>
+      </c>
+      <c r="M168" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="161" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F161" t="s">
+    <row r="169" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F169" t="s">
         <v>65</v>
       </c>
-      <c r="G161" t="s">
-        <v>140</v>
-      </c>
-      <c r="J161" t="s">
-        <v>147</v>
-      </c>
-      <c r="K161" s="26">
-        <f t="shared" ref="K161:K165" si="2">(0)/0.43</f>
-        <v>0</v>
-      </c>
-      <c r="L161" t="s">
+      <c r="G169" t="s">
+        <v>154</v>
+      </c>
+      <c r="J169" t="s">
         <v>146</v>
       </c>
-      <c r="M161" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="162" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F162" t="s">
-        <v>65</v>
-      </c>
-      <c r="G162" t="s">
-        <v>155</v>
-      </c>
-      <c r="J162" t="s">
-        <v>147</v>
-      </c>
-      <c r="K162" s="8">
+      <c r="K169" s="8">
         <f>(0.00152)/0.43</f>
         <v>3.534883720930233E-3</v>
       </c>
-      <c r="L162" t="s">
+      <c r="L169" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="170" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F170" t="s">
+        <v>65</v>
+      </c>
+      <c r="G170" t="s">
+        <v>147</v>
+      </c>
+      <c r="J170" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="163" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F163" t="s">
-        <v>65</v>
-      </c>
-      <c r="G163" t="s">
-        <v>148</v>
-      </c>
-      <c r="J163" t="s">
-        <v>147</v>
-      </c>
-      <c r="K163" s="25">
+      <c r="K170" s="25">
         <f>(0.00016)/0.43</f>
         <v>3.7209302325581399E-4</v>
       </c>
-      <c r="L163" t="s">
+      <c r="L170" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="171" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F171" t="s">
+        <v>72</v>
+      </c>
+      <c r="G171" t="s">
+        <v>148</v>
+      </c>
+      <c r="J171" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="164" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F164" t="s">
-        <v>72</v>
-      </c>
-      <c r="G164" t="s">
-        <v>149</v>
-      </c>
-      <c r="J164" t="s">
-        <v>147</v>
-      </c>
-      <c r="K164" s="8">
+      <c r="K171" s="8">
         <f>(0.000218)/0.43</f>
         <v>5.0697674418604657E-4</v>
       </c>
-      <c r="L164" t="s">
+      <c r="L171" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="172" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F172" t="s">
+        <v>73</v>
+      </c>
+      <c r="G172" t="s">
+        <v>73</v>
+      </c>
+      <c r="J172" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="165" spans="6:13" x14ac:dyDescent="0.25">
-      <c r="F165" t="s">
-        <v>73</v>
-      </c>
-      <c r="G165" t="s">
-        <v>73</v>
-      </c>
-      <c r="J165" t="s">
-        <v>147</v>
-      </c>
-      <c r="K165" s="17">
+      <c r="K172" s="17">
         <f>(0.00343)/0.43</f>
         <v>7.9767441860465107E-3</v>
       </c>
-      <c r="L165" t="s">
-        <v>146</v>
+      <c r="L172" t="s">
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3478,7 +3591,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Fix typo in data 'CH4'->'CH4bio'
</commit_message>
<xml_diff>
--- a/data/default/WasteAndCircularity.xlsx
+++ b/data/default/WasteAndCircularity.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jnka0003\Git repos\CIBUSmod\data\default\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B023967-62ED-42C3-A4B9-BF4FD2C641EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94707B7A-9C7D-46A8-90DE-C208AF78F8A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="450" windowWidth="28770" windowHeight="15450" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38520" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="742" uniqueCount="228">
   <si>
     <t>parameter</t>
   </si>
@@ -532,9 +532,6 @@
   </si>
   <si>
     <t>COD</t>
-  </si>
-  <si>
-    <t>CH4</t>
   </si>
   <si>
     <t>kg/kg COD</t>
@@ -1353,7 +1350,7 @@
         <v>64</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>95</v>
@@ -1411,10 +1408,10 @@
         <v>6</v>
       </c>
       <c r="N5" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="O5" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
@@ -1422,7 +1419,7 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="L7" s="25"/>
     </row>
@@ -1431,20 +1428,20 @@
         <v>142</v>
       </c>
       <c r="K8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L8" s="25">
         <f>3+17</f>
         <v>20</v>
       </c>
       <c r="M8" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q8" s="35" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="R8" s="36"/>
       <c r="S8" s="36"/>
@@ -1458,7 +1455,7 @@
         <v>164</v>
       </c>
       <c r="K9" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L9" s="25">
         <f>3+23</f>
@@ -1468,19 +1465,19 @@
         <v>159</v>
       </c>
       <c r="O9" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q9" s="29" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="R9" s="16">
         <v>8.6331450000000007</v>
       </c>
       <c r="S9" s="39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="U9" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="W9" s="30"/>
     </row>
@@ -1489,29 +1486,29 @@
         <v>65</v>
       </c>
       <c r="K10" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L10" s="26">
         <f>4+0.5</f>
         <v>4.5</v>
       </c>
       <c r="M10" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O10" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q10" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R10">
         <v>204.3</v>
       </c>
       <c r="S10" s="39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="U10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="W10" s="30"/>
     </row>
@@ -1520,17 +1517,17 @@
         <v>72</v>
       </c>
       <c r="K11" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L11" s="16">
         <f>0.33+0.18</f>
         <v>0.51</v>
       </c>
       <c r="M11" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O11" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q11" s="29"/>
       <c r="R11" s="26">
@@ -1538,10 +1535,10 @@
         <v>23.664608899769433</v>
       </c>
       <c r="S11" s="39" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="U11" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="W11" s="30"/>
     </row>
@@ -1550,20 +1547,20 @@
         <v>73</v>
       </c>
       <c r="K12" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="L12" s="16">
         <f>0.88+0.33</f>
         <v>1.21</v>
       </c>
       <c r="M12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="O12" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q12" s="29" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="R12">
         <v>0.7</v>
@@ -1584,11 +1581,11 @@
         <v>16.565226229838604</v>
       </c>
       <c r="S13" s="40" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="T13" s="33"/>
       <c r="U13" s="33" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="V13" s="33"/>
       <c r="W13" s="34"/>
@@ -1598,16 +1595,16 @@
         <v>142</v>
       </c>
       <c r="K14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L14" s="25">
         <v>15</v>
       </c>
       <c r="M14" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="O14" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.25">
@@ -1615,7 +1612,7 @@
         <v>164</v>
       </c>
       <c r="K15" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L15" s="25">
         <v>23</v>
@@ -1624,10 +1621,10 @@
         <v>159</v>
       </c>
       <c r="O15" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q15" s="35" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="R15" s="36"/>
       <c r="S15" s="36"/>
@@ -1641,28 +1638,28 @@
         <v>65</v>
       </c>
       <c r="K16" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L16" s="26">
         <v>0.6</v>
       </c>
       <c r="M16" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O16" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q16" s="29"/>
       <c r="R16" s="42" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="S16" s="42" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
       <c r="V16" s="42" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="W16" s="30"/>
     </row>
@@ -1671,19 +1668,19 @@
         <v>72</v>
       </c>
       <c r="K17" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L17" s="16">
         <v>0.25</v>
       </c>
       <c r="M17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="O17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q17" s="29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="R17" s="43">
         <f>(661848+480002+1158543+1002205+5055019)/1000000</f>
@@ -1694,7 +1691,7 @@
         <v>8.3800653749999992</v>
       </c>
       <c r="T17" s="39" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="V17" s="47">
         <f>(S17-R17)/R17</f>
@@ -1707,19 +1704,19 @@
         <v>73</v>
       </c>
       <c r="K18" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="L18" s="16">
         <v>0.28999999999999998</v>
       </c>
       <c r="M18" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="O18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="Q18" s="29" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="R18" s="44">
         <v>197778</v>
@@ -1729,7 +1726,7 @@
         <v>198310.96965387464</v>
       </c>
       <c r="T18" s="39" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="V18" s="47">
         <f t="shared" ref="V18" si="0">(S18-R18)/R18</f>
@@ -1741,33 +1738,33 @@
       <c r="L19" s="26"/>
       <c r="O19" s="27"/>
       <c r="Q19" s="29" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="R19" s="44">
         <v>47624.39</v>
       </c>
       <c r="S19" s="45"/>
       <c r="T19" s="39" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="V19" s="47"/>
       <c r="W19" s="30"/>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A20" s="28" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="L20" s="26"/>
       <c r="O20" s="27"/>
       <c r="Q20" s="29" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="R20" s="44">
         <v>26638.48</v>
       </c>
       <c r="S20" s="45"/>
       <c r="T20" s="39" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="V20" s="47"/>
       <c r="W20" s="30"/>
@@ -1792,7 +1789,7 @@
         <v>9402.4333507499978</v>
       </c>
       <c r="T21" s="39" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="V21" s="47">
         <f>(S21-R21)/R21</f>
@@ -1834,7 +1831,7 @@
         <v>5731.9647165000006</v>
       </c>
       <c r="T22" s="39" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="V22" s="47">
         <f>(S22-R22)/R22</f>
@@ -1853,7 +1850,7 @@
         <v>161</v>
       </c>
       <c r="N23" s="7" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="Q23" s="31" t="s">
         <v>73</v>
@@ -1864,7 +1861,7 @@
         <v>188.55147093749997</v>
       </c>
       <c r="T23" s="40" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="U23" s="33"/>
       <c r="V23" s="41"/>
@@ -1878,10 +1875,10 @@
         <v>72</v>
       </c>
       <c r="M24" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="N24" s="7" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.25">
@@ -1889,7 +1886,7 @@
         <v>164</v>
       </c>
       <c r="G25" t="s">
-        <v>165</v>
+        <v>143</v>
       </c>
       <c r="K25" t="s">
         <v>160</v>
@@ -1899,7 +1896,7 @@
         <v>2.7000000000000001E-3</v>
       </c>
       <c r="M25" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.25">
@@ -1907,7 +1904,7 @@
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.25">
       <c r="K27" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="L27" s="3">
         <v>0</v>
@@ -1919,7 +1916,7 @@
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.25">
       <c r="K29" s="3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L29" s="3">
         <v>0</v>
@@ -1936,19 +1933,19 @@
         <v>78</v>
       </c>
       <c r="K30" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L30">
         <v>0.83399999999999996</v>
       </c>
       <c r="M30" t="s">
+        <v>167</v>
+      </c>
+      <c r="N30" t="s">
         <v>168</v>
       </c>
-      <c r="N30" t="s">
+      <c r="O30" t="s">
         <v>169</v>
-      </c>
-      <c r="O30" t="s">
-        <v>170</v>
       </c>
       <c r="S30" s="16"/>
       <c r="T30" s="16"/>
@@ -1961,19 +1958,19 @@
         <v>79</v>
       </c>
       <c r="K31" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="L31">
         <v>0.50600000000000001</v>
       </c>
       <c r="M31" t="s">
+        <v>167</v>
+      </c>
+      <c r="N31" t="s">
         <v>168</v>
       </c>
-      <c r="N31" t="s">
+      <c r="O31" t="s">
         <v>169</v>
-      </c>
-      <c r="O31" t="s">
-        <v>170</v>
       </c>
       <c r="S31" s="16"/>
       <c r="T31" s="16"/>
@@ -1987,17 +1984,17 @@
         <v>142</v>
       </c>
       <c r="K33" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L33" s="25">
         <f>R13/(L8+L14)*100</f>
         <v>47.329217799538867</v>
       </c>
       <c r="M33" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="N33" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="S33" s="16"/>
     </row>
@@ -2006,19 +2003,19 @@
         <v>65</v>
       </c>
       <c r="K34" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L34">
         <v>22</v>
       </c>
       <c r="M34" t="s">
+        <v>170</v>
+      </c>
+      <c r="N34" t="s">
         <v>171</v>
       </c>
-      <c r="N34" t="s">
+      <c r="O34" t="s">
         <v>172</v>
-      </c>
-      <c r="O34" t="s">
-        <v>173</v>
       </c>
       <c r="S34" s="16"/>
       <c r="T34" s="38"/>
@@ -2028,19 +2025,19 @@
         <v>72</v>
       </c>
       <c r="K35" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L35" s="4">
         <v>90</v>
       </c>
       <c r="M35" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="N35" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="O35" t="s">
         <v>222</v>
-      </c>
-      <c r="O35" t="s">
-        <v>223</v>
       </c>
       <c r="T35" s="38"/>
     </row>
@@ -2049,19 +2046,19 @@
         <v>73</v>
       </c>
       <c r="K36" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="L36">
         <v>1.5</v>
       </c>
       <c r="M36" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="N36" t="s">
+        <v>173</v>
+      </c>
+      <c r="O36" t="s">
         <v>174</v>
-      </c>
-      <c r="O36" t="s">
-        <v>175</v>
       </c>
       <c r="T36" s="38"/>
     </row>
@@ -2419,7 +2416,7 @@
         <v>6</v>
       </c>
       <c r="N63" s="7" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.25">
@@ -2442,7 +2439,7 @@
     </row>
     <row r="65" spans="1:16" x14ac:dyDescent="0.25">
       <c r="C65" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
@@ -2457,7 +2454,7 @@
         <v>6</v>
       </c>
       <c r="N65" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.25">
@@ -3629,7 +3626,7 @@
         <v>29</v>
       </c>
       <c r="N138" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="O138" t="s">
         <v>44</v>
@@ -4263,7 +4260,7 @@
         <v>29</v>
       </c>
       <c r="N177" s="7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="O177" t="s">
         <v>53</v>
@@ -4424,12 +4421,12 @@
     </row>
     <row r="190" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A190" s="28" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="191" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K191" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L191">
         <v>100</v>
@@ -4438,7 +4435,7 @@
         <v>6</v>
       </c>
       <c r="O191" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="192" spans="1:15" x14ac:dyDescent="0.25">
@@ -4446,7 +4443,7 @@
         <v>156</v>
       </c>
       <c r="K192" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="L192">
         <v>47</v>
@@ -4455,7 +4452,7 @@
         <v>6</v>
       </c>
       <c r="O192" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="194" spans="1:15" x14ac:dyDescent="0.25">
@@ -4868,27 +4865,27 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>